<commit_message>
Changed test_output variable name in data.default.xlsx, and ran line 30 in 0_create_input_data.R
</commit_message>
<xml_diff>
--- a/data-raw/data.default.xlsx
+++ b/data-raw/data.default.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10210"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/trotsiuk/Documents/Research/software/r3PG/pkg/data-raw/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Forrester\Models\3-PG\r3PG\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37F69C00-1A31-0D4B-AE90-B60C879C3EB2}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7D4B1DB-C209-4CD2-9C1E-16211B50C510}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="24800" yWindow="560" windowWidth="25020" windowHeight="28120" activeTab="2" xr2:uid="{61EEFE5B-6AE1-A641-A9AB-273DC4213F59}"/>
+    <workbookView xWindow="59400" yWindow="-120" windowWidth="38640" windowHeight="21240" activeTab="2" xr2:uid="{61EEFE5B-6AE1-A641-A9AB-273DC4213F59}"/>
   </bookViews>
   <sheets>
     <sheet name="parameters" sheetId="8" r:id="rId1"/>
@@ -1730,9 +1730,6 @@
     <t>Stem mortality</t>
   </si>
   <si>
-    <t>var_8_5</t>
-  </si>
-  <si>
     <t>volume_extracted</t>
   </si>
   <si>
@@ -1998,13 +1995,16 @@
   </si>
   <si>
     <t>apar</t>
+  </si>
+  <si>
+    <t>test_output</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -2016,6 +2016,19 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -2039,8 +2052,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2060,9 +2075,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2100,7 +2115,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -2206,7 +2221,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2348,7 +2363,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2357,9 +2372,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E287297-02C0-BF44-BF0C-8FADE2A87F8F}">
   <dimension ref="A1:D83"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>117</v>
       </c>
@@ -2373,7 +2388,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -2387,7 +2402,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -2401,7 +2416,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -2415,7 +2430,7 @@
         <v>9.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -2429,7 +2444,7 @@
         <v>2.4</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -2443,7 +2458,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -2457,7 +2472,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -2471,7 +2486,7 @@
         <v>2.7E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -2485,7 +2500,7 @@
         <v>1E-3</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -2499,7 +2514,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -2513,7 +2528,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -2527,7 +2542,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -2541,7 +2556,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>13</v>
       </c>
@@ -2555,7 +2570,7 @@
         <v>8.5</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>14</v>
       </c>
@@ -2569,7 +2584,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>15</v>
       </c>
@@ -2583,7 +2598,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>16</v>
       </c>
@@ -2597,7 +2612,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>17</v>
       </c>
@@ -2611,7 +2626,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>18</v>
       </c>
@@ -2625,7 +2640,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>19</v>
       </c>
@@ -2639,7 +2654,7 @@
         <v>1.4</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -2653,7 +2668,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>21</v>
       </c>
@@ -2667,7 +2682,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>22</v>
       </c>
@@ -2681,7 +2696,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>23</v>
       </c>
@@ -2695,7 +2710,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>24</v>
       </c>
@@ -2709,7 +2724,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>25</v>
       </c>
@@ -2723,7 +2738,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>26</v>
       </c>
@@ -2737,7 +2752,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>27</v>
       </c>
@@ -2751,7 +2766,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>28</v>
       </c>
@@ -2765,7 +2780,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>29</v>
       </c>
@@ -2779,7 +2794,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>30</v>
       </c>
@@ -2793,7 +2808,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>31</v>
       </c>
@@ -2807,7 +2822,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>32</v>
       </c>
@@ -2821,7 +2836,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>33</v>
       </c>
@@ -2835,7 +2850,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>34</v>
       </c>
@@ -2849,7 +2864,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>35</v>
       </c>
@@ -2863,7 +2878,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>36</v>
       </c>
@@ -2877,7 +2892,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>37</v>
       </c>
@@ -2891,7 +2906,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>38</v>
       </c>
@@ -2905,7 +2920,7 @@
         <v>2.5</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>39</v>
       </c>
@@ -2919,7 +2934,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>40</v>
       </c>
@@ -2933,7 +2948,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>41</v>
       </c>
@@ -2947,7 +2962,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>42</v>
       </c>
@@ -2961,7 +2976,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>43</v>
       </c>
@@ -2975,7 +2990,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>44</v>
       </c>
@@ -2989,7 +3004,7 @@
         <v>0.06</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>45</v>
       </c>
@@ -3003,7 +3018,7 @@
         <v>0.47</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>46</v>
       </c>
@@ -3017,7 +3032,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>47</v>
       </c>
@@ -3031,7 +3046,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>48</v>
       </c>
@@ -3045,7 +3060,7 @@
         <v>3.33</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>49</v>
       </c>
@@ -3059,7 +3074,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>50</v>
       </c>
@@ -3073,7 +3088,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>51</v>
       </c>
@@ -3087,7 +3102,7 @@
         <v>0.66</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>52</v>
       </c>
@@ -3101,7 +3116,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>53</v>
       </c>
@@ -3115,7 +3130,7 @@
         <v>4.4000000000000004</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>54</v>
       </c>
@@ -3129,7 +3144,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>55</v>
       </c>
@@ -3143,7 +3158,7 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>56</v>
       </c>
@@ -3157,7 +3172,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>57</v>
       </c>
@@ -3171,7 +3186,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>58</v>
       </c>
@@ -3185,7 +3200,7 @@
         <v>0.45</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>59</v>
       </c>
@@ -3199,7 +3214,7 @@
         <v>0.45</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>60</v>
       </c>
@@ -3213,7 +3228,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>68</v>
       </c>
@@ -3227,7 +3242,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>61</v>
       </c>
@@ -3241,7 +3256,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>62</v>
       </c>
@@ -3255,7 +3270,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>63</v>
       </c>
@@ -3269,7 +3284,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>64</v>
       </c>
@@ -3283,7 +3298,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>65</v>
       </c>
@@ -3297,7 +3312,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>66</v>
       </c>
@@ -3311,7 +3326,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>67</v>
       </c>
@@ -3325,7 +3340,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>69</v>
       </c>
@@ -3339,7 +3354,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>70</v>
       </c>
@@ -3353,7 +3368,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>71</v>
       </c>
@@ -3367,7 +3382,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>72</v>
       </c>
@@ -3381,7 +3396,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>73</v>
       </c>
@@ -3395,7 +3410,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>74</v>
       </c>
@@ -3409,7 +3424,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>75</v>
       </c>
@@ -3423,7 +3438,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>76</v>
       </c>
@@ -3437,7 +3452,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>77</v>
       </c>
@@ -3451,7 +3466,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>78</v>
       </c>
@@ -3465,7 +3480,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>109</v>
       </c>
@@ -3479,7 +3494,7 @@
         <v>-90</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>110</v>
       </c>
@@ -3493,7 +3508,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>111</v>
       </c>
@@ -3507,7 +3522,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>112</v>
       </c>
@@ -3529,9 +3544,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FAF000D6-A72C-6444-9177-22D437B8361A}">
   <dimension ref="A1:D31"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>117</v>
       </c>
@@ -3545,7 +3560,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>79</v>
       </c>
@@ -3559,7 +3574,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>80</v>
       </c>
@@ -3573,7 +3588,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>81</v>
       </c>
@@ -3587,7 +3602,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>82</v>
       </c>
@@ -3601,7 +3616,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>83</v>
       </c>
@@ -3615,7 +3630,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>84</v>
       </c>
@@ -3629,7 +3644,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>85</v>
       </c>
@@ -3643,7 +3658,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>86</v>
       </c>
@@ -3657,7 +3672,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>87</v>
       </c>
@@ -3671,7 +3686,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>88</v>
       </c>
@@ -3685,7 +3700,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>89</v>
       </c>
@@ -3699,7 +3714,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>90</v>
       </c>
@@ -3713,7 +3728,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>91</v>
       </c>
@@ -3727,7 +3742,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>92</v>
       </c>
@@ -3741,7 +3756,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>93</v>
       </c>
@@ -3755,7 +3770,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>94</v>
       </c>
@@ -3769,7 +3784,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>95</v>
       </c>
@@ -3783,7 +3798,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>96</v>
       </c>
@@ -3797,7 +3812,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>97</v>
       </c>
@@ -3811,7 +3826,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>98</v>
       </c>
@@ -3825,7 +3840,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>99</v>
       </c>
@@ -3839,7 +3854,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>100</v>
       </c>
@@ -3853,7 +3868,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>101</v>
       </c>
@@ -3867,7 +3882,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>102</v>
       </c>
@@ -3881,7 +3896,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>103</v>
       </c>
@@ -3895,7 +3910,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>104</v>
       </c>
@@ -3909,7 +3924,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>105</v>
       </c>
@@ -3923,7 +3938,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>106</v>
       </c>
@@ -3937,7 +3952,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>107</v>
       </c>
@@ -3951,7 +3966,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>108</v>
       </c>
@@ -3973,9 +3988,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA3706E6-9BD2-3A49-A255-D2B55C8D9AB1}">
   <dimension ref="A1:G151"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="4" max="4" width="20" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="179" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>256</v>
       </c>
@@ -3998,7 +4017,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -4021,7 +4040,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -4044,7 +4063,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>1</v>
       </c>
@@ -4067,7 +4086,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>1</v>
       </c>
@@ -4090,7 +4109,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>1</v>
       </c>
@@ -4113,7 +4132,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>1</v>
       </c>
@@ -4136,7 +4155,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>1</v>
       </c>
@@ -4159,7 +4178,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>1</v>
       </c>
@@ -4182,7 +4201,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>1</v>
       </c>
@@ -4205,7 +4224,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>1</v>
       </c>
@@ -4225,7 +4244,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>1</v>
       </c>
@@ -4248,7 +4267,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>1</v>
       </c>
@@ -4262,7 +4281,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>1</v>
       </c>
@@ -4276,7 +4295,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>1</v>
       </c>
@@ -4290,7 +4309,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>1</v>
       </c>
@@ -4304,7 +4323,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2</v>
       </c>
@@ -4327,7 +4346,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2</v>
       </c>
@@ -4350,7 +4369,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>2</v>
       </c>
@@ -4373,7 +4392,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>2</v>
       </c>
@@ -4396,7 +4415,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>2</v>
       </c>
@@ -4419,7 +4438,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>2</v>
       </c>
@@ -4442,7 +4461,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>2</v>
       </c>
@@ -4465,7 +4484,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>2</v>
       </c>
@@ -4488,7 +4507,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>2</v>
       </c>
@@ -4511,7 +4530,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>2</v>
       </c>
@@ -4534,7 +4553,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>2</v>
       </c>
@@ -4557,7 +4576,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>2</v>
       </c>
@@ -4580,7 +4599,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>2</v>
       </c>
@@ -4603,7 +4622,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>2</v>
       </c>
@@ -4617,7 +4636,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>2</v>
       </c>
@@ -4631,7 +4650,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>3</v>
       </c>
@@ -4654,7 +4673,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>3</v>
       </c>
@@ -4677,7 +4696,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>3</v>
       </c>
@@ -4700,7 +4719,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>3</v>
       </c>
@@ -4723,7 +4742,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>3</v>
       </c>
@@ -4743,7 +4762,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>3</v>
       </c>
@@ -4766,7 +4785,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>3</v>
       </c>
@@ -4789,7 +4808,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>3</v>
       </c>
@@ -4812,7 +4831,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>3</v>
       </c>
@@ -4835,7 +4854,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>3</v>
       </c>
@@ -4858,7 +4877,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>3</v>
       </c>
@@ -4881,7 +4900,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>3</v>
       </c>
@@ -4895,7 +4914,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>3</v>
       </c>
@@ -4909,7 +4928,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>3</v>
       </c>
@@ -4923,7 +4942,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>3</v>
       </c>
@@ -4937,7 +4956,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>4</v>
       </c>
@@ -4960,7 +4979,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>4</v>
       </c>
@@ -4983,7 +5002,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>4</v>
       </c>
@@ -5006,7 +5025,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>4</v>
       </c>
@@ -5029,7 +5048,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>4</v>
       </c>
@@ -5052,7 +5071,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>4</v>
       </c>
@@ -5072,7 +5091,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>4</v>
       </c>
@@ -5095,7 +5114,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>4</v>
       </c>
@@ -5118,7 +5137,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>4</v>
       </c>
@@ -5141,7 +5160,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>4</v>
       </c>
@@ -5164,7 +5183,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>4</v>
       </c>
@@ -5187,7 +5206,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>4</v>
       </c>
@@ -5201,7 +5220,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>4</v>
       </c>
@@ -5215,7 +5234,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>4</v>
       </c>
@@ -5229,7 +5248,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>4</v>
       </c>
@@ -5243,7 +5262,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>5</v>
       </c>
@@ -5266,7 +5285,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>5</v>
       </c>
@@ -5289,7 +5308,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>5</v>
       </c>
@@ -5312,7 +5331,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>5</v>
       </c>
@@ -5335,7 +5354,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>5</v>
       </c>
@@ -5358,7 +5377,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>5</v>
       </c>
@@ -5381,7 +5400,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>5</v>
       </c>
@@ -5404,7 +5423,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>5</v>
       </c>
@@ -5427,7 +5446,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>5</v>
       </c>
@@ -5450,7 +5469,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>5</v>
       </c>
@@ -5473,7 +5492,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>5</v>
       </c>
@@ -5496,7 +5515,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>5</v>
       </c>
@@ -5516,7 +5535,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>5</v>
       </c>
@@ -5530,7 +5549,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>5</v>
       </c>
@@ -5544,7 +5563,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>5</v>
       </c>
@@ -5558,7 +5577,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>6</v>
       </c>
@@ -5581,7 +5600,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>6</v>
       </c>
@@ -5604,7 +5623,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>6</v>
       </c>
@@ -5612,7 +5631,7 @@
         <v>3</v>
       </c>
       <c r="C79" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="D79" t="s">
         <v>468</v>
@@ -5627,7 +5646,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>6</v>
       </c>
@@ -5650,7 +5669,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>6</v>
       </c>
@@ -5673,7 +5692,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>6</v>
       </c>
@@ -5696,7 +5715,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>6</v>
       </c>
@@ -5719,7 +5738,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>6</v>
       </c>
@@ -5742,7 +5761,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>6</v>
       </c>
@@ -5765,7 +5784,7 @@
         <v>495</v>
       </c>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>6</v>
       </c>
@@ -5788,7 +5807,7 @@
         <v>498</v>
       </c>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>6</v>
       </c>
@@ -5811,7 +5830,7 @@
         <v>501</v>
       </c>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>6</v>
       </c>
@@ -5834,7 +5853,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>6</v>
       </c>
@@ -5857,7 +5876,7 @@
         <v>506</v>
       </c>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>6</v>
       </c>
@@ -5871,7 +5890,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>6</v>
       </c>
@@ -5885,7 +5904,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>7</v>
       </c>
@@ -5908,7 +5927,7 @@
         <v>511</v>
       </c>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>7</v>
       </c>
@@ -5931,7 +5950,7 @@
         <v>514</v>
       </c>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>7</v>
       </c>
@@ -5954,7 +5973,7 @@
         <v>518</v>
       </c>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>7</v>
       </c>
@@ -5977,7 +5996,7 @@
         <v>522</v>
       </c>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>7</v>
       </c>
@@ -6000,7 +6019,7 @@
         <v>525</v>
       </c>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>7</v>
       </c>
@@ -6023,7 +6042,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>7</v>
       </c>
@@ -6046,7 +6065,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>7</v>
       </c>
@@ -6069,7 +6088,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>7</v>
       </c>
@@ -6092,7 +6111,7 @@
         <v>538</v>
       </c>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>7</v>
       </c>
@@ -6115,7 +6134,7 @@
         <v>541</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>7</v>
       </c>
@@ -6138,7 +6157,7 @@
         <v>544</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>7</v>
       </c>
@@ -6161,7 +6180,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>7</v>
       </c>
@@ -6184,7 +6203,7 @@
         <v>550</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>7</v>
       </c>
@@ -6198,7 +6217,7 @@
         <v>510</v>
       </c>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>7</v>
       </c>
@@ -6212,7 +6231,7 @@
         <v>510</v>
       </c>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>8</v>
       </c>
@@ -6235,7 +6254,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>8</v>
       </c>
@@ -6258,7 +6277,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>8</v>
       </c>
@@ -6281,7 +6300,7 @@
         <v>563</v>
       </c>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>8</v>
       </c>
@@ -6304,21 +6323,21 @@
         <v>566</v>
       </c>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A111">
+    <row r="111" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A111" s="2">
         <v>8</v>
       </c>
-      <c r="B111">
+      <c r="B111" s="2">
         <v>5</v>
       </c>
-      <c r="C111" t="s">
-        <v>567</v>
-      </c>
-      <c r="D111" t="s">
+      <c r="C111" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="D111" s="2" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A112">
         <v>8</v>
       </c>
@@ -6326,22 +6345,22 @@
         <v>6</v>
       </c>
       <c r="C112" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="D112" t="s">
         <v>554</v>
       </c>
       <c r="E112" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="F112" t="s">
         <v>333</v>
       </c>
       <c r="G112" t="s">
-        <v>570</v>
-      </c>
-    </row>
-    <row r="113" spans="1:7" x14ac:dyDescent="0.2">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="113" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>8</v>
       </c>
@@ -6349,13 +6368,13 @@
         <v>7</v>
       </c>
       <c r="C113" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="D113" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="114" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A114">
         <v>8</v>
       </c>
@@ -6363,22 +6382,22 @@
         <v>8</v>
       </c>
       <c r="C114" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="D114" t="s">
         <v>554</v>
       </c>
       <c r="E114" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="F114" t="s">
         <v>305</v>
       </c>
       <c r="G114" t="s">
-        <v>574</v>
-      </c>
-    </row>
-    <row r="115" spans="1:7" x14ac:dyDescent="0.2">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="115" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>8</v>
       </c>
@@ -6386,7 +6405,7 @@
         <v>9</v>
       </c>
       <c r="C115" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="D115" t="s">
         <v>554</v>
@@ -6398,10 +6417,10 @@
         <v>317</v>
       </c>
       <c r="G115" t="s">
-        <v>576</v>
-      </c>
-    </row>
-    <row r="116" spans="1:7" x14ac:dyDescent="0.2">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="116" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A116">
         <v>8</v>
       </c>
@@ -6409,7 +6428,7 @@
         <v>10</v>
       </c>
       <c r="C116" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="D116" t="s">
         <v>554</v>
@@ -6421,10 +6440,10 @@
         <v>309</v>
       </c>
       <c r="G116" t="s">
-        <v>578</v>
-      </c>
-    </row>
-    <row r="117" spans="1:7" x14ac:dyDescent="0.2">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="117" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A117">
         <v>8</v>
       </c>
@@ -6432,7 +6451,7 @@
         <v>11</v>
       </c>
       <c r="C117" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="D117" t="s">
         <v>554</v>
@@ -6444,10 +6463,10 @@
         <v>333</v>
       </c>
       <c r="G117" t="s">
-        <v>580</v>
-      </c>
-    </row>
-    <row r="118" spans="1:7" x14ac:dyDescent="0.2">
+        <v>579</v>
+      </c>
+    </row>
+    <row r="118" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A118">
         <v>8</v>
       </c>
@@ -6455,7 +6474,7 @@
         <v>12</v>
       </c>
       <c r="C118" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="D118" t="s">
         <v>554</v>
@@ -6467,10 +6486,10 @@
         <v>320</v>
       </c>
       <c r="G118" t="s">
-        <v>582</v>
-      </c>
-    </row>
-    <row r="119" spans="1:7" x14ac:dyDescent="0.2">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="119" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A119">
         <v>8</v>
       </c>
@@ -6478,7 +6497,7 @@
         <v>13</v>
       </c>
       <c r="C119" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="D119" t="s">
         <v>554</v>
@@ -6490,10 +6509,10 @@
         <v>391</v>
       </c>
       <c r="G119" t="s">
-        <v>584</v>
-      </c>
-    </row>
-    <row r="120" spans="1:7" x14ac:dyDescent="0.2">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="120" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A120">
         <v>8</v>
       </c>
@@ -6501,13 +6520,13 @@
         <v>14</v>
       </c>
       <c r="C120" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="D120" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="121" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A121">
         <v>8</v>
       </c>
@@ -6515,13 +6534,13 @@
         <v>15</v>
       </c>
       <c r="C121" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="D121" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="122" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A122">
         <v>9</v>
       </c>
@@ -6529,22 +6548,22 @@
         <v>1</v>
       </c>
       <c r="C122" t="s">
+        <v>586</v>
+      </c>
+      <c r="D122" t="s">
         <v>587</v>
       </c>
-      <c r="D122" t="s">
+      <c r="E122" t="s">
         <v>588</v>
       </c>
-      <c r="E122" t="s">
+      <c r="F122" t="s">
         <v>589</v>
       </c>
-      <c r="F122" t="s">
+      <c r="G122" t="s">
         <v>590</v>
       </c>
-      <c r="G122" t="s">
-        <v>591</v>
-      </c>
-    </row>
-    <row r="123" spans="1:7" x14ac:dyDescent="0.2">
+    </row>
+    <row r="123" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A123">
         <v>9</v>
       </c>
@@ -6552,22 +6571,22 @@
         <v>2</v>
       </c>
       <c r="C123" t="s">
+        <v>591</v>
+      </c>
+      <c r="D123" t="s">
+        <v>587</v>
+      </c>
+      <c r="E123" t="s">
         <v>592</v>
       </c>
-      <c r="D123" t="s">
-        <v>588</v>
-      </c>
-      <c r="E123" t="s">
+      <c r="F123" t="s">
+        <v>589</v>
+      </c>
+      <c r="G123" t="s">
         <v>593</v>
       </c>
-      <c r="F123" t="s">
-        <v>590</v>
-      </c>
-      <c r="G123" t="s">
-        <v>594</v>
-      </c>
-    </row>
-    <row r="124" spans="1:7" x14ac:dyDescent="0.2">
+    </row>
+    <row r="124" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A124">
         <v>9</v>
       </c>
@@ -6575,19 +6594,19 @@
         <v>3</v>
       </c>
       <c r="C124" t="s">
+        <v>594</v>
+      </c>
+      <c r="D124" t="s">
+        <v>587</v>
+      </c>
+      <c r="E124" t="s">
         <v>595</v>
       </c>
-      <c r="D124" t="s">
-        <v>588</v>
-      </c>
-      <c r="E124" t="s">
-        <v>596</v>
-      </c>
       <c r="G124" t="s">
-        <v>595</v>
-      </c>
-    </row>
-    <row r="125" spans="1:7" x14ac:dyDescent="0.2">
+        <v>594</v>
+      </c>
+    </row>
+    <row r="125" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A125">
         <v>9</v>
       </c>
@@ -6595,19 +6614,19 @@
         <v>4</v>
       </c>
       <c r="C125" t="s">
+        <v>596</v>
+      </c>
+      <c r="D125" t="s">
+        <v>587</v>
+      </c>
+      <c r="E125" t="s">
         <v>597</v>
       </c>
-      <c r="D125" t="s">
-        <v>588</v>
-      </c>
-      <c r="E125" t="s">
-        <v>598</v>
-      </c>
       <c r="G125" t="s">
-        <v>597</v>
-      </c>
-    </row>
-    <row r="126" spans="1:7" x14ac:dyDescent="0.2">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="126" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A126">
         <v>9</v>
       </c>
@@ -6615,22 +6634,22 @@
         <v>5</v>
       </c>
       <c r="C126" t="s">
+        <v>598</v>
+      </c>
+      <c r="D126" t="s">
+        <v>587</v>
+      </c>
+      <c r="E126" t="s">
         <v>599</v>
-      </c>
-      <c r="D126" t="s">
-        <v>588</v>
-      </c>
-      <c r="E126" t="s">
-        <v>600</v>
       </c>
       <c r="F126" t="s">
         <v>288</v>
       </c>
       <c r="G126" t="s">
-        <v>601</v>
-      </c>
-    </row>
-    <row r="127" spans="1:7" x14ac:dyDescent="0.2">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="127" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A127">
         <v>9</v>
       </c>
@@ -6638,13 +6657,13 @@
         <v>6</v>
       </c>
       <c r="C127" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="D127" t="s">
-        <v>588</v>
-      </c>
-    </row>
-    <row r="128" spans="1:7" x14ac:dyDescent="0.2">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="128" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A128">
         <v>9</v>
       </c>
@@ -6652,13 +6671,13 @@
         <v>7</v>
       </c>
       <c r="C128" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D128" t="s">
-        <v>588</v>
-      </c>
-    </row>
-    <row r="129" spans="1:7" x14ac:dyDescent="0.2">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="129" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A129">
         <v>9</v>
       </c>
@@ -6666,13 +6685,13 @@
         <v>8</v>
       </c>
       <c r="C129" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="D129" t="s">
-        <v>588</v>
-      </c>
-    </row>
-    <row r="130" spans="1:7" x14ac:dyDescent="0.2">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="130" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A130">
         <v>9</v>
       </c>
@@ -6680,13 +6699,13 @@
         <v>9</v>
       </c>
       <c r="C130" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="D130" t="s">
-        <v>588</v>
-      </c>
-    </row>
-    <row r="131" spans="1:7" x14ac:dyDescent="0.2">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="131" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A131">
         <v>9</v>
       </c>
@@ -6694,13 +6713,13 @@
         <v>10</v>
       </c>
       <c r="C131" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="D131" t="s">
-        <v>588</v>
-      </c>
-    </row>
-    <row r="132" spans="1:7" x14ac:dyDescent="0.2">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="132" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A132">
         <v>9</v>
       </c>
@@ -6708,13 +6727,13 @@
         <v>11</v>
       </c>
       <c r="C132" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="D132" t="s">
-        <v>588</v>
-      </c>
-    </row>
-    <row r="133" spans="1:7" x14ac:dyDescent="0.2">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="133" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A133">
         <v>9</v>
       </c>
@@ -6722,13 +6741,13 @@
         <v>12</v>
       </c>
       <c r="C133" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="D133" t="s">
-        <v>588</v>
-      </c>
-    </row>
-    <row r="134" spans="1:7" x14ac:dyDescent="0.2">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="134" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A134">
         <v>9</v>
       </c>
@@ -6736,13 +6755,13 @@
         <v>13</v>
       </c>
       <c r="C134" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="D134" t="s">
-        <v>588</v>
-      </c>
-    </row>
-    <row r="135" spans="1:7" x14ac:dyDescent="0.2">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="135" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A135">
         <v>9</v>
       </c>
@@ -6750,13 +6769,13 @@
         <v>14</v>
       </c>
       <c r="C135" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="D135" t="s">
-        <v>588</v>
-      </c>
-    </row>
-    <row r="136" spans="1:7" x14ac:dyDescent="0.2">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="136" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A136">
         <v>9</v>
       </c>
@@ -6764,13 +6783,13 @@
         <v>15</v>
       </c>
       <c r="C136" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="D136" t="s">
-        <v>588</v>
-      </c>
-    </row>
-    <row r="137" spans="1:7" x14ac:dyDescent="0.2">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="137" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A137">
         <v>10</v>
       </c>
@@ -6778,22 +6797,22 @@
         <v>1</v>
       </c>
       <c r="C137" t="s">
+        <v>611</v>
+      </c>
+      <c r="D137" t="s">
         <v>612</v>
       </c>
-      <c r="D137" t="s">
+      <c r="E137" t="s">
         <v>613</v>
       </c>
-      <c r="E137" t="s">
+      <c r="F137" t="s">
+        <v>128</v>
+      </c>
+      <c r="G137" t="s">
         <v>614</v>
       </c>
-      <c r="F137" t="s">
-        <v>128</v>
-      </c>
-      <c r="G137" t="s">
-        <v>615</v>
-      </c>
-    </row>
-    <row r="138" spans="1:7" x14ac:dyDescent="0.2">
+    </row>
+    <row r="138" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A138">
         <v>10</v>
       </c>
@@ -6801,22 +6820,22 @@
         <v>2</v>
       </c>
       <c r="C138" t="s">
+        <v>615</v>
+      </c>
+      <c r="D138" t="s">
+        <v>612</v>
+      </c>
+      <c r="E138" t="s">
         <v>616</v>
       </c>
-      <c r="D138" t="s">
-        <v>613</v>
-      </c>
-      <c r="E138" t="s">
+      <c r="F138" t="s">
+        <v>128</v>
+      </c>
+      <c r="G138" t="s">
         <v>617</v>
       </c>
-      <c r="F138" t="s">
-        <v>128</v>
-      </c>
-      <c r="G138" t="s">
-        <v>618</v>
-      </c>
-    </row>
-    <row r="139" spans="1:7" x14ac:dyDescent="0.2">
+    </row>
+    <row r="139" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A139">
         <v>10</v>
       </c>
@@ -6824,22 +6843,22 @@
         <v>3</v>
       </c>
       <c r="C139" t="s">
+        <v>618</v>
+      </c>
+      <c r="D139" t="s">
+        <v>612</v>
+      </c>
+      <c r="E139" t="s">
         <v>619</v>
       </c>
-      <c r="D139" t="s">
-        <v>613</v>
-      </c>
-      <c r="E139" t="s">
+      <c r="F139" t="s">
+        <v>128</v>
+      </c>
+      <c r="G139" t="s">
         <v>620</v>
       </c>
-      <c r="F139" t="s">
-        <v>128</v>
-      </c>
-      <c r="G139" t="s">
-        <v>621</v>
-      </c>
-    </row>
-    <row r="140" spans="1:7" x14ac:dyDescent="0.2">
+    </row>
+    <row r="140" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A140">
         <v>10</v>
       </c>
@@ -6847,22 +6866,22 @@
         <v>4</v>
       </c>
       <c r="C140" t="s">
+        <v>621</v>
+      </c>
+      <c r="D140" t="s">
+        <v>612</v>
+      </c>
+      <c r="E140" t="s">
         <v>622</v>
       </c>
-      <c r="D140" t="s">
-        <v>613</v>
-      </c>
-      <c r="E140" t="s">
+      <c r="F140" t="s">
+        <v>128</v>
+      </c>
+      <c r="G140" t="s">
         <v>623</v>
       </c>
-      <c r="F140" t="s">
-        <v>128</v>
-      </c>
-      <c r="G140" t="s">
-        <v>624</v>
-      </c>
-    </row>
-    <row r="141" spans="1:7" x14ac:dyDescent="0.2">
+    </row>
+    <row r="141" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A141">
         <v>10</v>
       </c>
@@ -6870,22 +6889,22 @@
         <v>5</v>
       </c>
       <c r="C141" t="s">
+        <v>624</v>
+      </c>
+      <c r="D141" t="s">
+        <v>612</v>
+      </c>
+      <c r="E141" t="s">
         <v>625</v>
       </c>
-      <c r="D141" t="s">
-        <v>613</v>
-      </c>
-      <c r="E141" t="s">
+      <c r="F141" t="s">
+        <v>128</v>
+      </c>
+      <c r="G141" t="s">
         <v>626</v>
       </c>
-      <c r="F141" t="s">
-        <v>128</v>
-      </c>
-      <c r="G141" t="s">
-        <v>627</v>
-      </c>
-    </row>
-    <row r="142" spans="1:7" x14ac:dyDescent="0.2">
+    </row>
+    <row r="142" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A142">
         <v>10</v>
       </c>
@@ -6893,22 +6912,22 @@
         <v>6</v>
       </c>
       <c r="C142" t="s">
+        <v>627</v>
+      </c>
+      <c r="D142" t="s">
+        <v>612</v>
+      </c>
+      <c r="E142" t="s">
         <v>628</v>
       </c>
-      <c r="D142" t="s">
-        <v>613</v>
-      </c>
-      <c r="E142" t="s">
+      <c r="F142" t="s">
+        <v>128</v>
+      </c>
+      <c r="G142" t="s">
         <v>629</v>
       </c>
-      <c r="F142" t="s">
-        <v>128</v>
-      </c>
-      <c r="G142" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="143" spans="1:7" x14ac:dyDescent="0.2">
+    </row>
+    <row r="143" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A143">
         <v>10</v>
       </c>
@@ -6916,22 +6935,22 @@
         <v>7</v>
       </c>
       <c r="C143" t="s">
+        <v>630</v>
+      </c>
+      <c r="D143" t="s">
+        <v>612</v>
+      </c>
+      <c r="E143" t="s">
         <v>631</v>
-      </c>
-      <c r="D143" t="s">
-        <v>613</v>
-      </c>
-      <c r="E143" t="s">
-        <v>632</v>
       </c>
       <c r="F143" t="s">
         <v>367</v>
       </c>
       <c r="G143" t="s">
-        <v>633</v>
-      </c>
-    </row>
-    <row r="144" spans="1:7" x14ac:dyDescent="0.2">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="144" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A144">
         <v>10</v>
       </c>
@@ -6939,22 +6958,22 @@
         <v>8</v>
       </c>
       <c r="C144" t="s">
+        <v>633</v>
+      </c>
+      <c r="D144" t="s">
+        <v>612</v>
+      </c>
+      <c r="E144" t="s">
         <v>634</v>
-      </c>
-      <c r="D144" t="s">
-        <v>613</v>
-      </c>
-      <c r="E144" t="s">
-        <v>635</v>
       </c>
       <c r="F144" t="s">
         <v>367</v>
       </c>
       <c r="G144" t="s">
-        <v>636</v>
-      </c>
-    </row>
-    <row r="145" spans="1:7" x14ac:dyDescent="0.2">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="145" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A145">
         <v>10</v>
       </c>
@@ -6962,22 +6981,22 @@
         <v>9</v>
       </c>
       <c r="C145" t="s">
+        <v>636</v>
+      </c>
+      <c r="D145" t="s">
+        <v>612</v>
+      </c>
+      <c r="E145" t="s">
         <v>637</v>
-      </c>
-      <c r="D145" t="s">
-        <v>613</v>
-      </c>
-      <c r="E145" t="s">
-        <v>638</v>
       </c>
       <c r="F145" t="s">
         <v>367</v>
       </c>
       <c r="G145" t="s">
-        <v>639</v>
-      </c>
-    </row>
-    <row r="146" spans="1:7" x14ac:dyDescent="0.2">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="146" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A146">
         <v>10</v>
       </c>
@@ -6985,22 +7004,22 @@
         <v>10</v>
       </c>
       <c r="C146" t="s">
+        <v>639</v>
+      </c>
+      <c r="D146" t="s">
+        <v>612</v>
+      </c>
+      <c r="E146" t="s">
         <v>640</v>
-      </c>
-      <c r="D146" t="s">
-        <v>613</v>
-      </c>
-      <c r="E146" t="s">
-        <v>641</v>
       </c>
       <c r="F146" t="s">
         <v>367</v>
       </c>
       <c r="G146" t="s">
-        <v>642</v>
-      </c>
-    </row>
-    <row r="147" spans="1:7" x14ac:dyDescent="0.2">
+        <v>641</v>
+      </c>
+    </row>
+    <row r="147" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A147">
         <v>10</v>
       </c>
@@ -7008,22 +7027,22 @@
         <v>11</v>
       </c>
       <c r="C147" t="s">
+        <v>642</v>
+      </c>
+      <c r="D147" t="s">
+        <v>612</v>
+      </c>
+      <c r="E147" t="s">
         <v>643</v>
-      </c>
-      <c r="D147" t="s">
-        <v>613</v>
-      </c>
-      <c r="E147" t="s">
-        <v>644</v>
       </c>
       <c r="F147" t="s">
         <v>367</v>
       </c>
       <c r="G147" t="s">
-        <v>645</v>
-      </c>
-    </row>
-    <row r="148" spans="1:7" x14ac:dyDescent="0.2">
+        <v>644</v>
+      </c>
+    </row>
+    <row r="148" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A148">
         <v>10</v>
       </c>
@@ -7031,22 +7050,22 @@
         <v>12</v>
       </c>
       <c r="C148" t="s">
+        <v>645</v>
+      </c>
+      <c r="D148" t="s">
+        <v>612</v>
+      </c>
+      <c r="E148" t="s">
         <v>646</v>
-      </c>
-      <c r="D148" t="s">
-        <v>613</v>
-      </c>
-      <c r="E148" t="s">
-        <v>647</v>
       </c>
       <c r="F148" t="s">
         <v>367</v>
       </c>
       <c r="G148" t="s">
-        <v>648</v>
-      </c>
-    </row>
-    <row r="149" spans="1:7" x14ac:dyDescent="0.2">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="149" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A149">
         <v>10</v>
       </c>
@@ -7054,22 +7073,22 @@
         <v>13</v>
       </c>
       <c r="C149" t="s">
+        <v>648</v>
+      </c>
+      <c r="D149" t="s">
+        <v>612</v>
+      </c>
+      <c r="E149" t="s">
         <v>649</v>
-      </c>
-      <c r="D149" t="s">
-        <v>613</v>
-      </c>
-      <c r="E149" t="s">
-        <v>650</v>
       </c>
       <c r="F149" t="s">
         <v>367</v>
       </c>
       <c r="G149" t="s">
-        <v>651</v>
-      </c>
-    </row>
-    <row r="150" spans="1:7" x14ac:dyDescent="0.2">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="150" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A150">
         <v>10</v>
       </c>
@@ -7077,22 +7096,22 @@
         <v>14</v>
       </c>
       <c r="C150" t="s">
+        <v>651</v>
+      </c>
+      <c r="D150" t="s">
+        <v>612</v>
+      </c>
+      <c r="E150" t="s">
         <v>652</v>
-      </c>
-      <c r="D150" t="s">
-        <v>613</v>
-      </c>
-      <c r="E150" t="s">
-        <v>653</v>
       </c>
       <c r="F150" t="s">
         <v>367</v>
       </c>
       <c r="G150" t="s">
-        <v>654</v>
-      </c>
-    </row>
-    <row r="151" spans="1:7" x14ac:dyDescent="0.2">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="151" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A151">
         <v>10</v>
       </c>
@@ -7100,10 +7119,10 @@
         <v>15</v>
       </c>
       <c r="C151" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="D151" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
issue #103 cleaning the mortality model to have it more systematic and reduce redundancy
</commit_message>
<xml_diff>
--- a/data-raw/data.default.xlsx
+++ b/data-raw/data.default.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11110"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Forrester\Models\3-PG\r3PG\data-raw\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/trotsiuk/Documents/Research/software/r3PG/data-raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D10201B4-0DF6-47FB-8335-B8B0A023989D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91EF81DE-07A2-5E4F-8014-C289F453FBE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="59400" yWindow="-120" windowWidth="38640" windowHeight="21240" activeTab="2" xr2:uid="{61EEFE5B-6AE1-A641-A9AB-273DC4213F59}"/>
+    <workbookView xWindow="1080" yWindow="500" windowWidth="50120" windowHeight="28300" activeTab="2" xr2:uid="{61EEFE5B-6AE1-A641-A9AB-273DC4213F59}"/>
   </bookViews>
   <sheets>
     <sheet name="parameters" sheetId="8" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="999" uniqueCount="669">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1000" uniqueCount="670">
   <si>
     <t>pFS2</t>
   </si>
@@ -2034,6 +2034,9 @@
   </si>
   <si>
     <t>stems_n_total</t>
+  </si>
+  <si>
+    <t>Stems number of the active cohorts</t>
   </si>
 </sst>
 </file>
@@ -2413,9 +2416,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E287297-02C0-BF44-BF0C-8FADE2A87F8F}">
   <dimension ref="A1:D89"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>117</v>
       </c>
@@ -2429,7 +2432,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -2443,7 +2446,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -2457,7 +2460,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -2471,7 +2474,7 @@
         <v>9.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -2485,7 +2488,7 @@
         <v>2.4</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -2499,7 +2502,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -2513,7 +2516,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -2527,7 +2530,7 @@
         <v>2.7E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -2541,7 +2544,7 @@
         <v>1E-3</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -2555,7 +2558,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -2569,7 +2572,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -2583,7 +2586,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -2597,7 +2600,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>13</v>
       </c>
@@ -2611,7 +2614,7 @@
         <v>8.5</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>14</v>
       </c>
@@ -2625,7 +2628,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>15</v>
       </c>
@@ -2639,7 +2642,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>16</v>
       </c>
@@ -2653,7 +2656,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>17</v>
       </c>
@@ -2667,7 +2670,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>18</v>
       </c>
@@ -2681,7 +2684,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>19</v>
       </c>
@@ -2695,7 +2698,7 @@
         <v>1.4</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -2709,7 +2712,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>21</v>
       </c>
@@ -2723,7 +2726,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>22</v>
       </c>
@@ -2737,7 +2740,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>23</v>
       </c>
@@ -2751,7 +2754,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>24</v>
       </c>
@@ -2765,7 +2768,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>25</v>
       </c>
@@ -2779,7 +2782,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>26</v>
       </c>
@@ -2793,7 +2796,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>27</v>
       </c>
@@ -2807,7 +2810,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>28</v>
       </c>
@@ -2821,7 +2824,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>29</v>
       </c>
@@ -2835,7 +2838,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>30</v>
       </c>
@@ -2849,7 +2852,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>31</v>
       </c>
@@ -2863,7 +2866,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>32</v>
       </c>
@@ -2877,7 +2880,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
         <v>648</v>
       </c>
@@ -2889,7 +2892,7 @@
         <v>-20.399999999999999</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
         <v>649</v>
       </c>
@@ -2901,7 +2904,7 @@
         <v>1.86</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
         <v>650</v>
       </c>
@@ -2913,7 +2916,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
         <v>651</v>
       </c>
@@ -2925,7 +2928,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
         <v>652</v>
       </c>
@@ -2937,7 +2940,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
         <v>653</v>
       </c>
@@ -2949,7 +2952,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>33</v>
       </c>
@@ -2963,7 +2966,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>34</v>
       </c>
@@ -2977,7 +2980,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>35</v>
       </c>
@@ -2991,7 +2994,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>36</v>
       </c>
@@ -3005,7 +3008,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>37</v>
       </c>
@@ -3019,7 +3022,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>38</v>
       </c>
@@ -3033,7 +3036,7 @@
         <v>2.5</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>39</v>
       </c>
@@ -3047,7 +3050,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>40</v>
       </c>
@@ -3061,7 +3064,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>41</v>
       </c>
@@ -3075,7 +3078,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>42</v>
       </c>
@@ -3089,7 +3092,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>43</v>
       </c>
@@ -3103,7 +3106,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>44</v>
       </c>
@@ -3117,7 +3120,7 @@
         <v>0.06</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>45</v>
       </c>
@@ -3131,7 +3134,7 @@
         <v>0.47</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>46</v>
       </c>
@@ -3145,7 +3148,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>47</v>
       </c>
@@ -3159,7 +3162,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>48</v>
       </c>
@@ -3173,7 +3176,7 @@
         <v>3.33</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>49</v>
       </c>
@@ -3187,7 +3190,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>50</v>
       </c>
@@ -3201,7 +3204,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>51</v>
       </c>
@@ -3215,7 +3218,7 @@
         <v>0.66</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>52</v>
       </c>
@@ -3229,7 +3232,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>53</v>
       </c>
@@ -3243,7 +3246,7 @@
         <v>4.4000000000000004</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>54</v>
       </c>
@@ -3257,7 +3260,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>55</v>
       </c>
@@ -3271,7 +3274,7 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>56</v>
       </c>
@@ -3285,7 +3288,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>57</v>
       </c>
@@ -3299,7 +3302,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>58</v>
       </c>
@@ -3313,7 +3316,7 @@
         <v>0.45</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>59</v>
       </c>
@@ -3327,7 +3330,7 @@
         <v>0.45</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>60</v>
       </c>
@@ -3341,7 +3344,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>68</v>
       </c>
@@ -3355,7 +3358,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>61</v>
       </c>
@@ -3369,7 +3372,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>62</v>
       </c>
@@ -3383,7 +3386,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>63</v>
       </c>
@@ -3397,7 +3400,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>64</v>
       </c>
@@ -3411,7 +3414,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>65</v>
       </c>
@@ -3425,7 +3428,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>66</v>
       </c>
@@ -3439,7 +3442,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>67</v>
       </c>
@@ -3453,7 +3456,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>69</v>
       </c>
@@ -3467,7 +3470,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>70</v>
       </c>
@@ -3481,7 +3484,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>71</v>
       </c>
@@ -3495,7 +3498,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>72</v>
       </c>
@@ -3509,7 +3512,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>73</v>
       </c>
@@ -3523,7 +3526,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>74</v>
       </c>
@@ -3537,7 +3540,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>75</v>
       </c>
@@ -3551,7 +3554,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>76</v>
       </c>
@@ -3565,7 +3568,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>77</v>
       </c>
@@ -3579,7 +3582,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>78</v>
       </c>
@@ -3593,7 +3596,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>109</v>
       </c>
@@ -3607,7 +3610,7 @@
         <v>-90</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>110</v>
       </c>
@@ -3621,7 +3624,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>111</v>
       </c>
@@ -3635,7 +3638,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>112</v>
       </c>
@@ -3657,9 +3660,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FAF000D6-A72C-6444-9177-22D437B8361A}">
   <dimension ref="A1:D31"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>117</v>
       </c>
@@ -3673,7 +3676,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>79</v>
       </c>
@@ -3687,7 +3690,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>80</v>
       </c>
@@ -3701,7 +3704,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>81</v>
       </c>
@@ -3715,7 +3718,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>82</v>
       </c>
@@ -3729,7 +3732,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>83</v>
       </c>
@@ -3743,7 +3746,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>84</v>
       </c>
@@ -3757,7 +3760,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>85</v>
       </c>
@@ -3771,7 +3774,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>86</v>
       </c>
@@ -3785,7 +3788,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>87</v>
       </c>
@@ -3799,7 +3802,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>88</v>
       </c>
@@ -3813,7 +3816,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>89</v>
       </c>
@@ -3827,7 +3830,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>90</v>
       </c>
@@ -3841,7 +3844,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>91</v>
       </c>
@@ -3855,7 +3858,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>92</v>
       </c>
@@ -3869,7 +3872,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>93</v>
       </c>
@@ -3883,7 +3886,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>94</v>
       </c>
@@ -3897,7 +3900,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>95</v>
       </c>
@@ -3911,7 +3914,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>96</v>
       </c>
@@ -3925,7 +3928,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>97</v>
       </c>
@@ -3939,7 +3942,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>98</v>
       </c>
@@ -3953,7 +3956,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>99</v>
       </c>
@@ -3967,7 +3970,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>100</v>
       </c>
@@ -3981,7 +3984,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>101</v>
       </c>
@@ -3995,7 +3998,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>102</v>
       </c>
@@ -4009,7 +4012,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>103</v>
       </c>
@@ -4023,7 +4026,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>104</v>
       </c>
@@ -4037,7 +4040,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>105</v>
       </c>
@@ -4051,7 +4054,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>106</v>
       </c>
@@ -4065,7 +4068,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>107</v>
       </c>
@@ -4079,7 +4082,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>108</v>
       </c>
@@ -4101,13 +4104,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA3706E6-9BD2-3A49-A255-D2B55C8D9AB1}">
   <dimension ref="A1:G151"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="3" max="3" width="51.1640625" customWidth="1"/>
     <col min="4" max="4" width="20" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="179" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>256</v>
       </c>
@@ -4130,7 +4134,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -4153,7 +4157,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>1</v>
       </c>
@@ -4176,7 +4180,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>1</v>
       </c>
@@ -4199,7 +4203,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>1</v>
       </c>
@@ -4222,7 +4226,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>1</v>
       </c>
@@ -4245,7 +4249,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>1</v>
       </c>
@@ -4268,7 +4272,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>1</v>
       </c>
@@ -4291,7 +4295,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>1</v>
       </c>
@@ -4314,7 +4318,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>1</v>
       </c>
@@ -4337,7 +4341,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>1</v>
       </c>
@@ -4357,7 +4361,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>1</v>
       </c>
@@ -4380,7 +4384,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>1</v>
       </c>
@@ -4394,7 +4398,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>1</v>
       </c>
@@ -4408,7 +4412,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>1</v>
       </c>
@@ -4422,7 +4426,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>1</v>
       </c>
@@ -4436,7 +4440,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>2</v>
       </c>
@@ -4459,7 +4463,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>2</v>
       </c>
@@ -4482,7 +4486,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>2</v>
       </c>
@@ -4505,7 +4509,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>2</v>
       </c>
@@ -4528,7 +4532,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>2</v>
       </c>
@@ -4551,7 +4555,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>2</v>
       </c>
@@ -4574,7 +4578,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>2</v>
       </c>
@@ -4597,7 +4601,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>2</v>
       </c>
@@ -4620,7 +4624,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>2</v>
       </c>
@@ -4643,7 +4647,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>2</v>
       </c>
@@ -4666,7 +4670,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>2</v>
       </c>
@@ -4689,7 +4693,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>2</v>
       </c>
@@ -4712,7 +4716,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>2</v>
       </c>
@@ -4735,7 +4739,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>2</v>
       </c>
@@ -4749,7 +4753,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>2</v>
       </c>
@@ -4763,7 +4767,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>3</v>
       </c>
@@ -4786,7 +4790,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>3</v>
       </c>
@@ -4809,7 +4813,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>3</v>
       </c>
@@ -4832,7 +4836,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>3</v>
       </c>
@@ -4855,7 +4859,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>3</v>
       </c>
@@ -4875,7 +4879,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>3</v>
       </c>
@@ -4898,7 +4902,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>3</v>
       </c>
@@ -4921,7 +4925,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>3</v>
       </c>
@@ -4944,7 +4948,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>3</v>
       </c>
@@ -4967,7 +4971,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>3</v>
       </c>
@@ -4990,7 +4994,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>3</v>
       </c>
@@ -5013,7 +5017,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>3</v>
       </c>
@@ -5027,7 +5031,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>3</v>
       </c>
@@ -5041,7 +5045,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>3</v>
       </c>
@@ -5055,7 +5059,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>3</v>
       </c>
@@ -5069,7 +5073,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>4</v>
       </c>
@@ -5092,7 +5096,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>4</v>
       </c>
@@ -5115,7 +5119,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>4</v>
       </c>
@@ -5138,7 +5142,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>4</v>
       </c>
@@ -5161,7 +5165,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>4</v>
       </c>
@@ -5184,7 +5188,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>4</v>
       </c>
@@ -5204,7 +5208,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>4</v>
       </c>
@@ -5227,7 +5231,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>4</v>
       </c>
@@ -5250,7 +5254,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>4</v>
       </c>
@@ -5273,7 +5277,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A56">
         <v>4</v>
       </c>
@@ -5296,7 +5300,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A57">
         <v>4</v>
       </c>
@@ -5319,7 +5323,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A58">
         <v>4</v>
       </c>
@@ -5333,7 +5337,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A59">
         <v>4</v>
       </c>
@@ -5347,7 +5351,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A60">
         <v>4</v>
       </c>
@@ -5361,7 +5365,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A61">
         <v>4</v>
       </c>
@@ -5375,7 +5379,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A62">
         <v>5</v>
       </c>
@@ -5398,7 +5402,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A63">
         <v>5</v>
       </c>
@@ -5421,7 +5425,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A64">
         <v>5</v>
       </c>
@@ -5444,7 +5448,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A65">
         <v>5</v>
       </c>
@@ -5467,7 +5471,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A66">
         <v>5</v>
       </c>
@@ -5490,7 +5494,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A67">
         <v>5</v>
       </c>
@@ -5513,7 +5517,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A68">
         <v>5</v>
       </c>
@@ -5536,7 +5540,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A69">
         <v>5</v>
       </c>
@@ -5559,7 +5563,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A70">
         <v>5</v>
       </c>
@@ -5582,7 +5586,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A71">
         <v>5</v>
       </c>
@@ -5605,7 +5609,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A72">
         <v>5</v>
       </c>
@@ -5628,7 +5632,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A73">
         <v>5</v>
       </c>
@@ -5648,7 +5652,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A74">
         <v>5</v>
       </c>
@@ -5662,7 +5666,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A75">
         <v>5</v>
       </c>
@@ -5676,7 +5680,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A76">
         <v>5</v>
       </c>
@@ -5690,7 +5694,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A77">
         <v>6</v>
       </c>
@@ -5713,7 +5717,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A78">
         <v>6</v>
       </c>
@@ -5736,7 +5740,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A79">
         <v>6</v>
       </c>
@@ -5759,7 +5763,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A80">
         <v>6</v>
       </c>
@@ -5782,7 +5786,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A81">
         <v>6</v>
       </c>
@@ -5805,7 +5809,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A82">
         <v>6</v>
       </c>
@@ -5828,7 +5832,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A83">
         <v>6</v>
       </c>
@@ -5851,7 +5855,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A84">
         <v>6</v>
       </c>
@@ -5874,7 +5878,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A85">
         <v>6</v>
       </c>
@@ -5897,7 +5901,7 @@
         <v>495</v>
       </c>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A86">
         <v>6</v>
       </c>
@@ -5920,7 +5924,7 @@
         <v>498</v>
       </c>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A87">
         <v>6</v>
       </c>
@@ -5943,7 +5947,7 @@
         <v>501</v>
       </c>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A88">
         <v>6</v>
       </c>
@@ -5966,7 +5970,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A89">
         <v>6</v>
       </c>
@@ -5989,7 +5993,7 @@
         <v>506</v>
       </c>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A90">
         <v>6</v>
       </c>
@@ -6003,7 +6007,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A91">
         <v>6</v>
       </c>
@@ -6017,7 +6021,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A92">
         <v>7</v>
       </c>
@@ -6040,7 +6044,7 @@
         <v>511</v>
       </c>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A93">
         <v>7</v>
       </c>
@@ -6063,7 +6067,7 @@
         <v>514</v>
       </c>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A94">
         <v>7</v>
       </c>
@@ -6086,7 +6090,7 @@
         <v>518</v>
       </c>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A95">
         <v>7</v>
       </c>
@@ -6109,7 +6113,7 @@
         <v>522</v>
       </c>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A96">
         <v>7</v>
       </c>
@@ -6132,7 +6136,7 @@
         <v>525</v>
       </c>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A97">
         <v>7</v>
       </c>
@@ -6155,7 +6159,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A98">
         <v>7</v>
       </c>
@@ -6178,7 +6182,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A99">
         <v>7</v>
       </c>
@@ -6201,7 +6205,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A100">
         <v>7</v>
       </c>
@@ -6224,7 +6228,7 @@
         <v>538</v>
       </c>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A101">
         <v>7</v>
       </c>
@@ -6247,7 +6251,7 @@
         <v>541</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A102">
         <v>7</v>
       </c>
@@ -6270,7 +6274,7 @@
         <v>544</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A103">
         <v>7</v>
       </c>
@@ -6293,7 +6297,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A104">
         <v>7</v>
       </c>
@@ -6316,7 +6320,7 @@
         <v>550</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A105">
         <v>7</v>
       </c>
@@ -6330,7 +6334,7 @@
         <v>510</v>
       </c>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A106">
         <v>7</v>
       </c>
@@ -6344,7 +6348,7 @@
         <v>510</v>
       </c>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A107">
         <v>8</v>
       </c>
@@ -6367,7 +6371,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A108">
         <v>8</v>
       </c>
@@ -6390,7 +6394,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A109">
         <v>8</v>
       </c>
@@ -6413,7 +6417,7 @@
         <v>563</v>
       </c>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A110">
         <v>8</v>
       </c>
@@ -6436,7 +6440,7 @@
         <v>566</v>
       </c>
     </row>
-    <row r="111" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A111" s="2">
         <v>8</v>
       </c>
@@ -6450,7 +6454,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A112">
         <v>8</v>
       </c>
@@ -6473,7 +6477,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="113" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A113">
         <v>8</v>
       </c>
@@ -6487,7 +6491,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="114" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A114">
         <v>8</v>
       </c>
@@ -6510,7 +6514,7 @@
         <v>570</v>
       </c>
     </row>
-    <row r="115" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A115">
         <v>8</v>
       </c>
@@ -6533,7 +6537,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="116" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A116">
         <v>8</v>
       </c>
@@ -6556,7 +6560,7 @@
         <v>572</v>
       </c>
     </row>
-    <row r="117" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A117">
         <v>8</v>
       </c>
@@ -6579,7 +6583,7 @@
         <v>573</v>
       </c>
     </row>
-    <row r="118" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A118">
         <v>8</v>
       </c>
@@ -6602,7 +6606,7 @@
         <v>574</v>
       </c>
     </row>
-    <row r="119" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A119">
         <v>8</v>
       </c>
@@ -6625,7 +6629,7 @@
         <v>575</v>
       </c>
     </row>
-    <row r="120" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A120">
         <v>8</v>
       </c>
@@ -6638,8 +6642,11 @@
       <c r="D120" t="s">
         <v>554</v>
       </c>
-    </row>
-    <row r="121" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E120" t="s">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="121" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A121">
         <v>8</v>
       </c>
@@ -6653,7 +6660,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="122" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A122">
         <v>9</v>
       </c>
@@ -6676,7 +6683,7 @@
         <v>581</v>
       </c>
     </row>
-    <row r="123" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A123">
         <v>9</v>
       </c>
@@ -6699,7 +6706,7 @@
         <v>584</v>
       </c>
     </row>
-    <row r="124" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A124">
         <v>9</v>
       </c>
@@ -6719,7 +6726,7 @@
         <v>585</v>
       </c>
     </row>
-    <row r="125" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A125">
         <v>9</v>
       </c>
@@ -6739,7 +6746,7 @@
         <v>587</v>
       </c>
     </row>
-    <row r="126" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A126">
         <v>9</v>
       </c>
@@ -6762,7 +6769,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="127" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A127">
         <v>9</v>
       </c>
@@ -6776,7 +6783,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="128" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A128">
         <v>9</v>
       </c>
@@ -6790,7 +6797,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="129" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A129">
         <v>9</v>
       </c>
@@ -6804,7 +6811,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="130" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A130">
         <v>9</v>
       </c>
@@ -6818,7 +6825,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="131" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A131">
         <v>9</v>
       </c>
@@ -6832,7 +6839,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="132" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A132">
         <v>9</v>
       </c>
@@ -6846,7 +6853,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="133" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A133">
         <v>9</v>
       </c>
@@ -6860,7 +6867,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="134" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A134">
         <v>9</v>
       </c>
@@ -6874,7 +6881,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="135" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A135">
         <v>9</v>
       </c>
@@ -6888,7 +6895,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="136" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A136">
         <v>9</v>
       </c>
@@ -6902,7 +6909,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="137" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A137">
         <v>10</v>
       </c>
@@ -6925,7 +6932,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="138" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A138">
         <v>10</v>
       </c>
@@ -6948,7 +6955,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="139" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A139">
         <v>10</v>
       </c>
@@ -6971,7 +6978,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="140" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A140">
         <v>10</v>
       </c>
@@ -6994,7 +7001,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="141" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A141">
         <v>10</v>
       </c>
@@ -7017,7 +7024,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="142" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A142">
         <v>10</v>
       </c>
@@ -7040,7 +7047,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="143" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A143">
         <v>10</v>
       </c>
@@ -7063,7 +7070,7 @@
         <v>623</v>
       </c>
     </row>
-    <row r="144" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A144">
         <v>10</v>
       </c>
@@ -7086,7 +7093,7 @@
         <v>626</v>
       </c>
     </row>
-    <row r="145" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A145">
         <v>10</v>
       </c>
@@ -7109,7 +7116,7 @@
         <v>629</v>
       </c>
     </row>
-    <row r="146" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A146">
         <v>10</v>
       </c>
@@ -7132,7 +7139,7 @@
         <v>632</v>
       </c>
     </row>
-    <row r="147" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A147">
         <v>10</v>
       </c>
@@ -7155,7 +7162,7 @@
         <v>635</v>
       </c>
     </row>
-    <row r="148" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A148">
         <v>10</v>
       </c>
@@ -7178,7 +7185,7 @@
         <v>638</v>
       </c>
     </row>
-    <row r="149" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A149">
         <v>10</v>
       </c>
@@ -7201,7 +7208,7 @@
         <v>641</v>
       </c>
     </row>
-    <row r="150" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A150">
         <v>10</v>
       </c>
@@ -7224,7 +7231,7 @@
         <v>644</v>
       </c>
     </row>
-    <row r="151" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A151">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
issue #103 cleaning and updating Fortran code for the new mortality model
</commit_message>
<xml_diff>
--- a/data-raw/data.default.xlsx
+++ b/data-raw/data.default.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/trotsiuk/Documents/Research/software/r3PG/data-raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91EF81DE-07A2-5E4F-8014-C289F453FBE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A47CA2A5-5A50-1149-9B29-EEBFA797CD28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1080" yWindow="500" windowWidth="50120" windowHeight="28300" activeTab="2" xr2:uid="{61EEFE5B-6AE1-A641-A9AB-273DC4213F59}"/>
+    <workbookView xWindow="41960" yWindow="6500" windowWidth="33860" windowHeight="28300" activeTab="2" xr2:uid="{61EEFE5B-6AE1-A641-A9AB-273DC4213F59}"/>
   </bookViews>
   <sheets>
     <sheet name="parameters" sheetId="8" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1000" uniqueCount="670">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="984" uniqueCount="662">
   <si>
     <t>pFS2</t>
   </si>
@@ -1730,33 +1730,6 @@
     <t>Stem mortality</t>
   </si>
   <si>
-    <t>Volume extracted during the most recent thinning event</t>
-  </si>
-  <si>
-    <t>Latest extracted volume</t>
-  </si>
-  <si>
-    <t>Number of crop trees (x)</t>
-  </si>
-  <si>
-    <t>CropTrees per ha</t>
-  </si>
-  <si>
-    <t>CropTree Mean DBH</t>
-  </si>
-  <si>
-    <t>CropTree Basal area</t>
-  </si>
-  <si>
-    <t>CropTree volume</t>
-  </si>
-  <si>
-    <t>CropTree Height</t>
-  </si>
-  <si>
-    <t>CropTree Stem DM</t>
-  </si>
-  <si>
     <t>var_8_15</t>
   </si>
   <si>
@@ -1970,9 +1943,6 @@
     <t>apar</t>
   </si>
   <si>
-    <t>test_output</t>
-  </si>
-  <si>
     <t>beta0</t>
   </si>
   <si>
@@ -2012,31 +1982,37 @@
     <t>mort_thinn_total</t>
   </si>
   <si>
-    <t>ave_lt_fN</t>
-  </si>
-  <si>
-    <t>ave_lt_fT</t>
-  </si>
-  <si>
-    <t>ave_lt_fPhys</t>
-  </si>
-  <si>
-    <t>lt_fN</t>
-  </si>
-  <si>
-    <t>lt_fT</t>
-  </si>
-  <si>
-    <t>lt_fPhys</t>
-  </si>
-  <si>
     <t>dbh_total</t>
   </si>
   <si>
     <t>stems_n_total</t>
   </si>
   <si>
-    <t>Stems number of the active cohorts</t>
+    <t>var_8_11</t>
+  </si>
+  <si>
+    <t>var_8_12</t>
+  </si>
+  <si>
+    <t>var_8_13</t>
+  </si>
+  <si>
+    <t>var_8_14</t>
+  </si>
+  <si>
+    <t>Total number of trees that died due to density-dependent mortality</t>
+  </si>
+  <si>
+    <t>lt_fN_ave</t>
+  </si>
+  <si>
+    <t>lt_fT_ave</t>
+  </si>
+  <si>
+    <t>lt_fPhys_ave</t>
+  </si>
+  <si>
+    <t>Stems number of the alive cohorts</t>
   </si>
 </sst>
 </file>
@@ -2063,9 +2039,10 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
-      <name val="Aptos"/>
+      <sz val="8"/>
+      <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -2095,11 +2072,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2882,10 +2858,10 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
-        <v>648</v>
+        <v>638</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>654</v>
+        <v>644</v>
       </c>
       <c r="C34" s="1"/>
       <c r="D34" s="1">
@@ -2894,10 +2870,10 @@
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
-        <v>649</v>
+        <v>639</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>655</v>
+        <v>645</v>
       </c>
       <c r="C35" s="1"/>
       <c r="D35" s="1">
@@ -2906,10 +2882,10 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
-        <v>650</v>
+        <v>640</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>656</v>
+        <v>646</v>
       </c>
       <c r="C36" s="1"/>
       <c r="D36" s="1">
@@ -2918,10 +2894,10 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
-        <v>651</v>
+        <v>641</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>657</v>
+        <v>647</v>
       </c>
       <c r="C37" s="1"/>
       <c r="D37" s="1">
@@ -2930,10 +2906,10 @@
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
-        <v>652</v>
+        <v>642</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>658</v>
+        <v>648</v>
       </c>
       <c r="C38" s="1"/>
       <c r="D38" s="1">
@@ -2942,10 +2918,10 @@
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
-        <v>653</v>
+        <v>643</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>659</v>
+        <v>649</v>
       </c>
       <c r="C39" s="1"/>
       <c r="D39" s="1">
@@ -5748,7 +5724,7 @@
         <v>3</v>
       </c>
       <c r="C79" t="s">
-        <v>646</v>
+        <v>637</v>
       </c>
       <c r="D79" t="s">
         <v>468</v>
@@ -6447,11 +6423,20 @@
       <c r="B111" s="2">
         <v>5</v>
       </c>
-      <c r="C111" s="3" t="s">
-        <v>647</v>
-      </c>
-      <c r="D111" s="2" t="s">
+      <c r="C111" s="1" t="s">
+        <v>650</v>
+      </c>
+      <c r="D111" t="s">
         <v>554</v>
+      </c>
+      <c r="E111" t="s">
+        <v>657</v>
+      </c>
+      <c r="F111" t="s">
+        <v>305</v>
+      </c>
+      <c r="G111" t="s">
+        <v>563</v>
       </c>
     </row>
     <row r="112" spans="1:7" x14ac:dyDescent="0.2">
@@ -6462,19 +6447,10 @@
         <v>6</v>
       </c>
       <c r="C112" s="1" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="D112" t="s">
         <v>554</v>
-      </c>
-      <c r="E112" t="s">
-        <v>567</v>
-      </c>
-      <c r="F112" t="s">
-        <v>333</v>
-      </c>
-      <c r="G112" t="s">
-        <v>568</v>
       </c>
     </row>
     <row r="113" spans="1:7" x14ac:dyDescent="0.2">
@@ -6485,7 +6461,7 @@
         <v>7</v>
       </c>
       <c r="C113" s="1" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="D113" t="s">
         <v>554</v>
@@ -6499,19 +6475,13 @@
         <v>8</v>
       </c>
       <c r="C114" s="1" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="D114" t="s">
         <v>554</v>
       </c>
       <c r="E114" t="s">
-        <v>569</v>
-      </c>
-      <c r="F114" t="s">
-        <v>305</v>
-      </c>
-      <c r="G114" t="s">
-        <v>570</v>
+        <v>316</v>
       </c>
     </row>
     <row r="115" spans="1:7" x14ac:dyDescent="0.2">
@@ -6522,19 +6492,13 @@
         <v>9</v>
       </c>
       <c r="C115" s="1" t="s">
-        <v>663</v>
+        <v>651</v>
       </c>
       <c r="D115" t="s">
         <v>554</v>
       </c>
       <c r="E115" t="s">
         <v>316</v>
-      </c>
-      <c r="F115" t="s">
-        <v>317</v>
-      </c>
-      <c r="G115" t="s">
-        <v>571</v>
       </c>
     </row>
     <row r="116" spans="1:7" x14ac:dyDescent="0.2">
@@ -6545,19 +6509,13 @@
         <v>10</v>
       </c>
       <c r="C116" s="1" t="s">
-        <v>664</v>
+        <v>652</v>
       </c>
       <c r="D116" t="s">
         <v>554</v>
       </c>
       <c r="E116" t="s">
-        <v>308</v>
-      </c>
-      <c r="F116" t="s">
-        <v>309</v>
-      </c>
-      <c r="G116" t="s">
-        <v>572</v>
+        <v>661</v>
       </c>
     </row>
     <row r="117" spans="1:7" x14ac:dyDescent="0.2">
@@ -6568,19 +6526,10 @@
         <v>11</v>
       </c>
       <c r="C117" s="1" t="s">
-        <v>665</v>
+        <v>653</v>
       </c>
       <c r="D117" t="s">
         <v>554</v>
-      </c>
-      <c r="E117" t="s">
-        <v>332</v>
-      </c>
-      <c r="F117" t="s">
-        <v>333</v>
-      </c>
-      <c r="G117" t="s">
-        <v>573</v>
       </c>
     </row>
     <row r="118" spans="1:7" x14ac:dyDescent="0.2">
@@ -6591,19 +6540,10 @@
         <v>12</v>
       </c>
       <c r="C118" s="1" t="s">
-        <v>666</v>
+        <v>654</v>
       </c>
       <c r="D118" t="s">
         <v>554</v>
-      </c>
-      <c r="E118" t="s">
-        <v>319</v>
-      </c>
-      <c r="F118" t="s">
-        <v>320</v>
-      </c>
-      <c r="G118" t="s">
-        <v>574</v>
       </c>
     </row>
     <row r="119" spans="1:7" x14ac:dyDescent="0.2">
@@ -6614,19 +6554,10 @@
         <v>13</v>
       </c>
       <c r="C119" s="1" t="s">
-        <v>667</v>
+        <v>655</v>
       </c>
       <c r="D119" t="s">
         <v>554</v>
-      </c>
-      <c r="E119" t="s">
-        <v>390</v>
-      </c>
-      <c r="F119" t="s">
-        <v>391</v>
-      </c>
-      <c r="G119" t="s">
-        <v>575</v>
       </c>
     </row>
     <row r="120" spans="1:7" x14ac:dyDescent="0.2">
@@ -6637,13 +6568,10 @@
         <v>14</v>
       </c>
       <c r="C120" s="1" t="s">
-        <v>668</v>
+        <v>656</v>
       </c>
       <c r="D120" t="s">
         <v>554</v>
-      </c>
-      <c r="E120" t="s">
-        <v>669</v>
       </c>
     </row>
     <row r="121" spans="1:7" x14ac:dyDescent="0.2">
@@ -6654,7 +6582,7 @@
         <v>15</v>
       </c>
       <c r="C121" t="s">
-        <v>576</v>
+        <v>567</v>
       </c>
       <c r="D121" t="s">
         <v>554</v>
@@ -6668,19 +6596,19 @@
         <v>1</v>
       </c>
       <c r="C122" t="s">
-        <v>577</v>
+        <v>568</v>
       </c>
       <c r="D122" t="s">
-        <v>578</v>
+        <v>569</v>
       </c>
       <c r="E122" t="s">
-        <v>579</v>
+        <v>570</v>
       </c>
       <c r="F122" t="s">
-        <v>580</v>
+        <v>571</v>
       </c>
       <c r="G122" t="s">
-        <v>581</v>
+        <v>572</v>
       </c>
     </row>
     <row r="123" spans="1:7" x14ac:dyDescent="0.2">
@@ -6691,19 +6619,19 @@
         <v>2</v>
       </c>
       <c r="C123" t="s">
-        <v>582</v>
+        <v>573</v>
       </c>
       <c r="D123" t="s">
-        <v>578</v>
+        <v>569</v>
       </c>
       <c r="E123" t="s">
-        <v>583</v>
+        <v>574</v>
       </c>
       <c r="F123" t="s">
-        <v>580</v>
+        <v>571</v>
       </c>
       <c r="G123" t="s">
-        <v>584</v>
+        <v>575</v>
       </c>
     </row>
     <row r="124" spans="1:7" x14ac:dyDescent="0.2">
@@ -6714,16 +6642,16 @@
         <v>3</v>
       </c>
       <c r="C124" t="s">
-        <v>585</v>
+        <v>576</v>
       </c>
       <c r="D124" t="s">
-        <v>578</v>
+        <v>569</v>
       </c>
       <c r="E124" t="s">
-        <v>586</v>
+        <v>577</v>
       </c>
       <c r="G124" t="s">
-        <v>585</v>
+        <v>576</v>
       </c>
     </row>
     <row r="125" spans="1:7" x14ac:dyDescent="0.2">
@@ -6734,16 +6662,16 @@
         <v>4</v>
       </c>
       <c r="C125" t="s">
-        <v>587</v>
+        <v>578</v>
       </c>
       <c r="D125" t="s">
+        <v>569</v>
+      </c>
+      <c r="E125" t="s">
+        <v>579</v>
+      </c>
+      <c r="G125" t="s">
         <v>578</v>
-      </c>
-      <c r="E125" t="s">
-        <v>588</v>
-      </c>
-      <c r="G125" t="s">
-        <v>587</v>
       </c>
     </row>
     <row r="126" spans="1:7" x14ac:dyDescent="0.2">
@@ -6754,19 +6682,19 @@
         <v>5</v>
       </c>
       <c r="C126" t="s">
-        <v>589</v>
+        <v>580</v>
       </c>
       <c r="D126" t="s">
-        <v>578</v>
+        <v>569</v>
       </c>
       <c r="E126" t="s">
-        <v>590</v>
+        <v>581</v>
       </c>
       <c r="F126" t="s">
         <v>288</v>
       </c>
       <c r="G126" t="s">
-        <v>591</v>
+        <v>582</v>
       </c>
     </row>
     <row r="127" spans="1:7" x14ac:dyDescent="0.2">
@@ -6777,10 +6705,10 @@
         <v>6</v>
       </c>
       <c r="C127" t="s">
-        <v>592</v>
+        <v>583</v>
       </c>
       <c r="D127" t="s">
-        <v>578</v>
+        <v>569</v>
       </c>
     </row>
     <row r="128" spans="1:7" x14ac:dyDescent="0.2">
@@ -6791,10 +6719,10 @@
         <v>7</v>
       </c>
       <c r="C128" t="s">
-        <v>593</v>
+        <v>584</v>
       </c>
       <c r="D128" t="s">
-        <v>578</v>
+        <v>569</v>
       </c>
     </row>
     <row r="129" spans="1:7" x14ac:dyDescent="0.2">
@@ -6805,10 +6733,10 @@
         <v>8</v>
       </c>
       <c r="C129" t="s">
-        <v>594</v>
+        <v>585</v>
       </c>
       <c r="D129" t="s">
-        <v>578</v>
+        <v>569</v>
       </c>
     </row>
     <row r="130" spans="1:7" x14ac:dyDescent="0.2">
@@ -6819,10 +6747,10 @@
         <v>9</v>
       </c>
       <c r="C130" t="s">
-        <v>595</v>
+        <v>586</v>
       </c>
       <c r="D130" t="s">
-        <v>578</v>
+        <v>569</v>
       </c>
     </row>
     <row r="131" spans="1:7" x14ac:dyDescent="0.2">
@@ -6833,10 +6761,10 @@
         <v>10</v>
       </c>
       <c r="C131" t="s">
-        <v>596</v>
+        <v>587</v>
       </c>
       <c r="D131" t="s">
-        <v>578</v>
+        <v>569</v>
       </c>
     </row>
     <row r="132" spans="1:7" x14ac:dyDescent="0.2">
@@ -6847,10 +6775,10 @@
         <v>11</v>
       </c>
       <c r="C132" t="s">
-        <v>597</v>
+        <v>588</v>
       </c>
       <c r="D132" t="s">
-        <v>578</v>
+        <v>569</v>
       </c>
     </row>
     <row r="133" spans="1:7" x14ac:dyDescent="0.2">
@@ -6861,10 +6789,10 @@
         <v>12</v>
       </c>
       <c r="C133" t="s">
-        <v>598</v>
+        <v>589</v>
       </c>
       <c r="D133" t="s">
-        <v>578</v>
+        <v>569</v>
       </c>
     </row>
     <row r="134" spans="1:7" x14ac:dyDescent="0.2">
@@ -6875,10 +6803,10 @@
         <v>13</v>
       </c>
       <c r="C134" t="s">
-        <v>599</v>
+        <v>590</v>
       </c>
       <c r="D134" t="s">
-        <v>578</v>
+        <v>569</v>
       </c>
     </row>
     <row r="135" spans="1:7" x14ac:dyDescent="0.2">
@@ -6889,10 +6817,10 @@
         <v>14</v>
       </c>
       <c r="C135" t="s">
-        <v>600</v>
+        <v>591</v>
       </c>
       <c r="D135" t="s">
-        <v>578</v>
+        <v>569</v>
       </c>
     </row>
     <row r="136" spans="1:7" x14ac:dyDescent="0.2">
@@ -6903,10 +6831,10 @@
         <v>15</v>
       </c>
       <c r="C136" t="s">
-        <v>601</v>
+        <v>592</v>
       </c>
       <c r="D136" t="s">
-        <v>578</v>
+        <v>569</v>
       </c>
     </row>
     <row r="137" spans="1:7" x14ac:dyDescent="0.2">
@@ -6917,19 +6845,19 @@
         <v>1</v>
       </c>
       <c r="C137" t="s">
-        <v>602</v>
+        <v>593</v>
       </c>
       <c r="D137" t="s">
-        <v>603</v>
+        <v>594</v>
       </c>
       <c r="E137" t="s">
-        <v>604</v>
+        <v>595</v>
       </c>
       <c r="F137" t="s">
         <v>128</v>
       </c>
       <c r="G137" t="s">
-        <v>605</v>
+        <v>596</v>
       </c>
     </row>
     <row r="138" spans="1:7" x14ac:dyDescent="0.2">
@@ -6940,19 +6868,19 @@
         <v>2</v>
       </c>
       <c r="C138" t="s">
-        <v>606</v>
+        <v>597</v>
       </c>
       <c r="D138" t="s">
-        <v>603</v>
+        <v>594</v>
       </c>
       <c r="E138" t="s">
-        <v>607</v>
+        <v>598</v>
       </c>
       <c r="F138" t="s">
         <v>128</v>
       </c>
       <c r="G138" t="s">
-        <v>608</v>
+        <v>599</v>
       </c>
     </row>
     <row r="139" spans="1:7" x14ac:dyDescent="0.2">
@@ -6963,19 +6891,19 @@
         <v>3</v>
       </c>
       <c r="C139" t="s">
-        <v>609</v>
+        <v>600</v>
       </c>
       <c r="D139" t="s">
-        <v>603</v>
+        <v>594</v>
       </c>
       <c r="E139" t="s">
-        <v>610</v>
+        <v>601</v>
       </c>
       <c r="F139" t="s">
         <v>128</v>
       </c>
       <c r="G139" t="s">
-        <v>611</v>
+        <v>602</v>
       </c>
     </row>
     <row r="140" spans="1:7" x14ac:dyDescent="0.2">
@@ -6986,19 +6914,19 @@
         <v>4</v>
       </c>
       <c r="C140" t="s">
-        <v>612</v>
+        <v>603</v>
       </c>
       <c r="D140" t="s">
-        <v>603</v>
+        <v>594</v>
       </c>
       <c r="E140" t="s">
-        <v>613</v>
+        <v>604</v>
       </c>
       <c r="F140" t="s">
         <v>128</v>
       </c>
       <c r="G140" t="s">
-        <v>614</v>
+        <v>605</v>
       </c>
     </row>
     <row r="141" spans="1:7" x14ac:dyDescent="0.2">
@@ -7009,19 +6937,19 @@
         <v>5</v>
       </c>
       <c r="C141" t="s">
-        <v>615</v>
+        <v>606</v>
       </c>
       <c r="D141" t="s">
-        <v>603</v>
+        <v>594</v>
       </c>
       <c r="E141" t="s">
-        <v>616</v>
+        <v>607</v>
       </c>
       <c r="F141" t="s">
         <v>128</v>
       </c>
       <c r="G141" t="s">
-        <v>617</v>
+        <v>608</v>
       </c>
     </row>
     <row r="142" spans="1:7" x14ac:dyDescent="0.2">
@@ -7032,19 +6960,19 @@
         <v>6</v>
       </c>
       <c r="C142" t="s">
-        <v>618</v>
+        <v>609</v>
       </c>
       <c r="D142" t="s">
-        <v>603</v>
+        <v>594</v>
       </c>
       <c r="E142" t="s">
-        <v>619</v>
+        <v>610</v>
       </c>
       <c r="F142" t="s">
         <v>128</v>
       </c>
       <c r="G142" t="s">
-        <v>620</v>
+        <v>611</v>
       </c>
     </row>
     <row r="143" spans="1:7" x14ac:dyDescent="0.2">
@@ -7055,19 +6983,19 @@
         <v>7</v>
       </c>
       <c r="C143" t="s">
-        <v>621</v>
+        <v>612</v>
       </c>
       <c r="D143" t="s">
-        <v>603</v>
+        <v>594</v>
       </c>
       <c r="E143" t="s">
-        <v>622</v>
+        <v>613</v>
       </c>
       <c r="F143" t="s">
         <v>367</v>
       </c>
       <c r="G143" t="s">
-        <v>623</v>
+        <v>614</v>
       </c>
     </row>
     <row r="144" spans="1:7" x14ac:dyDescent="0.2">
@@ -7078,19 +7006,19 @@
         <v>8</v>
       </c>
       <c r="C144" t="s">
-        <v>624</v>
+        <v>615</v>
       </c>
       <c r="D144" t="s">
-        <v>603</v>
+        <v>594</v>
       </c>
       <c r="E144" t="s">
-        <v>625</v>
+        <v>616</v>
       </c>
       <c r="F144" t="s">
         <v>367</v>
       </c>
       <c r="G144" t="s">
-        <v>626</v>
+        <v>617</v>
       </c>
     </row>
     <row r="145" spans="1:7" x14ac:dyDescent="0.2">
@@ -7101,19 +7029,19 @@
         <v>9</v>
       </c>
       <c r="C145" t="s">
-        <v>627</v>
+        <v>618</v>
       </c>
       <c r="D145" t="s">
-        <v>603</v>
+        <v>594</v>
       </c>
       <c r="E145" t="s">
-        <v>628</v>
+        <v>619</v>
       </c>
       <c r="F145" t="s">
         <v>367</v>
       </c>
       <c r="G145" t="s">
-        <v>629</v>
+        <v>620</v>
       </c>
     </row>
     <row r="146" spans="1:7" x14ac:dyDescent="0.2">
@@ -7124,19 +7052,19 @@
         <v>10</v>
       </c>
       <c r="C146" t="s">
-        <v>630</v>
+        <v>621</v>
       </c>
       <c r="D146" t="s">
-        <v>603</v>
+        <v>594</v>
       </c>
       <c r="E146" t="s">
-        <v>631</v>
+        <v>622</v>
       </c>
       <c r="F146" t="s">
         <v>367</v>
       </c>
       <c r="G146" t="s">
-        <v>632</v>
+        <v>623</v>
       </c>
     </row>
     <row r="147" spans="1:7" x14ac:dyDescent="0.2">
@@ -7147,19 +7075,19 @@
         <v>11</v>
       </c>
       <c r="C147" t="s">
-        <v>633</v>
+        <v>624</v>
       </c>
       <c r="D147" t="s">
-        <v>603</v>
+        <v>594</v>
       </c>
       <c r="E147" t="s">
-        <v>634</v>
+        <v>625</v>
       </c>
       <c r="F147" t="s">
         <v>367</v>
       </c>
       <c r="G147" t="s">
-        <v>635</v>
+        <v>626</v>
       </c>
     </row>
     <row r="148" spans="1:7" x14ac:dyDescent="0.2">
@@ -7170,19 +7098,19 @@
         <v>12</v>
       </c>
       <c r="C148" t="s">
-        <v>636</v>
+        <v>627</v>
       </c>
       <c r="D148" t="s">
-        <v>603</v>
+        <v>594</v>
       </c>
       <c r="E148" t="s">
-        <v>637</v>
+        <v>628</v>
       </c>
       <c r="F148" t="s">
         <v>367</v>
       </c>
       <c r="G148" t="s">
-        <v>638</v>
+        <v>629</v>
       </c>
     </row>
     <row r="149" spans="1:7" x14ac:dyDescent="0.2">
@@ -7193,19 +7121,19 @@
         <v>13</v>
       </c>
       <c r="C149" t="s">
-        <v>639</v>
+        <v>630</v>
       </c>
       <c r="D149" t="s">
-        <v>603</v>
+        <v>594</v>
       </c>
       <c r="E149" t="s">
-        <v>640</v>
+        <v>631</v>
       </c>
       <c r="F149" t="s">
         <v>367</v>
       </c>
       <c r="G149" t="s">
-        <v>641</v>
+        <v>632</v>
       </c>
     </row>
     <row r="150" spans="1:7" x14ac:dyDescent="0.2">
@@ -7216,19 +7144,19 @@
         <v>14</v>
       </c>
       <c r="C150" t="s">
-        <v>642</v>
+        <v>633</v>
       </c>
       <c r="D150" t="s">
-        <v>603</v>
+        <v>594</v>
       </c>
       <c r="E150" t="s">
-        <v>643</v>
+        <v>634</v>
       </c>
       <c r="F150" t="s">
         <v>367</v>
       </c>
       <c r="G150" t="s">
-        <v>644</v>
+        <v>635</v>
       </c>
     </row>
     <row r="151" spans="1:7" x14ac:dyDescent="0.2">
@@ -7239,13 +7167,14 @@
         <v>15</v>
       </c>
       <c r="C151" t="s">
-        <v>645</v>
+        <v>636</v>
       </c>
       <c r="D151" t="s">
-        <v>603</v>
+        <v>594</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
issue #104 #103 Implementing the new management based on the tree number or based on the biomass
</commit_message>
<xml_diff>
--- a/data-raw/data.default.xlsx
+++ b/data-raw/data.default.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/trotsiuk/Documents/Research/software/r3PG/data-raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A47CA2A5-5A50-1149-9B29-EEBFA797CD28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40F20C6D-95FF-BA47-A3C4-4F3EFB45FAF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="41960" yWindow="6500" windowWidth="33860" windowHeight="28300" activeTab="2" xr2:uid="{61EEFE5B-6AE1-A641-A9AB-273DC4213F59}"/>
+    <workbookView xWindow="34000" yWindow="2200" windowWidth="33860" windowHeight="28300" activeTab="2" xr2:uid="{61EEFE5B-6AE1-A641-A9AB-273DC4213F59}"/>
   </bookViews>
   <sheets>
     <sheet name="parameters" sheetId="8" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="984" uniqueCount="662">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1022" uniqueCount="682">
   <si>
     <t>pFS2</t>
   </si>
@@ -2013,6 +2013,66 @@
   </si>
   <si>
     <t>Stems number of the alive cohorts</t>
+  </si>
+  <si>
+    <t>mortality_details</t>
+  </si>
+  <si>
+    <t>stems_loss_manag</t>
+  </si>
+  <si>
+    <t>biom_loss_stem_manag</t>
+  </si>
+  <si>
+    <t>biom_loss_root_manag</t>
+  </si>
+  <si>
+    <t>biom_loss_foliage_manag</t>
+  </si>
+  <si>
+    <t>var_11_6</t>
+  </si>
+  <si>
+    <t>var_11_7</t>
+  </si>
+  <si>
+    <t>var_11_8</t>
+  </si>
+  <si>
+    <t>var_11_9</t>
+  </si>
+  <si>
+    <t>var_11_10</t>
+  </si>
+  <si>
+    <t>var_11_11</t>
+  </si>
+  <si>
+    <t>var_11_12</t>
+  </si>
+  <si>
+    <t>var_11_13</t>
+  </si>
+  <si>
+    <t>var_11_14</t>
+  </si>
+  <si>
+    <t>var_11_15</t>
+  </si>
+  <si>
+    <t>var_11_5</t>
+  </si>
+  <si>
+    <t>Number of trees removed due to management</t>
+  </si>
+  <si>
+    <t>Stem biomass removed due to management</t>
+  </si>
+  <si>
+    <t>Root biomass removed due to management</t>
+  </si>
+  <si>
+    <t>Foliage biomass remoed due to management</t>
   </si>
 </sst>
 </file>
@@ -4079,7 +4139,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA3706E6-9BD2-3A49-A255-D2B55C8D9AB1}">
-  <dimension ref="A1:G151"/>
+  <dimension ref="A1:G166"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="51.1640625" customWidth="1"/>
@@ -7173,6 +7233,240 @@
         <v>594</v>
       </c>
     </row>
+    <row r="152" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A152">
+        <v>11</v>
+      </c>
+      <c r="B152">
+        <v>1</v>
+      </c>
+      <c r="C152" t="s">
+        <v>663</v>
+      </c>
+      <c r="D152" t="s">
+        <v>662</v>
+      </c>
+      <c r="E152" t="s">
+        <v>678</v>
+      </c>
+      <c r="F152" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="153" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A153">
+        <v>11</v>
+      </c>
+      <c r="B153">
+        <v>2</v>
+      </c>
+      <c r="C153" t="s">
+        <v>664</v>
+      </c>
+      <c r="D153" t="s">
+        <v>662</v>
+      </c>
+      <c r="E153" t="s">
+        <v>679</v>
+      </c>
+      <c r="F153" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="154" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A154">
+        <v>11</v>
+      </c>
+      <c r="B154">
+        <v>3</v>
+      </c>
+      <c r="C154" t="s">
+        <v>665</v>
+      </c>
+      <c r="D154" t="s">
+        <v>662</v>
+      </c>
+      <c r="E154" t="s">
+        <v>680</v>
+      </c>
+      <c r="F154" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="155" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A155">
+        <v>11</v>
+      </c>
+      <c r="B155">
+        <v>4</v>
+      </c>
+      <c r="C155" t="s">
+        <v>666</v>
+      </c>
+      <c r="D155" t="s">
+        <v>662</v>
+      </c>
+      <c r="E155" t="s">
+        <v>681</v>
+      </c>
+      <c r="F155" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="156" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A156">
+        <v>11</v>
+      </c>
+      <c r="B156">
+        <v>5</v>
+      </c>
+      <c r="C156" t="s">
+        <v>677</v>
+      </c>
+      <c r="D156" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="157" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A157">
+        <v>11</v>
+      </c>
+      <c r="B157">
+        <v>6</v>
+      </c>
+      <c r="C157" t="s">
+        <v>667</v>
+      </c>
+      <c r="D157" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="158" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A158">
+        <v>11</v>
+      </c>
+      <c r="B158">
+        <v>7</v>
+      </c>
+      <c r="C158" t="s">
+        <v>668</v>
+      </c>
+      <c r="D158" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="159" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A159">
+        <v>11</v>
+      </c>
+      <c r="B159">
+        <v>8</v>
+      </c>
+      <c r="C159" t="s">
+        <v>669</v>
+      </c>
+      <c r="D159" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="160" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A160">
+        <v>11</v>
+      </c>
+      <c r="B160">
+        <v>9</v>
+      </c>
+      <c r="C160" t="s">
+        <v>670</v>
+      </c>
+      <c r="D160" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="161" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A161">
+        <v>11</v>
+      </c>
+      <c r="B161">
+        <v>10</v>
+      </c>
+      <c r="C161" t="s">
+        <v>671</v>
+      </c>
+      <c r="D161" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="162" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A162">
+        <v>11</v>
+      </c>
+      <c r="B162">
+        <v>11</v>
+      </c>
+      <c r="C162" t="s">
+        <v>672</v>
+      </c>
+      <c r="D162" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="163" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A163">
+        <v>11</v>
+      </c>
+      <c r="B163">
+        <v>12</v>
+      </c>
+      <c r="C163" t="s">
+        <v>673</v>
+      </c>
+      <c r="D163" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="164" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A164">
+        <v>11</v>
+      </c>
+      <c r="B164">
+        <v>13</v>
+      </c>
+      <c r="C164" t="s">
+        <v>674</v>
+      </c>
+      <c r="D164" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="165" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A165">
+        <v>11</v>
+      </c>
+      <c r="B165">
+        <v>14</v>
+      </c>
+      <c r="C165" t="s">
+        <v>675</v>
+      </c>
+      <c r="D165" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="166" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A166">
+        <v>11</v>
+      </c>
+      <c r="B166">
+        <v>15</v>
+      </c>
+      <c r="C166" t="s">
+        <v>676</v>
+      </c>
+      <c r="D166" t="s">
+        <v>662</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
stress related mortality: - adjust the mortality output to the standard format - reset mortality to 0 if nothing was done
</commit_message>
<xml_diff>
--- a/data-raw/data.default.xlsx
+++ b/data-raw/data.default.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10309"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/trotsiuk/Documents/Research/software/r3PG/data-raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40F20C6D-95FF-BA47-A3C4-4F3EFB45FAF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A696D98-0593-CB41-9451-677977712FB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="34000" yWindow="2200" windowWidth="33860" windowHeight="28300" activeTab="2" xr2:uid="{61EEFE5B-6AE1-A641-A9AB-273DC4213F59}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1022" uniqueCount="682">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1030" uniqueCount="686">
   <si>
     <t>pFS2</t>
   </si>
@@ -2030,15 +2030,6 @@
     <t>biom_loss_foliage_manag</t>
   </si>
   <si>
-    <t>var_11_6</t>
-  </si>
-  <si>
-    <t>var_11_7</t>
-  </si>
-  <si>
-    <t>var_11_8</t>
-  </si>
-  <si>
     <t>var_11_9</t>
   </si>
   <si>
@@ -2060,9 +2051,6 @@
     <t>var_11_15</t>
   </si>
   <si>
-    <t>var_11_5</t>
-  </si>
-  <si>
     <t>Number of trees removed due to management</t>
   </si>
   <si>
@@ -2073,6 +2061,30 @@
   </si>
   <si>
     <t>Foliage biomass remoed due to management</t>
+  </si>
+  <si>
+    <t>stems_loss_stress</t>
+  </si>
+  <si>
+    <t>biom_loss_stem_stress</t>
+  </si>
+  <si>
+    <t>biom_loss_root_stress</t>
+  </si>
+  <si>
+    <t>biom_loss_foliage_stress</t>
+  </si>
+  <si>
+    <t>Number of trees removed due to stress related mortality</t>
+  </si>
+  <si>
+    <t>Stem biomass removed due to stress related mortality</t>
+  </si>
+  <si>
+    <t>Root biomass removed due to stress related mortality</t>
+  </si>
+  <si>
+    <t>Foliage biomass remoed due to stress related mortality</t>
   </si>
 </sst>
 </file>
@@ -7247,7 +7259,7 @@
         <v>662</v>
       </c>
       <c r="E152" t="s">
-        <v>678</v>
+        <v>674</v>
       </c>
       <c r="F152" t="s">
         <v>305</v>
@@ -7267,7 +7279,7 @@
         <v>662</v>
       </c>
       <c r="E153" t="s">
-        <v>679</v>
+        <v>675</v>
       </c>
       <c r="F153" t="s">
         <v>391</v>
@@ -7287,7 +7299,7 @@
         <v>662</v>
       </c>
       <c r="E154" t="s">
-        <v>680</v>
+        <v>676</v>
       </c>
       <c r="F154" t="s">
         <v>391</v>
@@ -7307,7 +7319,7 @@
         <v>662</v>
       </c>
       <c r="E155" t="s">
-        <v>681</v>
+        <v>677</v>
       </c>
       <c r="F155" t="s">
         <v>391</v>
@@ -7321,10 +7333,16 @@
         <v>5</v>
       </c>
       <c r="C156" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="D156" t="s">
         <v>662</v>
+      </c>
+      <c r="E156" t="s">
+        <v>682</v>
+      </c>
+      <c r="F156" t="s">
+        <v>305</v>
       </c>
     </row>
     <row r="157" spans="1:7" x14ac:dyDescent="0.2">
@@ -7335,10 +7353,16 @@
         <v>6</v>
       </c>
       <c r="C157" t="s">
-        <v>667</v>
+        <v>679</v>
       </c>
       <c r="D157" t="s">
         <v>662</v>
+      </c>
+      <c r="E157" t="s">
+        <v>683</v>
+      </c>
+      <c r="F157" t="s">
+        <v>391</v>
       </c>
     </row>
     <row r="158" spans="1:7" x14ac:dyDescent="0.2">
@@ -7349,10 +7373,16 @@
         <v>7</v>
       </c>
       <c r="C158" t="s">
-        <v>668</v>
+        <v>680</v>
       </c>
       <c r="D158" t="s">
         <v>662</v>
+      </c>
+      <c r="E158" t="s">
+        <v>684</v>
+      </c>
+      <c r="F158" t="s">
+        <v>391</v>
       </c>
     </row>
     <row r="159" spans="1:7" x14ac:dyDescent="0.2">
@@ -7363,10 +7393,16 @@
         <v>8</v>
       </c>
       <c r="C159" t="s">
-        <v>669</v>
+        <v>681</v>
       </c>
       <c r="D159" t="s">
         <v>662</v>
+      </c>
+      <c r="E159" t="s">
+        <v>685</v>
+      </c>
+      <c r="F159" t="s">
+        <v>391</v>
       </c>
     </row>
     <row r="160" spans="1:7" x14ac:dyDescent="0.2">
@@ -7377,7 +7413,7 @@
         <v>9</v>
       </c>
       <c r="C160" t="s">
-        <v>670</v>
+        <v>667</v>
       </c>
       <c r="D160" t="s">
         <v>662</v>
@@ -7391,7 +7427,7 @@
         <v>10</v>
       </c>
       <c r="C161" t="s">
-        <v>671</v>
+        <v>668</v>
       </c>
       <c r="D161" t="s">
         <v>662</v>
@@ -7405,7 +7441,7 @@
         <v>11</v>
       </c>
       <c r="C162" t="s">
-        <v>672</v>
+        <v>669</v>
       </c>
       <c r="D162" t="s">
         <v>662</v>
@@ -7419,7 +7455,7 @@
         <v>12</v>
       </c>
       <c r="C163" t="s">
-        <v>673</v>
+        <v>670</v>
       </c>
       <c r="D163" t="s">
         <v>662</v>
@@ -7433,7 +7469,7 @@
         <v>13</v>
       </c>
       <c r="C164" t="s">
-        <v>674</v>
+        <v>671</v>
       </c>
       <c r="D164" t="s">
         <v>662</v>
@@ -7447,7 +7483,7 @@
         <v>14</v>
       </c>
       <c r="C165" t="s">
-        <v>675</v>
+        <v>672</v>
       </c>
       <c r="D165" t="s">
         <v>662</v>
@@ -7461,7 +7497,7 @@
         <v>15</v>
       </c>
       <c r="C166" t="s">
-        <v>676</v>
+        <v>673</v>
       </c>
       <c r="D166" t="s">
         <v>662</v>

</xml_diff>

<commit_message>
further unification of the mortality part.
</commit_message>
<xml_diff>
--- a/data-raw/data.default.xlsx
+++ b/data-raw/data.default.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/trotsiuk/Documents/Research/software/r3PG/data-raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A696D98-0593-CB41-9451-677977712FB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDF03FDC-2B21-AC49-A84E-0B01CA2D4B5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34000" yWindow="2200" windowWidth="33860" windowHeight="28300" activeTab="2" xr2:uid="{61EEFE5B-6AE1-A641-A9AB-273DC4213F59}"/>
+    <workbookView xWindow="17340" yWindow="500" windowWidth="33860" windowHeight="28300" activeTab="2" xr2:uid="{61EEFE5B-6AE1-A641-A9AB-273DC4213F59}"/>
   </bookViews>
   <sheets>
     <sheet name="parameters" sheetId="8" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1030" uniqueCount="686">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1038" uniqueCount="688">
   <si>
     <t>pFS2</t>
   </si>
@@ -1712,18 +1712,12 @@
     <t>month-1</t>
   </si>
   <si>
-    <t>mort_thinn</t>
-  </si>
-  <si>
     <t>Number of trees that died due to density-dependent mortality</t>
   </si>
   <si>
     <t>Self thinning</t>
   </si>
   <si>
-    <t>mort_stress</t>
-  </si>
-  <si>
     <t>Number of trees that died due to stress-related mortality</t>
   </si>
   <si>
@@ -2030,18 +2024,6 @@
     <t>biom_loss_foliage_manag</t>
   </si>
   <si>
-    <t>var_11_9</t>
-  </si>
-  <si>
-    <t>var_11_10</t>
-  </si>
-  <si>
-    <t>var_11_11</t>
-  </si>
-  <si>
-    <t>var_11_12</t>
-  </si>
-  <si>
     <t>var_11_13</t>
   </si>
   <si>
@@ -2085,6 +2067,30 @@
   </si>
   <si>
     <t>Foliage biomass remoed due to stress related mortality</t>
+  </si>
+  <si>
+    <t>stems_loss_density</t>
+  </si>
+  <si>
+    <t>biom_loss_stem_density</t>
+  </si>
+  <si>
+    <t>biom_loss_root_density</t>
+  </si>
+  <si>
+    <t>biom_loss_foliage_density</t>
+  </si>
+  <si>
+    <t>Number of trees removed due to density dependet mortality</t>
+  </si>
+  <si>
+    <t>Stem biomass removed due to density dependet mortality</t>
+  </si>
+  <si>
+    <t>Root biomass removed due to density dependet mortality</t>
+  </si>
+  <si>
+    <t>Foliage biomass remoed due to density dependet mortality</t>
   </si>
 </sst>
 </file>
@@ -2930,10 +2936,10 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
-        <v>638</v>
+        <v>636</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>644</v>
+        <v>642</v>
       </c>
       <c r="C34" s="1"/>
       <c r="D34" s="1">
@@ -2942,10 +2948,10 @@
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
-        <v>639</v>
+        <v>637</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>645</v>
+        <v>643</v>
       </c>
       <c r="C35" s="1"/>
       <c r="D35" s="1">
@@ -2954,10 +2960,10 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
-        <v>640</v>
+        <v>638</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>646</v>
+        <v>644</v>
       </c>
       <c r="C36" s="1"/>
       <c r="D36" s="1">
@@ -2966,10 +2972,10 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
-        <v>641</v>
+        <v>639</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>647</v>
+        <v>645</v>
       </c>
       <c r="C37" s="1"/>
       <c r="D37" s="1">
@@ -2978,10 +2984,10 @@
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
-        <v>642</v>
+        <v>640</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>648</v>
+        <v>646</v>
       </c>
       <c r="C38" s="1"/>
       <c r="D38" s="1">
@@ -2990,10 +2996,10 @@
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>649</v>
+        <v>647</v>
       </c>
       <c r="C39" s="1"/>
       <c r="D39" s="1">
@@ -5796,7 +5802,7 @@
         <v>3</v>
       </c>
       <c r="C79" t="s">
-        <v>637</v>
+        <v>635</v>
       </c>
       <c r="D79" t="s">
         <v>468</v>
@@ -6450,19 +6456,19 @@
         <v>3</v>
       </c>
       <c r="C109" t="s">
-        <v>561</v>
+        <v>680</v>
       </c>
       <c r="D109" t="s">
         <v>554</v>
       </c>
       <c r="E109" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="F109" t="s">
         <v>305</v>
       </c>
       <c r="G109" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="110" spans="1:7" x14ac:dyDescent="0.2">
@@ -6473,19 +6479,19 @@
         <v>4</v>
       </c>
       <c r="C110" t="s">
-        <v>564</v>
+        <v>672</v>
       </c>
       <c r="D110" t="s">
         <v>554</v>
       </c>
       <c r="E110" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="F110" t="s">
         <v>305</v>
       </c>
       <c r="G110" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
     </row>
     <row r="111" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
@@ -6496,19 +6502,19 @@
         <v>5</v>
       </c>
       <c r="C111" s="1" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="D111" t="s">
         <v>554</v>
       </c>
       <c r="E111" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="F111" t="s">
         <v>305</v>
       </c>
       <c r="G111" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="112" spans="1:7" x14ac:dyDescent="0.2">
@@ -6519,7 +6525,7 @@
         <v>6</v>
       </c>
       <c r="C112" s="1" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
       <c r="D112" t="s">
         <v>554</v>
@@ -6533,7 +6539,7 @@
         <v>7</v>
       </c>
       <c r="C113" s="1" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="D113" t="s">
         <v>554</v>
@@ -6547,7 +6553,7 @@
         <v>8</v>
       </c>
       <c r="C114" s="1" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="D114" t="s">
         <v>554</v>
@@ -6564,7 +6570,7 @@
         <v>9</v>
       </c>
       <c r="C115" s="1" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="D115" t="s">
         <v>554</v>
@@ -6581,13 +6587,13 @@
         <v>10</v>
       </c>
       <c r="C116" s="1" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="D116" t="s">
         <v>554</v>
       </c>
       <c r="E116" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
     </row>
     <row r="117" spans="1:7" x14ac:dyDescent="0.2">
@@ -6598,7 +6604,7 @@
         <v>11</v>
       </c>
       <c r="C117" s="1" t="s">
-        <v>653</v>
+        <v>651</v>
       </c>
       <c r="D117" t="s">
         <v>554</v>
@@ -6612,7 +6618,7 @@
         <v>12</v>
       </c>
       <c r="C118" s="1" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="D118" t="s">
         <v>554</v>
@@ -6626,7 +6632,7 @@
         <v>13</v>
       </c>
       <c r="C119" s="1" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="D119" t="s">
         <v>554</v>
@@ -6640,7 +6646,7 @@
         <v>14</v>
       </c>
       <c r="C120" s="1" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="D120" t="s">
         <v>554</v>
@@ -6654,7 +6660,7 @@
         <v>15</v>
       </c>
       <c r="C121" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="D121" t="s">
         <v>554</v>
@@ -6668,19 +6674,19 @@
         <v>1</v>
       </c>
       <c r="C122" t="s">
+        <v>566</v>
+      </c>
+      <c r="D122" t="s">
+        <v>567</v>
+      </c>
+      <c r="E122" t="s">
         <v>568</v>
       </c>
-      <c r="D122" t="s">
+      <c r="F122" t="s">
         <v>569</v>
       </c>
-      <c r="E122" t="s">
+      <c r="G122" t="s">
         <v>570</v>
-      </c>
-      <c r="F122" t="s">
-        <v>571</v>
-      </c>
-      <c r="G122" t="s">
-        <v>572</v>
       </c>
     </row>
     <row r="123" spans="1:7" x14ac:dyDescent="0.2">
@@ -6691,19 +6697,19 @@
         <v>2</v>
       </c>
       <c r="C123" t="s">
+        <v>571</v>
+      </c>
+      <c r="D123" t="s">
+        <v>567</v>
+      </c>
+      <c r="E123" t="s">
+        <v>572</v>
+      </c>
+      <c r="F123" t="s">
+        <v>569</v>
+      </c>
+      <c r="G123" t="s">
         <v>573</v>
-      </c>
-      <c r="D123" t="s">
-        <v>569</v>
-      </c>
-      <c r="E123" t="s">
-        <v>574</v>
-      </c>
-      <c r="F123" t="s">
-        <v>571</v>
-      </c>
-      <c r="G123" t="s">
-        <v>575</v>
       </c>
     </row>
     <row r="124" spans="1:7" x14ac:dyDescent="0.2">
@@ -6714,16 +6720,16 @@
         <v>3</v>
       </c>
       <c r="C124" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="D124" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="E124" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="G124" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
     </row>
     <row r="125" spans="1:7" x14ac:dyDescent="0.2">
@@ -6734,16 +6740,16 @@
         <v>4</v>
       </c>
       <c r="C125" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="D125" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="E125" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="G125" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
     </row>
     <row r="126" spans="1:7" x14ac:dyDescent="0.2">
@@ -6754,19 +6760,19 @@
         <v>5</v>
       </c>
       <c r="C126" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="D126" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="E126" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="F126" t="s">
         <v>288</v>
       </c>
       <c r="G126" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
     </row>
     <row r="127" spans="1:7" x14ac:dyDescent="0.2">
@@ -6777,10 +6783,10 @@
         <v>6</v>
       </c>
       <c r="C127" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="D127" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
     </row>
     <row r="128" spans="1:7" x14ac:dyDescent="0.2">
@@ -6791,10 +6797,10 @@
         <v>7</v>
       </c>
       <c r="C128" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="D128" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
     </row>
     <row r="129" spans="1:7" x14ac:dyDescent="0.2">
@@ -6805,10 +6811,10 @@
         <v>8</v>
       </c>
       <c r="C129" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="D129" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
     </row>
     <row r="130" spans="1:7" x14ac:dyDescent="0.2">
@@ -6819,10 +6825,10 @@
         <v>9</v>
       </c>
       <c r="C130" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="D130" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
     </row>
     <row r="131" spans="1:7" x14ac:dyDescent="0.2">
@@ -6833,10 +6839,10 @@
         <v>10</v>
       </c>
       <c r="C131" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="D131" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
     </row>
     <row r="132" spans="1:7" x14ac:dyDescent="0.2">
@@ -6847,10 +6853,10 @@
         <v>11</v>
       </c>
       <c r="C132" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="D132" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
     </row>
     <row r="133" spans="1:7" x14ac:dyDescent="0.2">
@@ -6861,10 +6867,10 @@
         <v>12</v>
       </c>
       <c r="C133" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="D133" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
     </row>
     <row r="134" spans="1:7" x14ac:dyDescent="0.2">
@@ -6875,10 +6881,10 @@
         <v>13</v>
       </c>
       <c r="C134" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="D134" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
     </row>
     <row r="135" spans="1:7" x14ac:dyDescent="0.2">
@@ -6889,10 +6895,10 @@
         <v>14</v>
       </c>
       <c r="C135" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="D135" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
     </row>
     <row r="136" spans="1:7" x14ac:dyDescent="0.2">
@@ -6903,10 +6909,10 @@
         <v>15</v>
       </c>
       <c r="C136" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="D136" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
     </row>
     <row r="137" spans="1:7" x14ac:dyDescent="0.2">
@@ -6917,19 +6923,19 @@
         <v>1</v>
       </c>
       <c r="C137" t="s">
+        <v>591</v>
+      </c>
+      <c r="D137" t="s">
+        <v>592</v>
+      </c>
+      <c r="E137" t="s">
         <v>593</v>
       </c>
-      <c r="D137" t="s">
+      <c r="F137" t="s">
+        <v>128</v>
+      </c>
+      <c r="G137" t="s">
         <v>594</v>
-      </c>
-      <c r="E137" t="s">
-        <v>595</v>
-      </c>
-      <c r="F137" t="s">
-        <v>128</v>
-      </c>
-      <c r="G137" t="s">
-        <v>596</v>
       </c>
     </row>
     <row r="138" spans="1:7" x14ac:dyDescent="0.2">
@@ -6940,19 +6946,19 @@
         <v>2</v>
       </c>
       <c r="C138" t="s">
+        <v>595</v>
+      </c>
+      <c r="D138" t="s">
+        <v>592</v>
+      </c>
+      <c r="E138" t="s">
+        <v>596</v>
+      </c>
+      <c r="F138" t="s">
+        <v>128</v>
+      </c>
+      <c r="G138" t="s">
         <v>597</v>
-      </c>
-      <c r="D138" t="s">
-        <v>594</v>
-      </c>
-      <c r="E138" t="s">
-        <v>598</v>
-      </c>
-      <c r="F138" t="s">
-        <v>128</v>
-      </c>
-      <c r="G138" t="s">
-        <v>599</v>
       </c>
     </row>
     <row r="139" spans="1:7" x14ac:dyDescent="0.2">
@@ -6963,19 +6969,19 @@
         <v>3</v>
       </c>
       <c r="C139" t="s">
+        <v>598</v>
+      </c>
+      <c r="D139" t="s">
+        <v>592</v>
+      </c>
+      <c r="E139" t="s">
+        <v>599</v>
+      </c>
+      <c r="F139" t="s">
+        <v>128</v>
+      </c>
+      <c r="G139" t="s">
         <v>600</v>
-      </c>
-      <c r="D139" t="s">
-        <v>594</v>
-      </c>
-      <c r="E139" t="s">
-        <v>601</v>
-      </c>
-      <c r="F139" t="s">
-        <v>128</v>
-      </c>
-      <c r="G139" t="s">
-        <v>602</v>
       </c>
     </row>
     <row r="140" spans="1:7" x14ac:dyDescent="0.2">
@@ -6986,19 +6992,19 @@
         <v>4</v>
       </c>
       <c r="C140" t="s">
+        <v>601</v>
+      </c>
+      <c r="D140" t="s">
+        <v>592</v>
+      </c>
+      <c r="E140" t="s">
+        <v>602</v>
+      </c>
+      <c r="F140" t="s">
+        <v>128</v>
+      </c>
+      <c r="G140" t="s">
         <v>603</v>
-      </c>
-      <c r="D140" t="s">
-        <v>594</v>
-      </c>
-      <c r="E140" t="s">
-        <v>604</v>
-      </c>
-      <c r="F140" t="s">
-        <v>128</v>
-      </c>
-      <c r="G140" t="s">
-        <v>605</v>
       </c>
     </row>
     <row r="141" spans="1:7" x14ac:dyDescent="0.2">
@@ -7009,19 +7015,19 @@
         <v>5</v>
       </c>
       <c r="C141" t="s">
+        <v>604</v>
+      </c>
+      <c r="D141" t="s">
+        <v>592</v>
+      </c>
+      <c r="E141" t="s">
+        <v>605</v>
+      </c>
+      <c r="F141" t="s">
+        <v>128</v>
+      </c>
+      <c r="G141" t="s">
         <v>606</v>
-      </c>
-      <c r="D141" t="s">
-        <v>594</v>
-      </c>
-      <c r="E141" t="s">
-        <v>607</v>
-      </c>
-      <c r="F141" t="s">
-        <v>128</v>
-      </c>
-      <c r="G141" t="s">
-        <v>608</v>
       </c>
     </row>
     <row r="142" spans="1:7" x14ac:dyDescent="0.2">
@@ -7032,19 +7038,19 @@
         <v>6</v>
       </c>
       <c r="C142" t="s">
+        <v>607</v>
+      </c>
+      <c r="D142" t="s">
+        <v>592</v>
+      </c>
+      <c r="E142" t="s">
+        <v>608</v>
+      </c>
+      <c r="F142" t="s">
+        <v>128</v>
+      </c>
+      <c r="G142" t="s">
         <v>609</v>
-      </c>
-      <c r="D142" t="s">
-        <v>594</v>
-      </c>
-      <c r="E142" t="s">
-        <v>610</v>
-      </c>
-      <c r="F142" t="s">
-        <v>128</v>
-      </c>
-      <c r="G142" t="s">
-        <v>611</v>
       </c>
     </row>
     <row r="143" spans="1:7" x14ac:dyDescent="0.2">
@@ -7055,19 +7061,19 @@
         <v>7</v>
       </c>
       <c r="C143" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
       <c r="D143" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="E143" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="F143" t="s">
         <v>367</v>
       </c>
       <c r="G143" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
     </row>
     <row r="144" spans="1:7" x14ac:dyDescent="0.2">
@@ -7078,19 +7084,19 @@
         <v>8</v>
       </c>
       <c r="C144" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="D144" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="E144" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="F144" t="s">
         <v>367</v>
       </c>
       <c r="G144" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
     </row>
     <row r="145" spans="1:7" x14ac:dyDescent="0.2">
@@ -7101,19 +7107,19 @@
         <v>9</v>
       </c>
       <c r="C145" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
       <c r="D145" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="E145" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="F145" t="s">
         <v>367</v>
       </c>
       <c r="G145" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
     </row>
     <row r="146" spans="1:7" x14ac:dyDescent="0.2">
@@ -7124,19 +7130,19 @@
         <v>10</v>
       </c>
       <c r="C146" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
       <c r="D146" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="E146" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
       <c r="F146" t="s">
         <v>367</v>
       </c>
       <c r="G146" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
     </row>
     <row r="147" spans="1:7" x14ac:dyDescent="0.2">
@@ -7147,19 +7153,19 @@
         <v>11</v>
       </c>
       <c r="C147" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
       <c r="D147" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="E147" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="F147" t="s">
         <v>367</v>
       </c>
       <c r="G147" t="s">
-        <v>626</v>
+        <v>624</v>
       </c>
     </row>
     <row r="148" spans="1:7" x14ac:dyDescent="0.2">
@@ -7170,19 +7176,19 @@
         <v>12</v>
       </c>
       <c r="C148" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="D148" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="E148" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="F148" t="s">
         <v>367</v>
       </c>
       <c r="G148" t="s">
-        <v>629</v>
+        <v>627</v>
       </c>
     </row>
     <row r="149" spans="1:7" x14ac:dyDescent="0.2">
@@ -7193,19 +7199,19 @@
         <v>13</v>
       </c>
       <c r="C149" t="s">
-        <v>630</v>
+        <v>628</v>
       </c>
       <c r="D149" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="E149" t="s">
-        <v>631</v>
+        <v>629</v>
       </c>
       <c r="F149" t="s">
         <v>367</v>
       </c>
       <c r="G149" t="s">
-        <v>632</v>
+        <v>630</v>
       </c>
     </row>
     <row r="150" spans="1:7" x14ac:dyDescent="0.2">
@@ -7216,19 +7222,19 @@
         <v>14</v>
       </c>
       <c r="C150" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="D150" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="E150" t="s">
-        <v>634</v>
+        <v>632</v>
       </c>
       <c r="F150" t="s">
         <v>367</v>
       </c>
       <c r="G150" t="s">
-        <v>635</v>
+        <v>633</v>
       </c>
     </row>
     <row r="151" spans="1:7" x14ac:dyDescent="0.2">
@@ -7239,10 +7245,10 @@
         <v>15</v>
       </c>
       <c r="C151" t="s">
-        <v>636</v>
+        <v>634</v>
       </c>
       <c r="D151" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
     </row>
     <row r="152" spans="1:7" x14ac:dyDescent="0.2">
@@ -7253,13 +7259,13 @@
         <v>1</v>
       </c>
       <c r="C152" t="s">
-        <v>663</v>
+        <v>661</v>
       </c>
       <c r="D152" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="E152" t="s">
-        <v>674</v>
+        <v>668</v>
       </c>
       <c r="F152" t="s">
         <v>305</v>
@@ -7273,13 +7279,13 @@
         <v>2</v>
       </c>
       <c r="C153" t="s">
-        <v>664</v>
+        <v>662</v>
       </c>
       <c r="D153" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="E153" t="s">
-        <v>675</v>
+        <v>669</v>
       </c>
       <c r="F153" t="s">
         <v>391</v>
@@ -7293,13 +7299,13 @@
         <v>3</v>
       </c>
       <c r="C154" t="s">
-        <v>665</v>
+        <v>663</v>
       </c>
       <c r="D154" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="E154" t="s">
-        <v>676</v>
+        <v>670</v>
       </c>
       <c r="F154" t="s">
         <v>391</v>
@@ -7313,13 +7319,13 @@
         <v>4</v>
       </c>
       <c r="C155" t="s">
-        <v>666</v>
+        <v>664</v>
       </c>
       <c r="D155" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="E155" t="s">
-        <v>677</v>
+        <v>671</v>
       </c>
       <c r="F155" t="s">
         <v>391</v>
@@ -7333,13 +7339,13 @@
         <v>5</v>
       </c>
       <c r="C156" t="s">
-        <v>678</v>
+        <v>672</v>
       </c>
       <c r="D156" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="E156" t="s">
-        <v>682</v>
+        <v>676</v>
       </c>
       <c r="F156" t="s">
         <v>305</v>
@@ -7353,13 +7359,13 @@
         <v>6</v>
       </c>
       <c r="C157" t="s">
-        <v>679</v>
+        <v>673</v>
       </c>
       <c r="D157" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="E157" t="s">
-        <v>683</v>
+        <v>677</v>
       </c>
       <c r="F157" t="s">
         <v>391</v>
@@ -7373,13 +7379,13 @@
         <v>7</v>
       </c>
       <c r="C158" t="s">
-        <v>680</v>
+        <v>674</v>
       </c>
       <c r="D158" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="E158" t="s">
-        <v>684</v>
+        <v>678</v>
       </c>
       <c r="F158" t="s">
         <v>391</v>
@@ -7393,13 +7399,13 @@
         <v>8</v>
       </c>
       <c r="C159" t="s">
-        <v>681</v>
+        <v>675</v>
       </c>
       <c r="D159" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="E159" t="s">
-        <v>685</v>
+        <v>679</v>
       </c>
       <c r="F159" t="s">
         <v>391</v>
@@ -7413,13 +7419,19 @@
         <v>9</v>
       </c>
       <c r="C160" t="s">
-        <v>667</v>
+        <v>680</v>
       </c>
       <c r="D160" t="s">
-        <v>662</v>
-      </c>
-    </row>
-    <row r="161" spans="1:4" x14ac:dyDescent="0.2">
+        <v>660</v>
+      </c>
+      <c r="E160" t="s">
+        <v>684</v>
+      </c>
+      <c r="F160" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="161" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A161">
         <v>11</v>
       </c>
@@ -7427,13 +7439,19 @@
         <v>10</v>
       </c>
       <c r="C161" t="s">
-        <v>668</v>
+        <v>681</v>
       </c>
       <c r="D161" t="s">
-        <v>662</v>
-      </c>
-    </row>
-    <row r="162" spans="1:4" x14ac:dyDescent="0.2">
+        <v>660</v>
+      </c>
+      <c r="E161" t="s">
+        <v>685</v>
+      </c>
+      <c r="F161" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="162" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A162">
         <v>11</v>
       </c>
@@ -7441,13 +7459,19 @@
         <v>11</v>
       </c>
       <c r="C162" t="s">
-        <v>669</v>
+        <v>682</v>
       </c>
       <c r="D162" t="s">
-        <v>662</v>
-      </c>
-    </row>
-    <row r="163" spans="1:4" x14ac:dyDescent="0.2">
+        <v>660</v>
+      </c>
+      <c r="E162" t="s">
+        <v>686</v>
+      </c>
+      <c r="F162" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="163" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A163">
         <v>11</v>
       </c>
@@ -7455,13 +7479,19 @@
         <v>12</v>
       </c>
       <c r="C163" t="s">
-        <v>670</v>
+        <v>683</v>
       </c>
       <c r="D163" t="s">
-        <v>662</v>
-      </c>
-    </row>
-    <row r="164" spans="1:4" x14ac:dyDescent="0.2">
+        <v>660</v>
+      </c>
+      <c r="E163" t="s">
+        <v>687</v>
+      </c>
+      <c r="F163" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="164" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A164">
         <v>11</v>
       </c>
@@ -7469,13 +7499,13 @@
         <v>13</v>
       </c>
       <c r="C164" t="s">
-        <v>671</v>
+        <v>665</v>
       </c>
       <c r="D164" t="s">
-        <v>662</v>
-      </c>
-    </row>
-    <row r="165" spans="1:4" x14ac:dyDescent="0.2">
+        <v>660</v>
+      </c>
+    </row>
+    <row r="165" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A165">
         <v>11</v>
       </c>
@@ -7483,13 +7513,13 @@
         <v>14</v>
       </c>
       <c r="C165" t="s">
-        <v>672</v>
+        <v>666</v>
       </c>
       <c r="D165" t="s">
-        <v>662</v>
-      </c>
-    </row>
-    <row r="166" spans="1:4" x14ac:dyDescent="0.2">
+        <v>660</v>
+      </c>
+    </row>
+    <row r="166" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A166">
         <v>11</v>
       </c>
@@ -7497,10 +7527,10 @@
         <v>15</v>
       </c>
       <c r="C166" t="s">
-        <v>673</v>
+        <v>667</v>
       </c>
       <c r="D166" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added lt_fT and lt_fPhys as outputs to provide 10-year averages.
</commit_message>
<xml_diff>
--- a/data-raw/data.default.xlsx
+++ b/data-raw/data.default.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/trotsiuk/Documents/Research/software/r3PG/data-raw/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Forrester\Models\3-PG\r3PG_mortality_management_defoliation\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35F903BF-3827-1F46-9732-B29A8B79E7A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{391A5BF4-4965-477B-B28F-85BC38AF9E52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1420" yWindow="500" windowWidth="32960" windowHeight="28300" activeTab="2" xr2:uid="{61EEFE5B-6AE1-A641-A9AB-273DC4213F59}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{61EEFE5B-6AE1-A641-A9AB-273DC4213F59}"/>
   </bookViews>
   <sheets>
     <sheet name="parameters" sheetId="8" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1263" uniqueCount="745">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1264" uniqueCount="747">
   <si>
     <t>pFS2</t>
   </si>
@@ -1986,12 +1986,6 @@
     <t>stems_n_total</t>
   </si>
   <si>
-    <t>var_8_11</t>
-  </si>
-  <si>
-    <t>var_8_12</t>
-  </si>
-  <si>
     <t>var_8_13</t>
   </si>
   <si>
@@ -2266,13 +2260,25 @@
   </si>
   <si>
     <t>biom_loss_foliage_def</t>
+  </si>
+  <si>
+    <t>lt_fT</t>
+  </si>
+  <si>
+    <t>lt_fPhys</t>
+  </si>
+  <si>
+    <t>10-year average fT</t>
+  </si>
+  <si>
+    <t>10-year average fPhys</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="7">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -2667,9 +2673,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E287297-02C0-BF44-BF0C-8FADE2A87F8F}">
   <dimension ref="A1:D89"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4">
       <c r="A1" t="s">
         <v>117</v>
       </c>
@@ -2683,7 +2689,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -2697,7 +2703,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -2711,7 +2717,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -2725,7 +2731,7 @@
         <v>9.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -2739,7 +2745,7 @@
         <v>2.4</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -2753,7 +2759,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -2767,7 +2773,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -2781,7 +2787,7 @@
         <v>2.7E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -2795,7 +2801,7 @@
         <v>1E-3</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -2809,7 +2815,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -2823,7 +2829,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:4">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -2837,7 +2843,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -2851,7 +2857,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:4">
       <c r="A14" t="s">
         <v>13</v>
       </c>
@@ -2865,7 +2871,7 @@
         <v>8.5</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:4">
       <c r="A15" t="s">
         <v>14</v>
       </c>
@@ -2879,7 +2885,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:4">
       <c r="A16" t="s">
         <v>15</v>
       </c>
@@ -2893,7 +2899,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4">
       <c r="A17" t="s">
         <v>16</v>
       </c>
@@ -2907,7 +2913,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4">
       <c r="A18" t="s">
         <v>17</v>
       </c>
@@ -2921,7 +2927,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:4">
       <c r="A19" t="s">
         <v>18</v>
       </c>
@@ -2935,7 +2941,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:4">
       <c r="A20" t="s">
         <v>19</v>
       </c>
@@ -2949,7 +2955,7 @@
         <v>1.4</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:4">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -2963,7 +2969,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:4">
       <c r="A22" t="s">
         <v>21</v>
       </c>
@@ -2977,7 +2983,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:4">
       <c r="A23" t="s">
         <v>22</v>
       </c>
@@ -2991,7 +2997,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:4">
       <c r="A24" t="s">
         <v>23</v>
       </c>
@@ -3005,7 +3011,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:4">
       <c r="A25" t="s">
         <v>24</v>
       </c>
@@ -3019,7 +3025,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:4">
       <c r="A26" t="s">
         <v>25</v>
       </c>
@@ -3033,7 +3039,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:4">
       <c r="A27" t="s">
         <v>26</v>
       </c>
@@ -3047,7 +3053,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:4">
       <c r="A28" t="s">
         <v>27</v>
       </c>
@@ -3061,7 +3067,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:4">
       <c r="A29" t="s">
         <v>28</v>
       </c>
@@ -3075,7 +3081,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:4">
       <c r="A30" t="s">
         <v>29</v>
       </c>
@@ -3089,7 +3095,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:4">
       <c r="A31" t="s">
         <v>30</v>
       </c>
@@ -3103,7 +3109,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:4">
       <c r="A32" t="s">
         <v>31</v>
       </c>
@@ -3117,7 +3123,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:4">
       <c r="A33" t="s">
         <v>32</v>
       </c>
@@ -3131,7 +3137,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:4">
       <c r="A34" s="1" t="s">
         <v>636</v>
       </c>
@@ -3143,7 +3149,7 @@
         <v>-20.399999999999999</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:4">
       <c r="A35" s="1" t="s">
         <v>637</v>
       </c>
@@ -3155,7 +3161,7 @@
         <v>1.86</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:4">
       <c r="A36" s="1" t="s">
         <v>638</v>
       </c>
@@ -3167,7 +3173,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:4">
       <c r="A37" s="1" t="s">
         <v>639</v>
       </c>
@@ -3179,7 +3185,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:4">
       <c r="A38" s="1" t="s">
         <v>640</v>
       </c>
@@ -3191,7 +3197,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:4">
       <c r="A39" s="1" t="s">
         <v>641</v>
       </c>
@@ -3203,7 +3209,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:4">
       <c r="A40" t="s">
         <v>33</v>
       </c>
@@ -3217,7 +3223,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:4">
       <c r="A41" t="s">
         <v>34</v>
       </c>
@@ -3231,7 +3237,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:4">
       <c r="A42" t="s">
         <v>35</v>
       </c>
@@ -3245,7 +3251,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:4">
       <c r="A43" t="s">
         <v>36</v>
       </c>
@@ -3259,7 +3265,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:4">
       <c r="A44" t="s">
         <v>37</v>
       </c>
@@ -3273,7 +3279,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:4">
       <c r="A45" t="s">
         <v>38</v>
       </c>
@@ -3287,7 +3293,7 @@
         <v>2.5</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:4">
       <c r="A46" t="s">
         <v>39</v>
       </c>
@@ -3301,7 +3307,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:4">
       <c r="A47" t="s">
         <v>40</v>
       </c>
@@ -3315,7 +3321,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:4">
       <c r="A48" t="s">
         <v>41</v>
       </c>
@@ -3329,7 +3335,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:4">
       <c r="A49" t="s">
         <v>42</v>
       </c>
@@ -3343,7 +3349,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:4">
       <c r="A50" t="s">
         <v>43</v>
       </c>
@@ -3357,7 +3363,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:4">
       <c r="A51" t="s">
         <v>44</v>
       </c>
@@ -3371,7 +3377,7 @@
         <v>0.06</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:4">
       <c r="A52" t="s">
         <v>45</v>
       </c>
@@ -3385,7 +3391,7 @@
         <v>0.47</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:4">
       <c r="A53" t="s">
         <v>46</v>
       </c>
@@ -3399,7 +3405,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:4">
       <c r="A54" t="s">
         <v>47</v>
       </c>
@@ -3413,7 +3419,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:4">
       <c r="A55" t="s">
         <v>48</v>
       </c>
@@ -3427,7 +3433,7 @@
         <v>3.33</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:4">
       <c r="A56" t="s">
         <v>49</v>
       </c>
@@ -3441,7 +3447,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:4">
       <c r="A57" t="s">
         <v>50</v>
       </c>
@@ -3455,7 +3461,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:4">
       <c r="A58" t="s">
         <v>51</v>
       </c>
@@ -3469,7 +3475,7 @@
         <v>0.66</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:4">
       <c r="A59" t="s">
         <v>52</v>
       </c>
@@ -3483,7 +3489,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:4">
       <c r="A60" t="s">
         <v>53</v>
       </c>
@@ -3497,7 +3503,7 @@
         <v>4.4000000000000004</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:4">
       <c r="A61" t="s">
         <v>54</v>
       </c>
@@ -3511,7 +3517,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:4">
       <c r="A62" t="s">
         <v>55</v>
       </c>
@@ -3525,7 +3531,7 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:4">
       <c r="A63" t="s">
         <v>56</v>
       </c>
@@ -3539,7 +3545,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:4">
       <c r="A64" t="s">
         <v>57</v>
       </c>
@@ -3553,7 +3559,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:4">
       <c r="A65" t="s">
         <v>58</v>
       </c>
@@ -3567,7 +3573,7 @@
         <v>0.45</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:4">
       <c r="A66" t="s">
         <v>59</v>
       </c>
@@ -3581,7 +3587,7 @@
         <v>0.45</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:4">
       <c r="A67" t="s">
         <v>60</v>
       </c>
@@ -3595,7 +3601,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:4">
       <c r="A68" t="s">
         <v>68</v>
       </c>
@@ -3609,7 +3615,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:4">
       <c r="A69" t="s">
         <v>61</v>
       </c>
@@ -3623,7 +3629,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:4">
       <c r="A70" t="s">
         <v>62</v>
       </c>
@@ -3637,7 +3643,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:4">
       <c r="A71" t="s">
         <v>63</v>
       </c>
@@ -3651,7 +3657,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:4">
       <c r="A72" t="s">
         <v>64</v>
       </c>
@@ -3665,7 +3671,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:4">
       <c r="A73" t="s">
         <v>65</v>
       </c>
@@ -3679,7 +3685,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:4">
       <c r="A74" t="s">
         <v>66</v>
       </c>
@@ -3693,7 +3699,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:4">
       <c r="A75" t="s">
         <v>67</v>
       </c>
@@ -3707,7 +3713,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:4">
       <c r="A76" t="s">
         <v>69</v>
       </c>
@@ -3721,7 +3727,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:4">
       <c r="A77" t="s">
         <v>70</v>
       </c>
@@ -3735,7 +3741,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:4">
       <c r="A78" t="s">
         <v>71</v>
       </c>
@@ -3749,7 +3755,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:4">
       <c r="A79" t="s">
         <v>72</v>
       </c>
@@ -3763,7 +3769,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:4">
       <c r="A80" t="s">
         <v>73</v>
       </c>
@@ -3777,7 +3783,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:4">
       <c r="A81" t="s">
         <v>74</v>
       </c>
@@ -3791,7 +3797,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:4">
       <c r="A82" t="s">
         <v>75</v>
       </c>
@@ -3805,7 +3811,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:4">
       <c r="A83" t="s">
         <v>76</v>
       </c>
@@ -3819,7 +3825,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:4">
       <c r="A84" t="s">
         <v>77</v>
       </c>
@@ -3833,7 +3839,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:4">
       <c r="A85" t="s">
         <v>78</v>
       </c>
@@ -3847,7 +3853,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:4">
       <c r="A86" t="s">
         <v>109</v>
       </c>
@@ -3861,7 +3867,7 @@
         <v>-90</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:4">
       <c r="A87" t="s">
         <v>110</v>
       </c>
@@ -3875,7 +3881,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:4">
       <c r="A88" t="s">
         <v>111</v>
       </c>
@@ -3889,7 +3895,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:4">
       <c r="A89" t="s">
         <v>112</v>
       </c>
@@ -3905,15 +3911,19 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;"Aptos"&amp;12&amp;KFF0000 OFFICIAL&amp;1#_x000D_</oddHeader>
+    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Aptos"&amp;12&amp;KFF0000 OFFICIAL</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FAF000D6-A72C-6444-9177-22D437B8361A}">
   <dimension ref="A1:D31"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4">
       <c r="A1" t="s">
         <v>117</v>
       </c>
@@ -3927,7 +3937,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
         <v>79</v>
       </c>
@@ -3941,7 +3951,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4">
       <c r="A3" t="s">
         <v>80</v>
       </c>
@@ -3955,7 +3965,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4">
       <c r="A4" t="s">
         <v>81</v>
       </c>
@@ -3969,7 +3979,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4">
       <c r="A5" t="s">
         <v>82</v>
       </c>
@@ -3983,7 +3993,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4">
       <c r="A6" t="s">
         <v>83</v>
       </c>
@@ -3997,7 +4007,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4">
       <c r="A7" t="s">
         <v>84</v>
       </c>
@@ -4011,7 +4021,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4">
       <c r="A8" t="s">
         <v>85</v>
       </c>
@@ -4025,7 +4035,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4">
       <c r="A9" t="s">
         <v>86</v>
       </c>
@@ -4039,7 +4049,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4">
       <c r="A10" t="s">
         <v>87</v>
       </c>
@@ -4053,7 +4063,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4">
       <c r="A11" t="s">
         <v>88</v>
       </c>
@@ -4067,7 +4077,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:4">
       <c r="A12" t="s">
         <v>89</v>
       </c>
@@ -4081,7 +4091,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4">
       <c r="A13" t="s">
         <v>90</v>
       </c>
@@ -4095,7 +4105,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:4">
       <c r="A14" t="s">
         <v>91</v>
       </c>
@@ -4109,7 +4119,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:4">
       <c r="A15" t="s">
         <v>92</v>
       </c>
@@ -4123,7 +4133,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:4">
       <c r="A16" t="s">
         <v>93</v>
       </c>
@@ -4137,7 +4147,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4">
       <c r="A17" t="s">
         <v>94</v>
       </c>
@@ -4151,7 +4161,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4">
       <c r="A18" t="s">
         <v>95</v>
       </c>
@@ -4165,7 +4175,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:4">
       <c r="A19" t="s">
         <v>96</v>
       </c>
@@ -4179,7 +4189,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:4">
       <c r="A20" t="s">
         <v>97</v>
       </c>
@@ -4193,7 +4203,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:4">
       <c r="A21" t="s">
         <v>98</v>
       </c>
@@ -4207,7 +4217,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:4">
       <c r="A22" t="s">
         <v>99</v>
       </c>
@@ -4221,7 +4231,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:4">
       <c r="A23" t="s">
         <v>100</v>
       </c>
@@ -4235,7 +4245,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:4">
       <c r="A24" t="s">
         <v>101</v>
       </c>
@@ -4249,7 +4259,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:4">
       <c r="A25" t="s">
         <v>102</v>
       </c>
@@ -4263,7 +4273,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:4">
       <c r="A26" t="s">
         <v>103</v>
       </c>
@@ -4277,7 +4287,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:4">
       <c r="A27" t="s">
         <v>104</v>
       </c>
@@ -4291,7 +4301,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:4">
       <c r="A28" t="s">
         <v>105</v>
       </c>
@@ -4305,7 +4315,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:4">
       <c r="A29" t="s">
         <v>106</v>
       </c>
@@ -4319,7 +4329,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:4">
       <c r="A30" t="s">
         <v>107</v>
       </c>
@@ -4333,7 +4343,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:4">
       <c r="A31" t="s">
         <v>108</v>
       </c>
@@ -4349,20 +4359,24 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;"Aptos"&amp;12&amp;KFF0000 OFFICIAL&amp;1#_x000D_</oddHeader>
+    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Aptos"&amp;12&amp;KFF0000 OFFICIAL</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA3706E6-9BD2-3A49-A255-D2B55C8D9AB1}">
   <dimension ref="A1:G221"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
   <cols>
-    <col min="3" max="3" width="51.1640625" customWidth="1"/>
+    <col min="3" max="3" width="51.125" customWidth="1"/>
     <col min="4" max="4" width="20" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="179" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>256</v>
       </c>
@@ -4385,7 +4399,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7">
       <c r="A2">
         <v>1</v>
       </c>
@@ -4408,7 +4422,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7">
       <c r="A3">
         <v>1</v>
       </c>
@@ -4431,7 +4445,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7">
       <c r="A4">
         <v>1</v>
       </c>
@@ -4454,7 +4468,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7">
       <c r="A5">
         <v>1</v>
       </c>
@@ -4477,7 +4491,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7">
       <c r="A6">
         <v>1</v>
       </c>
@@ -4500,7 +4514,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7">
       <c r="A7">
         <v>1</v>
       </c>
@@ -4523,7 +4537,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7">
       <c r="A8">
         <v>1</v>
       </c>
@@ -4546,7 +4560,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7">
       <c r="A9">
         <v>1</v>
       </c>
@@ -4569,7 +4583,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7">
       <c r="A10">
         <v>1</v>
       </c>
@@ -4592,7 +4606,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7">
       <c r="A11">
         <v>1</v>
       </c>
@@ -4612,7 +4626,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7">
       <c r="A12">
         <v>1</v>
       </c>
@@ -4635,7 +4649,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7">
       <c r="A13">
         <v>1</v>
       </c>
@@ -4649,7 +4663,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7">
       <c r="A14">
         <v>1</v>
       </c>
@@ -4663,7 +4677,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7">
       <c r="A15">
         <v>1</v>
       </c>
@@ -4677,7 +4691,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7">
       <c r="A16">
         <v>1</v>
       </c>
@@ -4691,7 +4705,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:7">
       <c r="A17" s="4">
         <v>1</v>
       </c>
@@ -4699,13 +4713,13 @@
         <v>16</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>685</v>
+        <v>683</v>
       </c>
       <c r="D17" s="4" t="s">
         <v>261</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:7">
       <c r="A18" s="4">
         <v>1</v>
       </c>
@@ -4713,13 +4727,13 @@
         <v>17</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
       <c r="D18" s="4" t="s">
         <v>261</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:7">
       <c r="A19" s="4">
         <v>1</v>
       </c>
@@ -4727,13 +4741,13 @@
         <v>18</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>687</v>
+        <v>685</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>261</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:7">
       <c r="A20" s="4">
         <v>1</v>
       </c>
@@ -4741,13 +4755,13 @@
         <v>19</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>261</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:7">
       <c r="A21" s="4">
         <v>1</v>
       </c>
@@ -4755,13 +4769,13 @@
         <v>20</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>689</v>
+        <v>687</v>
       </c>
       <c r="D21" s="4" t="s">
         <v>261</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:7">
       <c r="A22">
         <v>2</v>
       </c>
@@ -4784,7 +4798,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:7">
       <c r="A23">
         <v>2</v>
       </c>
@@ -4807,7 +4821,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:7">
       <c r="A24">
         <v>2</v>
       </c>
@@ -4830,7 +4844,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:7">
       <c r="A25">
         <v>2</v>
       </c>
@@ -4853,7 +4867,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:7">
       <c r="A26">
         <v>2</v>
       </c>
@@ -4876,7 +4890,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:7">
       <c r="A27">
         <v>2</v>
       </c>
@@ -4899,7 +4913,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:7">
       <c r="A28">
         <v>2</v>
       </c>
@@ -4922,7 +4936,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:7">
       <c r="A29">
         <v>2</v>
       </c>
@@ -4945,7 +4959,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:7">
       <c r="A30">
         <v>2</v>
       </c>
@@ -4968,7 +4982,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:7">
       <c r="A31">
         <v>2</v>
       </c>
@@ -4991,7 +5005,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:7">
       <c r="A32">
         <v>2</v>
       </c>
@@ -5014,7 +5028,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:7">
       <c r="A33">
         <v>2</v>
       </c>
@@ -5037,7 +5051,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:7">
       <c r="A34">
         <v>2</v>
       </c>
@@ -5060,7 +5074,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:7">
       <c r="A35">
         <v>2</v>
       </c>
@@ -5074,7 +5088,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:7">
       <c r="A36">
         <v>2</v>
       </c>
@@ -5088,7 +5102,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:7">
       <c r="A37" s="4">
         <v>2</v>
       </c>
@@ -5096,13 +5110,13 @@
         <v>16</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>690</v>
+        <v>688</v>
       </c>
       <c r="D37" s="4" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:7">
       <c r="A38" s="4">
         <v>2</v>
       </c>
@@ -5110,13 +5124,13 @@
         <v>17</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>691</v>
+        <v>689</v>
       </c>
       <c r="D38" s="4" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:7">
       <c r="A39" s="4">
         <v>2</v>
       </c>
@@ -5124,13 +5138,13 @@
         <v>18</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="D39" s="4" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:7">
       <c r="A40" s="4">
         <v>2</v>
       </c>
@@ -5138,13 +5152,13 @@
         <v>19</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>693</v>
+        <v>691</v>
       </c>
       <c r="D40" s="4" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:7">
       <c r="A41" s="4">
         <v>2</v>
       </c>
@@ -5152,13 +5166,13 @@
         <v>20</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>694</v>
+        <v>692</v>
       </c>
       <c r="D41" s="4" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:7">
       <c r="A42">
         <v>3</v>
       </c>
@@ -5181,7 +5195,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:7">
       <c r="A43">
         <v>3</v>
       </c>
@@ -5204,7 +5218,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:7">
       <c r="A44">
         <v>3</v>
       </c>
@@ -5227,7 +5241,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:7">
       <c r="A45">
         <v>3</v>
       </c>
@@ -5250,7 +5264,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:7">
       <c r="A46">
         <v>3</v>
       </c>
@@ -5270,7 +5284,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:7">
       <c r="A47">
         <v>3</v>
       </c>
@@ -5293,7 +5307,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:7">
       <c r="A48">
         <v>3</v>
       </c>
@@ -5316,7 +5330,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:7">
       <c r="A49">
         <v>3</v>
       </c>
@@ -5339,7 +5353,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:7">
       <c r="A50">
         <v>3</v>
       </c>
@@ -5362,7 +5376,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:7">
       <c r="A51">
         <v>3</v>
       </c>
@@ -5385,7 +5399,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:7">
       <c r="A52">
         <v>3</v>
       </c>
@@ -5408,7 +5422,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:7">
       <c r="A53">
         <v>3</v>
       </c>
@@ -5422,7 +5436,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:7">
       <c r="A54">
         <v>3</v>
       </c>
@@ -5436,7 +5450,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:7">
       <c r="A55">
         <v>3</v>
       </c>
@@ -5450,7 +5464,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:7">
       <c r="A56">
         <v>3</v>
       </c>
@@ -5464,7 +5478,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:7">
       <c r="A57" s="4">
         <v>3</v>
       </c>
@@ -5472,13 +5486,13 @@
         <v>16</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>695</v>
+        <v>693</v>
       </c>
       <c r="D57" s="4" t="s">
         <v>348</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:7">
       <c r="A58" s="4">
         <v>3</v>
       </c>
@@ -5486,13 +5500,13 @@
         <v>17</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>696</v>
+        <v>694</v>
       </c>
       <c r="D58" s="4" t="s">
         <v>348</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:7">
       <c r="A59" s="4">
         <v>3</v>
       </c>
@@ -5500,13 +5514,13 @@
         <v>18</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>697</v>
+        <v>695</v>
       </c>
       <c r="D59" s="4" t="s">
         <v>348</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:7">
       <c r="A60" s="4">
         <v>3</v>
       </c>
@@ -5514,13 +5528,13 @@
         <v>19</v>
       </c>
       <c r="C60" s="4" t="s">
-        <v>698</v>
+        <v>696</v>
       </c>
       <c r="D60" s="4" t="s">
         <v>348</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:7">
       <c r="A61" s="4">
         <v>3</v>
       </c>
@@ -5528,13 +5542,13 @@
         <v>20</v>
       </c>
       <c r="C61" s="4" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="D61" s="4" t="s">
         <v>348</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:7">
       <c r="A62">
         <v>4</v>
       </c>
@@ -5557,7 +5571,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:7">
       <c r="A63">
         <v>4</v>
       </c>
@@ -5580,7 +5594,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:7">
       <c r="A64">
         <v>4</v>
       </c>
@@ -5603,7 +5617,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:7">
       <c r="A65">
         <v>4</v>
       </c>
@@ -5626,7 +5640,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:7">
       <c r="A66">
         <v>4</v>
       </c>
@@ -5649,7 +5663,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:7">
       <c r="A67">
         <v>4</v>
       </c>
@@ -5669,7 +5683,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:7">
       <c r="A68">
         <v>4</v>
       </c>
@@ -5692,7 +5706,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:7">
       <c r="A69">
         <v>4</v>
       </c>
@@ -5715,7 +5729,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:7">
       <c r="A70">
         <v>4</v>
       </c>
@@ -5738,7 +5752,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:7">
       <c r="A71">
         <v>4</v>
       </c>
@@ -5761,7 +5775,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:7">
       <c r="A72">
         <v>4</v>
       </c>
@@ -5784,7 +5798,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:7">
       <c r="A73">
         <v>4</v>
       </c>
@@ -5798,7 +5812,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:7">
       <c r="A74">
         <v>4</v>
       </c>
@@ -5812,7 +5826,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:7">
       <c r="A75">
         <v>4</v>
       </c>
@@ -5826,7 +5840,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:7">
       <c r="A76">
         <v>4</v>
       </c>
@@ -5840,7 +5854,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:7">
       <c r="A77" s="4">
         <v>4</v>
       </c>
@@ -5848,13 +5862,13 @@
         <v>16</v>
       </c>
       <c r="C77" s="4" t="s">
-        <v>700</v>
+        <v>698</v>
       </c>
       <c r="D77" s="4" t="s">
         <v>389</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:7">
       <c r="A78" s="4">
         <v>4</v>
       </c>
@@ -5862,13 +5876,13 @@
         <v>17</v>
       </c>
       <c r="C78" s="4" t="s">
-        <v>701</v>
+        <v>699</v>
       </c>
       <c r="D78" s="4" t="s">
         <v>389</v>
       </c>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:7">
       <c r="A79" s="4">
         <v>4</v>
       </c>
@@ -5876,13 +5890,13 @@
         <v>18</v>
       </c>
       <c r="C79" s="4" t="s">
-        <v>702</v>
+        <v>700</v>
       </c>
       <c r="D79" s="4" t="s">
         <v>389</v>
       </c>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:7">
       <c r="A80" s="4">
         <v>4</v>
       </c>
@@ -5890,13 +5904,13 @@
         <v>19</v>
       </c>
       <c r="C80" s="4" t="s">
-        <v>703</v>
+        <v>701</v>
       </c>
       <c r="D80" s="4" t="s">
         <v>389</v>
       </c>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:7">
       <c r="A81" s="4">
         <v>4</v>
       </c>
@@ -5904,13 +5918,13 @@
         <v>20</v>
       </c>
       <c r="C81" s="4" t="s">
-        <v>704</v>
+        <v>702</v>
       </c>
       <c r="D81" s="4" t="s">
         <v>389</v>
       </c>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:7">
       <c r="A82">
         <v>5</v>
       </c>
@@ -5933,7 +5947,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:7">
       <c r="A83">
         <v>5</v>
       </c>
@@ -5956,7 +5970,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:7">
       <c r="A84">
         <v>5</v>
       </c>
@@ -5979,7 +5993,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:7">
       <c r="A85">
         <v>5</v>
       </c>
@@ -6002,7 +6016,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:7">
       <c r="A86">
         <v>5</v>
       </c>
@@ -6025,7 +6039,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:7">
       <c r="A87">
         <v>5</v>
       </c>
@@ -6048,7 +6062,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:7">
       <c r="A88">
         <v>5</v>
       </c>
@@ -6071,7 +6085,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:7">
       <c r="A89">
         <v>5</v>
       </c>
@@ -6094,7 +6108,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:7">
       <c r="A90">
         <v>5</v>
       </c>
@@ -6117,7 +6131,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:7">
       <c r="A91">
         <v>5</v>
       </c>
@@ -6140,7 +6154,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:7">
       <c r="A92">
         <v>5</v>
       </c>
@@ -6163,7 +6177,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:7">
       <c r="A93">
         <v>5</v>
       </c>
@@ -6183,7 +6197,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:7">
       <c r="A94">
         <v>5</v>
       </c>
@@ -6197,7 +6211,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:7">
       <c r="A95">
         <v>5</v>
       </c>
@@ -6211,7 +6225,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:7">
       <c r="A96">
         <v>5</v>
       </c>
@@ -6225,7 +6239,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:7">
       <c r="A97" s="4">
         <v>5</v>
       </c>
@@ -6233,13 +6247,13 @@
         <v>16</v>
       </c>
       <c r="C97" s="4" t="s">
-        <v>705</v>
+        <v>703</v>
       </c>
       <c r="D97" s="4" t="s">
         <v>428</v>
       </c>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:7">
       <c r="A98" s="4">
         <v>5</v>
       </c>
@@ -6247,13 +6261,13 @@
         <v>17</v>
       </c>
       <c r="C98" s="4" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="D98" s="4" t="s">
         <v>428</v>
       </c>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:7">
       <c r="A99" s="4">
         <v>5</v>
       </c>
@@ -6261,13 +6275,13 @@
         <v>18</v>
       </c>
       <c r="C99" s="4" t="s">
-        <v>707</v>
+        <v>705</v>
       </c>
       <c r="D99" s="4" t="s">
         <v>428</v>
       </c>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:7">
       <c r="A100" s="4">
         <v>5</v>
       </c>
@@ -6275,13 +6289,13 @@
         <v>19</v>
       </c>
       <c r="C100" s="4" t="s">
-        <v>708</v>
+        <v>706</v>
       </c>
       <c r="D100" s="4" t="s">
         <v>428</v>
       </c>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:7">
       <c r="A101" s="4">
         <v>5</v>
       </c>
@@ -6289,13 +6303,13 @@
         <v>20</v>
       </c>
       <c r="C101" s="4" t="s">
-        <v>709</v>
+        <v>707</v>
       </c>
       <c r="D101" s="4" t="s">
         <v>428</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:7">
       <c r="A102">
         <v>6</v>
       </c>
@@ -6318,7 +6332,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:7">
       <c r="A103">
         <v>6</v>
       </c>
@@ -6341,7 +6355,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:7">
       <c r="A104">
         <v>6</v>
       </c>
@@ -6364,7 +6378,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:7">
       <c r="A105">
         <v>6</v>
       </c>
@@ -6387,7 +6401,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:7">
       <c r="A106">
         <v>6</v>
       </c>
@@ -6410,7 +6424,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:7">
       <c r="A107">
         <v>6</v>
       </c>
@@ -6433,7 +6447,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:7">
       <c r="A108">
         <v>6</v>
       </c>
@@ -6456,7 +6470,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:7">
       <c r="A109">
         <v>6</v>
       </c>
@@ -6479,7 +6493,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:7">
       <c r="A110">
         <v>6</v>
       </c>
@@ -6502,7 +6516,7 @@
         <v>495</v>
       </c>
     </row>
-    <row r="111" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:7" s="2" customFormat="1">
       <c r="A111">
         <v>6</v>
       </c>
@@ -6525,7 +6539,7 @@
         <v>498</v>
       </c>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:7">
       <c r="A112">
         <v>6</v>
       </c>
@@ -6548,7 +6562,7 @@
         <v>501</v>
       </c>
     </row>
-    <row r="113" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:7">
       <c r="A113">
         <v>6</v>
       </c>
@@ -6571,7 +6585,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="114" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:7">
       <c r="A114">
         <v>6</v>
       </c>
@@ -6594,7 +6608,7 @@
         <v>506</v>
       </c>
     </row>
-    <row r="115" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:7">
       <c r="A115">
         <v>6</v>
       </c>
@@ -6608,7 +6622,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="116" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:7">
       <c r="A116">
         <v>6</v>
       </c>
@@ -6622,7 +6636,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="117" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:7">
       <c r="A117" s="4">
         <v>6</v>
       </c>
@@ -6630,13 +6644,13 @@
         <v>16</v>
       </c>
       <c r="C117" s="4" t="s">
-        <v>710</v>
+        <v>708</v>
       </c>
       <c r="D117" s="4" t="s">
         <v>468</v>
       </c>
     </row>
-    <row r="118" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:7">
       <c r="A118" s="4">
         <v>6</v>
       </c>
@@ -6644,13 +6658,13 @@
         <v>17</v>
       </c>
       <c r="C118" s="4" t="s">
-        <v>711</v>
+        <v>709</v>
       </c>
       <c r="D118" s="4" t="s">
         <v>468</v>
       </c>
     </row>
-    <row r="119" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:7">
       <c r="A119" s="4">
         <v>6</v>
       </c>
@@ -6658,13 +6672,13 @@
         <v>18</v>
       </c>
       <c r="C119" s="4" t="s">
-        <v>712</v>
+        <v>710</v>
       </c>
       <c r="D119" s="4" t="s">
         <v>468</v>
       </c>
     </row>
-    <row r="120" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:7">
       <c r="A120" s="4">
         <v>6</v>
       </c>
@@ -6672,13 +6686,13 @@
         <v>19</v>
       </c>
       <c r="C120" s="4" t="s">
-        <v>713</v>
+        <v>711</v>
       </c>
       <c r="D120" s="4" t="s">
         <v>468</v>
       </c>
     </row>
-    <row r="121" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:7">
       <c r="A121" s="4">
         <v>6</v>
       </c>
@@ -6686,13 +6700,13 @@
         <v>20</v>
       </c>
       <c r="C121" s="4" t="s">
-        <v>714</v>
+        <v>712</v>
       </c>
       <c r="D121" s="4" t="s">
         <v>468</v>
       </c>
     </row>
-    <row r="122" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:7">
       <c r="A122">
         <v>7</v>
       </c>
@@ -6715,7 +6729,7 @@
         <v>511</v>
       </c>
     </row>
-    <row r="123" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:7">
       <c r="A123">
         <v>7</v>
       </c>
@@ -6738,7 +6752,7 @@
         <v>514</v>
       </c>
     </row>
-    <row r="124" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:7">
       <c r="A124">
         <v>7</v>
       </c>
@@ -6761,7 +6775,7 @@
         <v>518</v>
       </c>
     </row>
-    <row r="125" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:7">
       <c r="A125">
         <v>7</v>
       </c>
@@ -6784,7 +6798,7 @@
         <v>522</v>
       </c>
     </row>
-    <row r="126" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:7">
       <c r="A126">
         <v>7</v>
       </c>
@@ -6807,7 +6821,7 @@
         <v>525</v>
       </c>
     </row>
-    <row r="127" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:7">
       <c r="A127">
         <v>7</v>
       </c>
@@ -6830,7 +6844,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="128" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:7">
       <c r="A128">
         <v>7</v>
       </c>
@@ -6853,7 +6867,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="129" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:7">
       <c r="A129">
         <v>7</v>
       </c>
@@ -6876,7 +6890,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="130" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:7">
       <c r="A130">
         <v>7</v>
       </c>
@@ -6899,7 +6913,7 @@
         <v>538</v>
       </c>
     </row>
-    <row r="131" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:7">
       <c r="A131">
         <v>7</v>
       </c>
@@ -6922,7 +6936,7 @@
         <v>541</v>
       </c>
     </row>
-    <row r="132" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:7">
       <c r="A132">
         <v>7</v>
       </c>
@@ -6945,7 +6959,7 @@
         <v>544</v>
       </c>
     </row>
-    <row r="133" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:7">
       <c r="A133">
         <v>7</v>
       </c>
@@ -6968,7 +6982,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="134" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:7">
       <c r="A134">
         <v>7</v>
       </c>
@@ -6991,7 +7005,7 @@
         <v>550</v>
       </c>
     </row>
-    <row r="135" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:7">
       <c r="A135">
         <v>7</v>
       </c>
@@ -7005,7 +7019,7 @@
         <v>510</v>
       </c>
     </row>
-    <row r="136" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:7">
       <c r="A136">
         <v>7</v>
       </c>
@@ -7019,7 +7033,7 @@
         <v>510</v>
       </c>
     </row>
-    <row r="137" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:7">
       <c r="A137" s="4">
         <v>7</v>
       </c>
@@ -7027,13 +7041,13 @@
         <v>16</v>
       </c>
       <c r="C137" s="4" t="s">
-        <v>715</v>
+        <v>713</v>
       </c>
       <c r="D137" s="4" t="s">
         <v>510</v>
       </c>
     </row>
-    <row r="138" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:7">
       <c r="A138" s="4">
         <v>7</v>
       </c>
@@ -7041,13 +7055,13 @@
         <v>17</v>
       </c>
       <c r="C138" s="4" t="s">
-        <v>716</v>
+        <v>714</v>
       </c>
       <c r="D138" s="4" t="s">
         <v>510</v>
       </c>
     </row>
-    <row r="139" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:7">
       <c r="A139" s="4">
         <v>7</v>
       </c>
@@ -7055,13 +7069,13 @@
         <v>18</v>
       </c>
       <c r="C139" s="4" t="s">
-        <v>717</v>
+        <v>715</v>
       </c>
       <c r="D139" s="4" t="s">
         <v>510</v>
       </c>
     </row>
-    <row r="140" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:7">
       <c r="A140" s="4">
         <v>7</v>
       </c>
@@ -7069,13 +7083,13 @@
         <v>19</v>
       </c>
       <c r="C140" s="4" t="s">
-        <v>718</v>
+        <v>716</v>
       </c>
       <c r="D140" s="4" t="s">
         <v>510</v>
       </c>
     </row>
-    <row r="141" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:7">
       <c r="A141" s="4">
         <v>7</v>
       </c>
@@ -7083,13 +7097,13 @@
         <v>20</v>
       </c>
       <c r="C141" s="4" t="s">
-        <v>719</v>
+        <v>717</v>
       </c>
       <c r="D141" s="4" t="s">
         <v>510</v>
       </c>
     </row>
-    <row r="142" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:7">
       <c r="A142">
         <v>8</v>
       </c>
@@ -7112,7 +7126,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="143" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:7">
       <c r="A143">
         <v>8</v>
       </c>
@@ -7135,7 +7149,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="144" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:7">
       <c r="A144">
         <v>8</v>
       </c>
@@ -7143,7 +7157,7 @@
         <v>3</v>
       </c>
       <c r="C144" t="s">
-        <v>677</v>
+        <v>675</v>
       </c>
       <c r="D144" t="s">
         <v>554</v>
@@ -7158,7 +7172,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="145" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:7">
       <c r="A145">
         <v>8</v>
       </c>
@@ -7166,7 +7180,7 @@
         <v>4</v>
       </c>
       <c r="C145" t="s">
-        <v>669</v>
+        <v>667</v>
       </c>
       <c r="D145" t="s">
         <v>554</v>
@@ -7181,7 +7195,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="146" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:7">
       <c r="A146" s="2">
         <v>8</v>
       </c>
@@ -7195,7 +7209,7 @@
         <v>554</v>
       </c>
       <c r="E146" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="F146" t="s">
         <v>305</v>
@@ -7204,7 +7218,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="147" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:7">
       <c r="A147">
         <v>8</v>
       </c>
@@ -7212,13 +7226,13 @@
         <v>6</v>
       </c>
       <c r="C147" s="1" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="D147" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="148" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:7">
       <c r="A148">
         <v>8</v>
       </c>
@@ -7226,13 +7240,13 @@
         <v>7</v>
       </c>
       <c r="C148" s="1" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="D148" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="149" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:7">
       <c r="A149">
         <v>8</v>
       </c>
@@ -7240,16 +7254,13 @@
         <v>8</v>
       </c>
       <c r="C149" s="1" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
       <c r="D149" t="s">
         <v>554</v>
       </c>
-      <c r="E149" t="s">
-        <v>316</v>
-      </c>
-    </row>
-    <row r="150" spans="1:7" x14ac:dyDescent="0.2">
+    </row>
+    <row r="150" spans="1:7">
       <c r="A150">
         <v>8</v>
       </c>
@@ -7257,16 +7268,16 @@
         <v>9</v>
       </c>
       <c r="C150" s="1" t="s">
-        <v>649</v>
+        <v>743</v>
       </c>
       <c r="D150" t="s">
         <v>554</v>
       </c>
       <c r="E150" t="s">
-        <v>316</v>
-      </c>
-    </row>
-    <row r="151" spans="1:7" x14ac:dyDescent="0.2">
+        <v>745</v>
+      </c>
+    </row>
+    <row r="151" spans="1:7">
       <c r="A151">
         <v>8</v>
       </c>
@@ -7274,16 +7285,16 @@
         <v>10</v>
       </c>
       <c r="C151" s="1" t="s">
-        <v>650</v>
+        <v>744</v>
       </c>
       <c r="D151" t="s">
         <v>554</v>
       </c>
       <c r="E151" t="s">
-        <v>659</v>
-      </c>
-    </row>
-    <row r="152" spans="1:7" x14ac:dyDescent="0.2">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="152" spans="1:7">
       <c r="A152">
         <v>8</v>
       </c>
@@ -7291,13 +7302,16 @@
         <v>11</v>
       </c>
       <c r="C152" s="1" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="D152" t="s">
         <v>554</v>
       </c>
-    </row>
-    <row r="153" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="E152" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="153" spans="1:7">
       <c r="A153">
         <v>8</v>
       </c>
@@ -7305,13 +7319,16 @@
         <v>12</v>
       </c>
       <c r="C153" s="1" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="D153" t="s">
         <v>554</v>
       </c>
-    </row>
-    <row r="154" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="E153" t="s">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="154" spans="1:7">
       <c r="A154">
         <v>8</v>
       </c>
@@ -7319,13 +7336,13 @@
         <v>13</v>
       </c>
       <c r="C154" s="1" t="s">
-        <v>653</v>
+        <v>651</v>
       </c>
       <c r="D154" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="155" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:7">
       <c r="A155">
         <v>8</v>
       </c>
@@ -7333,13 +7350,13 @@
         <v>14</v>
       </c>
       <c r="C155" s="1" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="D155" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="156" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:7">
       <c r="A156">
         <v>8</v>
       </c>
@@ -7353,7 +7370,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="157" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:7">
       <c r="A157" s="4">
         <v>8</v>
       </c>
@@ -7361,13 +7378,13 @@
         <v>16</v>
       </c>
       <c r="C157" s="4" t="s">
-        <v>720</v>
+        <v>718</v>
       </c>
       <c r="D157" s="4" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="158" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:7">
       <c r="A158" s="4">
         <v>8</v>
       </c>
@@ -7375,13 +7392,13 @@
         <v>17</v>
       </c>
       <c r="C158" s="4" t="s">
-        <v>721</v>
+        <v>719</v>
       </c>
       <c r="D158" s="4" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="159" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:7">
       <c r="A159" s="4">
         <v>8</v>
       </c>
@@ -7389,13 +7406,13 @@
         <v>18</v>
       </c>
       <c r="C159" s="4" t="s">
-        <v>722</v>
+        <v>720</v>
       </c>
       <c r="D159" s="4" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="160" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:7">
       <c r="A160" s="4">
         <v>8</v>
       </c>
@@ -7403,13 +7420,13 @@
         <v>19</v>
       </c>
       <c r="C160" s="4" t="s">
-        <v>723</v>
+        <v>721</v>
       </c>
       <c r="D160" s="4" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="161" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:7">
       <c r="A161" s="4">
         <v>8</v>
       </c>
@@ -7417,13 +7434,13 @@
         <v>20</v>
       </c>
       <c r="C161" s="4" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="D161" s="4" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="162" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:7">
       <c r="A162">
         <v>9</v>
       </c>
@@ -7446,7 +7463,7 @@
         <v>570</v>
       </c>
     </row>
-    <row r="163" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:7">
       <c r="A163">
         <v>9</v>
       </c>
@@ -7469,7 +7486,7 @@
         <v>573</v>
       </c>
     </row>
-    <row r="164" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:7">
       <c r="A164">
         <v>9</v>
       </c>
@@ -7489,7 +7506,7 @@
         <v>574</v>
       </c>
     </row>
-    <row r="165" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:7">
       <c r="A165">
         <v>9</v>
       </c>
@@ -7509,7 +7526,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="166" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:7">
       <c r="A166">
         <v>9</v>
       </c>
@@ -7532,7 +7549,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="167" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:7">
       <c r="A167">
         <v>9</v>
       </c>
@@ -7546,7 +7563,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="168" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:7">
       <c r="A168">
         <v>9</v>
       </c>
@@ -7560,7 +7577,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="169" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:7">
       <c r="A169">
         <v>9</v>
       </c>
@@ -7574,7 +7591,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="170" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:7">
       <c r="A170">
         <v>9</v>
       </c>
@@ -7588,7 +7605,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="171" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:7">
       <c r="A171">
         <v>9</v>
       </c>
@@ -7602,7 +7619,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="172" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:7">
       <c r="A172">
         <v>9</v>
       </c>
@@ -7616,7 +7633,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="173" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:7">
       <c r="A173">
         <v>9</v>
       </c>
@@ -7630,7 +7647,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="174" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:7">
       <c r="A174">
         <v>9</v>
       </c>
@@ -7644,7 +7661,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="175" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:7">
       <c r="A175">
         <v>9</v>
       </c>
@@ -7658,7 +7675,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="176" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:7">
       <c r="A176">
         <v>9</v>
       </c>
@@ -7672,7 +7689,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="177" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:7">
       <c r="A177" s="4">
         <v>9</v>
       </c>
@@ -7680,13 +7697,13 @@
         <v>16</v>
       </c>
       <c r="C177" s="4" t="s">
-        <v>725</v>
+        <v>723</v>
       </c>
       <c r="D177" s="4" t="s">
         <v>567</v>
       </c>
     </row>
-    <row r="178" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:7">
       <c r="A178" s="4">
         <v>9</v>
       </c>
@@ -7694,13 +7711,13 @@
         <v>17</v>
       </c>
       <c r="C178" s="4" t="s">
-        <v>726</v>
+        <v>724</v>
       </c>
       <c r="D178" s="4" t="s">
         <v>567</v>
       </c>
     </row>
-    <row r="179" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:7">
       <c r="A179" s="4">
         <v>9</v>
       </c>
@@ -7708,13 +7725,13 @@
         <v>18</v>
       </c>
       <c r="C179" s="4" t="s">
-        <v>727</v>
+        <v>725</v>
       </c>
       <c r="D179" s="4" t="s">
         <v>567</v>
       </c>
     </row>
-    <row r="180" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:7">
       <c r="A180" s="4">
         <v>9</v>
       </c>
@@ -7722,13 +7739,13 @@
         <v>19</v>
       </c>
       <c r="C180" s="4" t="s">
-        <v>728</v>
+        <v>726</v>
       </c>
       <c r="D180" s="4" t="s">
         <v>567</v>
       </c>
     </row>
-    <row r="181" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:7">
       <c r="A181" s="4">
         <v>9</v>
       </c>
@@ -7736,13 +7753,13 @@
         <v>20</v>
       </c>
       <c r="C181" s="4" t="s">
-        <v>729</v>
+        <v>727</v>
       </c>
       <c r="D181" s="4" t="s">
         <v>567</v>
       </c>
     </row>
-    <row r="182" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:7">
       <c r="A182">
         <v>10</v>
       </c>
@@ -7765,7 +7782,7 @@
         <v>594</v>
       </c>
     </row>
-    <row r="183" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:7">
       <c r="A183">
         <v>10</v>
       </c>
@@ -7788,7 +7805,7 @@
         <v>597</v>
       </c>
     </row>
-    <row r="184" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:7">
       <c r="A184">
         <v>10</v>
       </c>
@@ -7811,7 +7828,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="185" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:7">
       <c r="A185">
         <v>10</v>
       </c>
@@ -7834,7 +7851,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="186" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:7">
       <c r="A186">
         <v>10</v>
       </c>
@@ -7857,7 +7874,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="187" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:7">
       <c r="A187">
         <v>10</v>
       </c>
@@ -7880,7 +7897,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="188" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:7">
       <c r="A188">
         <v>10</v>
       </c>
@@ -7903,7 +7920,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="189" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:7">
       <c r="A189">
         <v>10</v>
       </c>
@@ -7926,7 +7943,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="190" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:7">
       <c r="A190">
         <v>10</v>
       </c>
@@ -7949,7 +7966,7 @@
         <v>618</v>
       </c>
     </row>
-    <row r="191" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:7">
       <c r="A191">
         <v>10</v>
       </c>
@@ -7972,7 +7989,7 @@
         <v>621</v>
       </c>
     </row>
-    <row r="192" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="192" spans="1:7">
       <c r="A192">
         <v>10</v>
       </c>
@@ -7995,7 +8012,7 @@
         <v>624</v>
       </c>
     </row>
-    <row r="193" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:7">
       <c r="A193">
         <v>10</v>
       </c>
@@ -8018,7 +8035,7 @@
         <v>627</v>
       </c>
     </row>
-    <row r="194" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:7">
       <c r="A194">
         <v>10</v>
       </c>
@@ -8041,7 +8058,7 @@
         <v>630</v>
       </c>
     </row>
-    <row r="195" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="195" spans="1:7">
       <c r="A195">
         <v>10</v>
       </c>
@@ -8064,7 +8081,7 @@
         <v>633</v>
       </c>
     </row>
-    <row r="196" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="196" spans="1:7">
       <c r="A196">
         <v>10</v>
       </c>
@@ -8078,7 +8095,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="197" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="197" spans="1:7">
       <c r="A197" s="4">
         <v>10</v>
       </c>
@@ -8086,13 +8103,13 @@
         <v>16</v>
       </c>
       <c r="C197" s="4" t="s">
-        <v>730</v>
+        <v>728</v>
       </c>
       <c r="D197" s="4" t="s">
         <v>592</v>
       </c>
     </row>
-    <row r="198" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="198" spans="1:7">
       <c r="A198" s="4">
         <v>10</v>
       </c>
@@ -8100,13 +8117,13 @@
         <v>17</v>
       </c>
       <c r="C198" s="4" t="s">
-        <v>731</v>
+        <v>729</v>
       </c>
       <c r="D198" s="4" t="s">
         <v>592</v>
       </c>
     </row>
-    <row r="199" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="199" spans="1:7">
       <c r="A199" s="4">
         <v>10</v>
       </c>
@@ -8114,13 +8131,13 @@
         <v>18</v>
       </c>
       <c r="C199" s="4" t="s">
-        <v>732</v>
+        <v>730</v>
       </c>
       <c r="D199" s="4" t="s">
         <v>592</v>
       </c>
     </row>
-    <row r="200" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="200" spans="1:7">
       <c r="A200" s="4">
         <v>10</v>
       </c>
@@ -8128,13 +8145,13 @@
         <v>19</v>
       </c>
       <c r="C200" s="4" t="s">
-        <v>733</v>
+        <v>731</v>
       </c>
       <c r="D200" s="4" t="s">
         <v>592</v>
       </c>
     </row>
-    <row r="201" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="201" spans="1:7">
       <c r="A201" s="4">
         <v>10</v>
       </c>
@@ -8142,13 +8159,13 @@
         <v>20</v>
       </c>
       <c r="C201" s="4" t="s">
-        <v>734</v>
+        <v>732</v>
       </c>
       <c r="D201" s="4" t="s">
         <v>592</v>
       </c>
     </row>
-    <row r="202" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="202" spans="1:7">
       <c r="A202">
         <v>11</v>
       </c>
@@ -8156,19 +8173,19 @@
         <v>1</v>
       </c>
       <c r="C202" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="D202" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="E202" t="s">
-        <v>665</v>
+        <v>663</v>
       </c>
       <c r="F202" t="s">
         <v>305</v>
       </c>
     </row>
-    <row r="203" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="203" spans="1:7">
       <c r="A203">
         <v>11</v>
       </c>
@@ -8176,19 +8193,19 @@
         <v>2</v>
       </c>
       <c r="C203" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="D203" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="E203" t="s">
-        <v>666</v>
+        <v>664</v>
       </c>
       <c r="F203" t="s">
         <v>391</v>
       </c>
     </row>
-    <row r="204" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="204" spans="1:7">
       <c r="A204">
         <v>11</v>
       </c>
@@ -8196,19 +8213,19 @@
         <v>3</v>
       </c>
       <c r="C204" t="s">
-        <v>663</v>
+        <v>661</v>
       </c>
       <c r="D204" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="E204" t="s">
-        <v>667</v>
+        <v>665</v>
       </c>
       <c r="F204" t="s">
         <v>391</v>
       </c>
     </row>
-    <row r="205" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="205" spans="1:7">
       <c r="A205">
         <v>11</v>
       </c>
@@ -8216,19 +8233,19 @@
         <v>4</v>
       </c>
       <c r="C205" t="s">
-        <v>664</v>
+        <v>662</v>
       </c>
       <c r="D205" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="E205" t="s">
-        <v>668</v>
+        <v>666</v>
       </c>
       <c r="F205" t="s">
         <v>391</v>
       </c>
     </row>
-    <row r="206" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="206" spans="1:7">
       <c r="A206">
         <v>11</v>
       </c>
@@ -8236,19 +8253,19 @@
         <v>5</v>
       </c>
       <c r="C206" t="s">
-        <v>669</v>
+        <v>667</v>
       </c>
       <c r="D206" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="E206" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="F206" t="s">
         <v>305</v>
       </c>
     </row>
-    <row r="207" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="207" spans="1:7">
       <c r="A207">
         <v>11</v>
       </c>
@@ -8256,19 +8273,19 @@
         <v>6</v>
       </c>
       <c r="C207" t="s">
-        <v>670</v>
+        <v>668</v>
       </c>
       <c r="D207" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="E207" t="s">
-        <v>674</v>
+        <v>672</v>
       </c>
       <c r="F207" t="s">
         <v>391</v>
       </c>
     </row>
-    <row r="208" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="208" spans="1:7">
       <c r="A208">
         <v>11</v>
       </c>
@@ -8276,19 +8293,19 @@
         <v>7</v>
       </c>
       <c r="C208" t="s">
-        <v>671</v>
+        <v>669</v>
       </c>
       <c r="D208" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="E208" t="s">
-        <v>675</v>
+        <v>673</v>
       </c>
       <c r="F208" t="s">
         <v>391</v>
       </c>
     </row>
-    <row r="209" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="209" spans="1:6">
       <c r="A209">
         <v>11</v>
       </c>
@@ -8296,19 +8313,19 @@
         <v>8</v>
       </c>
       <c r="C209" t="s">
-        <v>672</v>
+        <v>670</v>
       </c>
       <c r="D209" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="E209" t="s">
-        <v>676</v>
+        <v>674</v>
       </c>
       <c r="F209" t="s">
         <v>391</v>
       </c>
     </row>
-    <row r="210" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:6">
       <c r="A210">
         <v>11</v>
       </c>
@@ -8316,19 +8333,19 @@
         <v>9</v>
       </c>
       <c r="C210" t="s">
-        <v>677</v>
+        <v>675</v>
       </c>
       <c r="D210" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="E210" t="s">
-        <v>681</v>
+        <v>679</v>
       </c>
       <c r="F210" t="s">
         <v>305</v>
       </c>
     </row>
-    <row r="211" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="211" spans="1:6">
       <c r="A211">
         <v>11</v>
       </c>
@@ -8336,19 +8353,19 @@
         <v>10</v>
       </c>
       <c r="C211" t="s">
-        <v>678</v>
+        <v>676</v>
       </c>
       <c r="D211" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="E211" t="s">
-        <v>682</v>
+        <v>680</v>
       </c>
       <c r="F211" t="s">
         <v>391</v>
       </c>
     </row>
-    <row r="212" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="212" spans="1:6">
       <c r="A212">
         <v>11</v>
       </c>
@@ -8356,19 +8373,19 @@
         <v>11</v>
       </c>
       <c r="C212" t="s">
-        <v>679</v>
+        <v>677</v>
       </c>
       <c r="D212" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="E212" t="s">
-        <v>683</v>
+        <v>681</v>
       </c>
       <c r="F212" t="s">
         <v>391</v>
       </c>
     </row>
-    <row r="213" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="213" spans="1:6">
       <c r="A213">
         <v>11</v>
       </c>
@@ -8376,19 +8393,19 @@
         <v>12</v>
       </c>
       <c r="C213" t="s">
-        <v>680</v>
+        <v>678</v>
       </c>
       <c r="D213" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="E213" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="F213" t="s">
         <v>391</v>
       </c>
     </row>
-    <row r="214" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="214" spans="1:6">
       <c r="A214">
         <v>11</v>
       </c>
@@ -8396,13 +8413,13 @@
         <v>13</v>
       </c>
       <c r="C214" t="s">
-        <v>741</v>
+        <v>739</v>
       </c>
       <c r="D214" t="s">
-        <v>660</v>
-      </c>
-    </row>
-    <row r="215" spans="1:6" x14ac:dyDescent="0.2">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="215" spans="1:6">
       <c r="A215">
         <v>11</v>
       </c>
@@ -8410,13 +8427,13 @@
         <v>14</v>
       </c>
       <c r="C215" t="s">
-        <v>742</v>
+        <v>740</v>
       </c>
       <c r="D215" t="s">
-        <v>660</v>
-      </c>
-    </row>
-    <row r="216" spans="1:6" x14ac:dyDescent="0.2">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="216" spans="1:6">
       <c r="A216">
         <v>11</v>
       </c>
@@ -8424,13 +8441,13 @@
         <v>15</v>
       </c>
       <c r="C216" t="s">
-        <v>743</v>
+        <v>741</v>
       </c>
       <c r="D216" t="s">
-        <v>660</v>
-      </c>
-    </row>
-    <row r="217" spans="1:6" x14ac:dyDescent="0.2">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="217" spans="1:6">
       <c r="A217" s="4">
         <v>11</v>
       </c>
@@ -8438,13 +8455,13 @@
         <v>16</v>
       </c>
       <c r="C217" t="s">
-        <v>744</v>
+        <v>742</v>
       </c>
       <c r="D217" s="4" t="s">
-        <v>660</v>
-      </c>
-    </row>
-    <row r="218" spans="1:6" x14ac:dyDescent="0.2">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="218" spans="1:6">
       <c r="A218" s="4">
         <v>11</v>
       </c>
@@ -8452,13 +8469,13 @@
         <v>17</v>
       </c>
       <c r="C218" s="4" t="s">
-        <v>736</v>
+        <v>734</v>
       </c>
       <c r="D218" s="4" t="s">
-        <v>660</v>
-      </c>
-    </row>
-    <row r="219" spans="1:6" x14ac:dyDescent="0.2">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="219" spans="1:6">
       <c r="A219" s="4">
         <v>11</v>
       </c>
@@ -8466,13 +8483,13 @@
         <v>18</v>
       </c>
       <c r="C219" s="4" t="s">
-        <v>737</v>
+        <v>735</v>
       </c>
       <c r="D219" s="4" t="s">
-        <v>660</v>
-      </c>
-    </row>
-    <row r="220" spans="1:6" x14ac:dyDescent="0.2">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="220" spans="1:6">
       <c r="A220" s="4">
         <v>11</v>
       </c>
@@ -8480,13 +8497,13 @@
         <v>19</v>
       </c>
       <c r="C220" s="4" t="s">
-        <v>738</v>
+        <v>736</v>
       </c>
       <c r="D220" s="4" t="s">
-        <v>660</v>
-      </c>
-    </row>
-    <row r="221" spans="1:6" x14ac:dyDescent="0.2">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="221" spans="1:6">
       <c r="A221" s="4">
         <v>11</v>
       </c>
@@ -8494,10 +8511,10 @@
         <v>20</v>
       </c>
       <c r="C221" s="4" t="s">
-        <v>739</v>
+        <v>737</v>
       </c>
       <c r="D221" s="4" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
     </row>
   </sheetData>
@@ -8508,15 +8525,19 @@
   </autoFilter>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;"Aptos"&amp;12&amp;KFF0000 OFFICIAL&amp;1#_x000D_</oddHeader>
+    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Aptos"&amp;12&amp;KFF0000 OFFICIAL</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2C146B8-AED1-D84E-BB27-CA28C1D97E3C}">
   <dimension ref="A1:E58"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5">
       <c r="A1" s="3"/>
       <c r="B1" s="3" t="s">
         <v>256</v>
@@ -8531,14 +8552,14 @@
         <v>259</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5">
       <c r="A2" s="3"/>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5">
       <c r="A3" s="3">
         <v>1</v>
       </c>
@@ -8549,13 +8570,13 @@
         <v>16</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>685</v>
+        <v>683</v>
       </c>
       <c r="E3" s="4" t="s">
         <v>261</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5">
       <c r="A4" s="3">
         <v>2</v>
       </c>
@@ -8566,13 +8587,13 @@
         <v>17</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>261</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5">
       <c r="A5" s="3">
         <v>3</v>
       </c>
@@ -8583,13 +8604,13 @@
         <v>18</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>687</v>
+        <v>685</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>261</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5">
       <c r="A6" s="3">
         <v>4</v>
       </c>
@@ -8600,13 +8621,13 @@
         <v>19</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>261</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5">
       <c r="A7" s="3">
         <v>5</v>
       </c>
@@ -8617,13 +8638,13 @@
         <v>20</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>689</v>
+        <v>687</v>
       </c>
       <c r="E7" s="4" t="s">
         <v>261</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5">
       <c r="A8" s="3">
         <v>6</v>
       </c>
@@ -8634,13 +8655,13 @@
         <v>16</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>690</v>
+        <v>688</v>
       </c>
       <c r="E8" s="4" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5">
       <c r="A9" s="3">
         <v>7</v>
       </c>
@@ -8651,13 +8672,13 @@
         <v>17</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>691</v>
+        <v>689</v>
       </c>
       <c r="E9" s="4" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5">
       <c r="A10" s="3">
         <v>8</v>
       </c>
@@ -8668,13 +8689,13 @@
         <v>18</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="E10" s="4" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:5">
       <c r="A11" s="3">
         <v>9</v>
       </c>
@@ -8685,13 +8706,13 @@
         <v>19</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>693</v>
+        <v>691</v>
       </c>
       <c r="E11" s="4" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:5">
       <c r="A12" s="3">
         <v>10</v>
       </c>
@@ -8702,13 +8723,13 @@
         <v>20</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>694</v>
+        <v>692</v>
       </c>
       <c r="E12" s="4" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:5">
       <c r="A13" s="3">
         <v>11</v>
       </c>
@@ -8719,13 +8740,13 @@
         <v>16</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>695</v>
+        <v>693</v>
       </c>
       <c r="E13" s="4" t="s">
         <v>348</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:5">
       <c r="A14" s="3">
         <v>12</v>
       </c>
@@ -8736,13 +8757,13 @@
         <v>17</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>696</v>
+        <v>694</v>
       </c>
       <c r="E14" s="4" t="s">
         <v>348</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:5">
       <c r="A15" s="3">
         <v>13</v>
       </c>
@@ -8753,13 +8774,13 @@
         <v>18</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>697</v>
+        <v>695</v>
       </c>
       <c r="E15" s="4" t="s">
         <v>348</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:5">
       <c r="A16" s="3">
         <v>14</v>
       </c>
@@ -8770,13 +8791,13 @@
         <v>19</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>698</v>
+        <v>696</v>
       </c>
       <c r="E16" s="4" t="s">
         <v>348</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:5">
       <c r="A17" s="3">
         <v>15</v>
       </c>
@@ -8787,13 +8808,13 @@
         <v>20</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="E17" s="4" t="s">
         <v>348</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:5">
       <c r="A18" s="3">
         <v>16</v>
       </c>
@@ -8804,13 +8825,13 @@
         <v>16</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>700</v>
+        <v>698</v>
       </c>
       <c r="E18" s="4" t="s">
         <v>389</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:5">
       <c r="A19" s="3">
         <v>17</v>
       </c>
@@ -8821,13 +8842,13 @@
         <v>17</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>701</v>
+        <v>699</v>
       </c>
       <c r="E19" s="4" t="s">
         <v>389</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:5">
       <c r="A20" s="3">
         <v>18</v>
       </c>
@@ -8838,13 +8859,13 @@
         <v>18</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>702</v>
+        <v>700</v>
       </c>
       <c r="E20" s="4" t="s">
         <v>389</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:5">
       <c r="A21" s="3">
         <v>19</v>
       </c>
@@ -8855,13 +8876,13 @@
         <v>19</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>703</v>
+        <v>701</v>
       </c>
       <c r="E21" s="4" t="s">
         <v>389</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:5">
       <c r="A22" s="3">
         <v>20</v>
       </c>
@@ -8872,13 +8893,13 @@
         <v>20</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>704</v>
+        <v>702</v>
       </c>
       <c r="E22" s="4" t="s">
         <v>389</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:5">
       <c r="A23" s="3">
         <v>21</v>
       </c>
@@ -8889,13 +8910,13 @@
         <v>16</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>705</v>
+        <v>703</v>
       </c>
       <c r="E23" s="4" t="s">
         <v>428</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:5">
       <c r="A24" s="3">
         <v>22</v>
       </c>
@@ -8906,13 +8927,13 @@
         <v>17</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="E24" s="4" t="s">
         <v>428</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:5">
       <c r="A25" s="3">
         <v>23</v>
       </c>
@@ -8923,13 +8944,13 @@
         <v>18</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>707</v>
+        <v>705</v>
       </c>
       <c r="E25" s="4" t="s">
         <v>428</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:5">
       <c r="A26" s="3">
         <v>24</v>
       </c>
@@ -8940,13 +8961,13 @@
         <v>19</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>708</v>
+        <v>706</v>
       </c>
       <c r="E26" s="4" t="s">
         <v>428</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:5">
       <c r="A27" s="3">
         <v>25</v>
       </c>
@@ -8957,13 +8978,13 @@
         <v>20</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>709</v>
+        <v>707</v>
       </c>
       <c r="E27" s="4" t="s">
         <v>428</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:5">
       <c r="A28" s="3">
         <v>26</v>
       </c>
@@ -8974,13 +8995,13 @@
         <v>16</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>710</v>
+        <v>708</v>
       </c>
       <c r="E28" s="4" t="s">
         <v>468</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:5">
       <c r="A29" s="3">
         <v>27</v>
       </c>
@@ -8991,13 +9012,13 @@
         <v>17</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>711</v>
+        <v>709</v>
       </c>
       <c r="E29" s="4" t="s">
         <v>468</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:5">
       <c r="A30" s="3">
         <v>28</v>
       </c>
@@ -9008,13 +9029,13 @@
         <v>18</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>712</v>
+        <v>710</v>
       </c>
       <c r="E30" s="4" t="s">
         <v>468</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:5">
       <c r="A31" s="3">
         <v>29</v>
       </c>
@@ -9025,13 +9046,13 @@
         <v>19</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>713</v>
+        <v>711</v>
       </c>
       <c r="E31" s="4" t="s">
         <v>468</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:5">
       <c r="A32" s="3">
         <v>30</v>
       </c>
@@ -9042,13 +9063,13 @@
         <v>20</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>714</v>
+        <v>712</v>
       </c>
       <c r="E32" s="4" t="s">
         <v>468</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:5">
       <c r="A33" s="3">
         <v>31</v>
       </c>
@@ -9059,13 +9080,13 @@
         <v>16</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>715</v>
+        <v>713</v>
       </c>
       <c r="E33" s="4" t="s">
         <v>510</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:5">
       <c r="A34" s="3">
         <v>32</v>
       </c>
@@ -9076,13 +9097,13 @@
         <v>17</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>716</v>
+        <v>714</v>
       </c>
       <c r="E34" s="4" t="s">
         <v>510</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:5">
       <c r="A35" s="3">
         <v>33</v>
       </c>
@@ -9093,13 +9114,13 @@
         <v>18</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>717</v>
+        <v>715</v>
       </c>
       <c r="E35" s="4" t="s">
         <v>510</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:5">
       <c r="A36" s="3">
         <v>34</v>
       </c>
@@ -9110,13 +9131,13 @@
         <v>19</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>718</v>
+        <v>716</v>
       </c>
       <c r="E36" s="4" t="s">
         <v>510</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:5">
       <c r="A37" s="3">
         <v>35</v>
       </c>
@@ -9127,13 +9148,13 @@
         <v>20</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>719</v>
+        <v>717</v>
       </c>
       <c r="E37" s="4" t="s">
         <v>510</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:5">
       <c r="A38" s="3">
         <v>36</v>
       </c>
@@ -9144,13 +9165,13 @@
         <v>16</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>720</v>
+        <v>718</v>
       </c>
       <c r="E38" s="4" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:5">
       <c r="A39" s="3">
         <v>37</v>
       </c>
@@ -9161,13 +9182,13 @@
         <v>17</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>721</v>
+        <v>719</v>
       </c>
       <c r="E39" s="4" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:5">
       <c r="A40" s="3">
         <v>38</v>
       </c>
@@ -9178,13 +9199,13 @@
         <v>18</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>722</v>
+        <v>720</v>
       </c>
       <c r="E40" s="4" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:5">
       <c r="A41" s="3">
         <v>39</v>
       </c>
@@ -9195,13 +9216,13 @@
         <v>19</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>723</v>
+        <v>721</v>
       </c>
       <c r="E41" s="4" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:5">
       <c r="A42" s="3">
         <v>40</v>
       </c>
@@ -9212,13 +9233,13 @@
         <v>20</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="E42" s="4" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:5">
       <c r="A43" s="3">
         <v>41</v>
       </c>
@@ -9229,13 +9250,13 @@
         <v>16</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>725</v>
+        <v>723</v>
       </c>
       <c r="E43" s="4" t="s">
         <v>567</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:5">
       <c r="A44" s="3">
         <v>42</v>
       </c>
@@ -9246,13 +9267,13 @@
         <v>17</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>726</v>
+        <v>724</v>
       </c>
       <c r="E44" s="4" t="s">
         <v>567</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:5">
       <c r="A45" s="3">
         <v>43</v>
       </c>
@@ -9263,13 +9284,13 @@
         <v>18</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>727</v>
+        <v>725</v>
       </c>
       <c r="E45" s="4" t="s">
         <v>567</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:5">
       <c r="A46" s="3">
         <v>44</v>
       </c>
@@ -9280,13 +9301,13 @@
         <v>19</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>728</v>
+        <v>726</v>
       </c>
       <c r="E46" s="4" t="s">
         <v>567</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:5">
       <c r="A47" s="3">
         <v>45</v>
       </c>
@@ -9297,13 +9318,13 @@
         <v>20</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>729</v>
+        <v>727</v>
       </c>
       <c r="E47" s="4" t="s">
         <v>567</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:5">
       <c r="A48" s="3">
         <v>46</v>
       </c>
@@ -9314,13 +9335,13 @@
         <v>16</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>730</v>
+        <v>728</v>
       </c>
       <c r="E48" s="4" t="s">
         <v>592</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:5">
       <c r="A49" s="3">
         <v>47</v>
       </c>
@@ -9331,13 +9352,13 @@
         <v>17</v>
       </c>
       <c r="D49" s="4" t="s">
-        <v>731</v>
+        <v>729</v>
       </c>
       <c r="E49" s="4" t="s">
         <v>592</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:5">
       <c r="A50" s="3">
         <v>48</v>
       </c>
@@ -9348,13 +9369,13 @@
         <v>18</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>732</v>
+        <v>730</v>
       </c>
       <c r="E50" s="4" t="s">
         <v>592</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:5">
       <c r="A51" s="3">
         <v>49</v>
       </c>
@@ -9365,13 +9386,13 @@
         <v>19</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>733</v>
+        <v>731</v>
       </c>
       <c r="E51" s="4" t="s">
         <v>592</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:5">
       <c r="A52" s="3">
         <v>50</v>
       </c>
@@ -9382,13 +9403,13 @@
         <v>20</v>
       </c>
       <c r="D52" s="4" t="s">
-        <v>734</v>
+        <v>732</v>
       </c>
       <c r="E52" s="4" t="s">
         <v>592</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:5">
       <c r="A53" s="3">
         <v>51</v>
       </c>
@@ -9399,13 +9420,13 @@
         <v>16</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>735</v>
+        <v>733</v>
       </c>
       <c r="E53" s="4" t="s">
-        <v>660</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5">
       <c r="A54" s="3">
         <v>52</v>
       </c>
@@ -9416,13 +9437,13 @@
         <v>17</v>
       </c>
       <c r="D54" s="4" t="s">
-        <v>736</v>
+        <v>734</v>
       </c>
       <c r="E54" s="4" t="s">
-        <v>660</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5">
       <c r="A55" s="3">
         <v>53</v>
       </c>
@@ -9433,13 +9454,13 @@
         <v>18</v>
       </c>
       <c r="D55" s="4" t="s">
-        <v>737</v>
+        <v>735</v>
       </c>
       <c r="E55" s="4" t="s">
-        <v>660</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5">
       <c r="A56" s="3">
         <v>54</v>
       </c>
@@ -9450,13 +9471,13 @@
         <v>19</v>
       </c>
       <c r="D56" s="4" t="s">
-        <v>738</v>
+        <v>736</v>
       </c>
       <c r="E56" s="4" t="s">
-        <v>660</v>
-      </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5">
       <c r="A57" s="3">
         <v>55</v>
       </c>
@@ -9467,18 +9488,22 @@
         <v>20</v>
       </c>
       <c r="D57" s="4" t="s">
-        <v>739</v>
+        <v>737</v>
       </c>
       <c r="E57" s="4" t="s">
-        <v>660</v>
-      </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5">
       <c r="A58" s="5" t="s">
-        <v>740</v>
+        <v>738</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;"Aptos"&amp;12&amp;KFF0000 OFFICIAL&amp;1#_x000D_</oddHeader>
+    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Aptos"&amp;12&amp;KFF0000 OFFICIAL</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added Hd parameter to input files
</commit_message>
<xml_diff>
--- a/data-raw/data.default.xlsx
+++ b/data-raw/data.default.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Forrester\Models\3-PG\r3PG_mortality_management_defoliation\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{391A5BF4-4965-477B-B28F-85BC38AF9E52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1508449C-9AC6-4417-AD96-1EAC476E3481}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{61EEFE5B-6AE1-A641-A9AB-273DC4213F59}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{61EEFE5B-6AE1-A641-A9AB-273DC4213F59}"/>
   </bookViews>
   <sheets>
     <sheet name="parameters" sheetId="8" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1264" uniqueCount="747">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1267" uniqueCount="749">
   <si>
     <t>pFS2</t>
   </si>
@@ -2272,6 +2272,12 @@
   </si>
   <si>
     <t>10-year average fPhys</t>
+  </si>
+  <si>
+    <t>Hd</t>
+  </si>
+  <si>
+    <t>Height (m) at which diameter was measured for background mortality and allometric equations</t>
   </si>
 </sst>
 </file>
@@ -2672,7 +2678,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E287297-02C0-BF44-BF0C-8FADE2A87F8F}">
-  <dimension ref="A1:D89"/>
+  <dimension ref="A1:D90"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -3616,25 +3622,25 @@
       </c>
     </row>
     <row r="69" spans="1:4">
-      <c r="A69" t="s">
-        <v>61</v>
-      </c>
-      <c r="B69" t="s">
-        <v>202</v>
-      </c>
-      <c r="C69" t="s">
-        <v>128</v>
-      </c>
-      <c r="D69">
-        <v>0</v>
+      <c r="A69" s="1" t="s">
+        <v>747</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>748</v>
+      </c>
+      <c r="C69" s="1" t="s">
+        <v>320</v>
+      </c>
+      <c r="D69" s="1">
+        <v>1.3</v>
       </c>
     </row>
     <row r="70" spans="1:4">
       <c r="A70" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B70" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C70" t="s">
         <v>128</v>
@@ -3645,10 +3651,10 @@
     </row>
     <row r="71" spans="1:4">
       <c r="A71" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B71" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C71" t="s">
         <v>128</v>
@@ -3659,10 +3665,10 @@
     </row>
     <row r="72" spans="1:4">
       <c r="A72" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B72" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C72" t="s">
         <v>128</v>
@@ -3673,10 +3679,10 @@
     </row>
     <row r="73" spans="1:4">
       <c r="A73" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B73" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C73" t="s">
         <v>128</v>
@@ -3687,10 +3693,10 @@
     </row>
     <row r="74" spans="1:4">
       <c r="A74" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B74" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C74" t="s">
         <v>128</v>
@@ -3701,10 +3707,10 @@
     </row>
     <row r="75" spans="1:4">
       <c r="A75" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B75" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C75" t="s">
         <v>128</v>
@@ -3715,10 +3721,10 @@
     </row>
     <row r="76" spans="1:4">
       <c r="A76" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B76" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C76" t="s">
         <v>128</v>
@@ -3729,10 +3735,10 @@
     </row>
     <row r="77" spans="1:4">
       <c r="A77" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B77" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C77" t="s">
         <v>128</v>
@@ -3743,10 +3749,10 @@
     </row>
     <row r="78" spans="1:4">
       <c r="A78" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B78" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C78" t="s">
         <v>128</v>
@@ -3757,10 +3763,10 @@
     </row>
     <row r="79" spans="1:4">
       <c r="A79" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B79" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C79" t="s">
         <v>128</v>
@@ -3771,10 +3777,10 @@
     </row>
     <row r="80" spans="1:4">
       <c r="A80" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B80" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C80" t="s">
         <v>128</v>
@@ -3785,10 +3791,10 @@
     </row>
     <row r="81" spans="1:4">
       <c r="A81" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B81" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C81" t="s">
         <v>128</v>
@@ -3799,10 +3805,10 @@
     </row>
     <row r="82" spans="1:4">
       <c r="A82" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B82" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C82" t="s">
         <v>128</v>
@@ -3813,10 +3819,10 @@
     </row>
     <row r="83" spans="1:4">
       <c r="A83" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B83" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C83" t="s">
         <v>128</v>
@@ -3827,10 +3833,10 @@
     </row>
     <row r="84" spans="1:4">
       <c r="A84" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B84" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C84" t="s">
         <v>128</v>
@@ -3841,10 +3847,10 @@
     </row>
     <row r="85" spans="1:4">
       <c r="A85" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B85" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C85" t="s">
         <v>128</v>
@@ -3855,57 +3861,71 @@
     </row>
     <row r="86" spans="1:4">
       <c r="A86" t="s">
-        <v>109</v>
+        <v>78</v>
       </c>
       <c r="B86" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C86" t="s">
-        <v>220</v>
+        <v>128</v>
       </c>
       <c r="D86">
-        <v>-90</v>
+        <v>0</v>
       </c>
     </row>
     <row r="87" spans="1:4">
       <c r="A87" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B87" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="C87" t="s">
-        <v>128</v>
+        <v>220</v>
       </c>
       <c r="D87">
-        <v>0.8</v>
+        <v>-90</v>
       </c>
     </row>
     <row r="88" spans="1:4">
       <c r="A88" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B88" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C88" t="s">
-        <v>223</v>
+        <v>128</v>
       </c>
       <c r="D88">
-        <v>24</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="89" spans="1:4">
       <c r="A89" t="s">
+        <v>111</v>
+      </c>
+      <c r="B89" t="s">
+        <v>222</v>
+      </c>
+      <c r="C89" t="s">
+        <v>223</v>
+      </c>
+      <c r="D89">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4">
+      <c r="A90" t="s">
         <v>112</v>
       </c>
-      <c r="B89" t="s">
+      <c r="B90" t="s">
         <v>224</v>
       </c>
-      <c r="C89" t="s">
+      <c r="C90" t="s">
         <v>225</v>
       </c>
-      <c r="D89">
+      <c r="D90">
         <v>2.2999999999999998</v>
       </c>
     </row>

</xml_diff>

<commit_message>
reset age related things for coppice events
</commit_message>
<xml_diff>
--- a/data-raw/data.default.xlsx
+++ b/data-raw/data.default.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Forrester\Models\3-PG\r3PG_mortality_management_defoliation\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E4E0500-B472-4C42-A9F9-4C08329D08B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2FF79BD-6090-42A3-80BF-86A66EB5E907}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{61EEFE5B-6AE1-A641-A9AB-273DC4213F59}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1270" uniqueCount="752">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1281" uniqueCount="760">
   <si>
     <t>pFS2</t>
   </si>
@@ -2287,6 +2287,30 @@
   </si>
   <si>
     <t>Modifier to amplify light benefit to shorter cohorts</t>
+  </si>
+  <si>
+    <t>def_type</t>
+  </si>
+  <si>
+    <t>def_recover_t</t>
+  </si>
+  <si>
+    <t>Number of trees removed due to defoliation</t>
+  </si>
+  <si>
+    <t>Stem biomass removed due to defoliation</t>
+  </si>
+  <si>
+    <t>Root biomass removed due to defoliation</t>
+  </si>
+  <si>
+    <t>Foliage biomass remoed due to defoliation</t>
+  </si>
+  <si>
+    <t>Defoliation type (1 = Pruning; 2 = Epicormic; 3 = Coppice; 4 = Stand-replacing)</t>
+  </si>
+  <si>
+    <t>Maximum number of months required to recover the pre-defoliation foliage biomass (pruning or epicormic responses) or foliage + stem mass (coppice responses) of the trees that survived the defoliation event.</t>
   </si>
 </sst>
 </file>
@@ -2365,13 +2389,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -8462,6 +8487,12 @@
       <c r="D214" t="s">
         <v>657</v>
       </c>
+      <c r="E214" t="s">
+        <v>754</v>
+      </c>
+      <c r="F214" t="s">
+        <v>305</v>
+      </c>
     </row>
     <row r="215" spans="1:6">
       <c r="A215">
@@ -8470,11 +8501,17 @@
       <c r="B215">
         <v>14</v>
       </c>
-      <c r="C215" t="s">
+      <c r="C215" s="1" t="s">
         <v>739</v>
       </c>
       <c r="D215" t="s">
         <v>657</v>
+      </c>
+      <c r="E215" t="s">
+        <v>755</v>
+      </c>
+      <c r="F215" t="s">
+        <v>390</v>
       </c>
     </row>
     <row r="216" spans="1:6">
@@ -8484,11 +8521,17 @@
       <c r="B216">
         <v>15</v>
       </c>
-      <c r="C216" t="s">
+      <c r="C216" s="1" t="s">
         <v>740</v>
       </c>
       <c r="D216" t="s">
         <v>657</v>
+      </c>
+      <c r="E216" t="s">
+        <v>756</v>
+      </c>
+      <c r="F216" t="s">
+        <v>390</v>
       </c>
     </row>
     <row r="217" spans="1:6">
@@ -8498,11 +8541,17 @@
       <c r="B217" s="4">
         <v>16</v>
       </c>
-      <c r="C217" t="s">
+      <c r="C217" s="1" t="s">
         <v>741</v>
       </c>
       <c r="D217" s="4" t="s">
         <v>657</v>
+      </c>
+      <c r="E217" t="s">
+        <v>757</v>
+      </c>
+      <c r="F217" t="s">
+        <v>390</v>
       </c>
     </row>
     <row r="218" spans="1:6">
@@ -8512,11 +8561,14 @@
       <c r="B218" s="4">
         <v>17</v>
       </c>
-      <c r="C218" s="4" t="s">
-        <v>733</v>
+      <c r="C218" s="6" t="s">
+        <v>752</v>
       </c>
       <c r="D218" s="4" t="s">
         <v>657</v>
+      </c>
+      <c r="E218" t="s">
+        <v>758</v>
       </c>
     </row>
     <row r="219" spans="1:6">
@@ -8526,11 +8578,17 @@
       <c r="B219" s="4">
         <v>18</v>
       </c>
-      <c r="C219" s="4" t="s">
-        <v>734</v>
+      <c r="C219" s="6" t="s">
+        <v>753</v>
       </c>
       <c r="D219" s="4" t="s">
         <v>657</v>
+      </c>
+      <c r="E219" t="s">
+        <v>759</v>
+      </c>
+      <c r="F219" s="4" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="220" spans="1:6">

</xml_diff>

<commit_message>
fixing biomass reduction due to defoliation
</commit_message>
<xml_diff>
--- a/data-raw/data.default.xlsx
+++ b/data-raw/data.default.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Forrester\Models\3-PG\r3PG_mortality_management_defoliation\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56F7C97A-0B8B-437E-A7F3-6C5A7420771B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E43DBBA-826E-4163-B061-5852093B1EA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="390" windowWidth="20940" windowHeight="21015" activeTab="2" xr2:uid="{61EEFE5B-6AE1-A641-A9AB-273DC4213F59}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{61EEFE5B-6AE1-A641-A9AB-273DC4213F59}"/>
   </bookViews>
   <sheets>
     <sheet name="parameters" sheetId="8" r:id="rId1"/>
@@ -2304,13 +2304,13 @@
     <t>Root biomass removed due to defoliation</t>
   </si>
   <si>
-    <t>Foliage biomass remoed due to defoliation</t>
-  </si>
-  <si>
     <t>Defoliation type (1 = Pruning; 2 = Epicormic; 3 = Coppice; 4 = Stand-replacing)</t>
   </si>
   <si>
     <t>Maximum number of months required to recover the pre-defoliation foliage biomass (pruning or epicormic responses) or foliage + stem mass (coppice responses) of the trees that survived the defoliation event.</t>
+  </si>
+  <si>
+    <t>Foliage biomass removed due to defoliation</t>
   </si>
 </sst>
 </file>
@@ -8548,7 +8548,7 @@
         <v>657</v>
       </c>
       <c r="E217" t="s">
-        <v>757</v>
+        <v>759</v>
       </c>
       <c r="F217" t="s">
         <v>390</v>
@@ -8568,7 +8568,7 @@
         <v>657</v>
       </c>
       <c r="E218" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
     </row>
     <row r="219" spans="1:6">
@@ -8585,7 +8585,7 @@
         <v>657</v>
       </c>
       <c r="E219" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="F219" s="4" t="s">
         <v>138</v>

</xml_diff>

<commit_message>
Add all 12 soil textures
</commit_message>
<xml_diff>
--- a/data-raw/data.default.xlsx
+++ b/data-raw/data.default.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Forrester\Models\3-PG\r3PG_mortality_management_defoliation\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{012E5397-90E6-48BB-8F7B-234485784936}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35E6E07D-6DC8-4E59-A391-D457F44847EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{61EEFE5B-6AE1-A641-A9AB-273DC4213F59}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{61EEFE5B-6AE1-A641-A9AB-273DC4213F59}"/>
   </bookViews>
   <sheets>
     <sheet name="parameters" sheetId="8" r:id="rId1"/>
@@ -2711,6 +2711,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E287297-02C0-BF44-BF0C-8FADE2A87F8F}">
   <dimension ref="A1:D91"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
+  <cols>
+    <col min="2" max="2" width="80" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">

</xml_diff>

<commit_message>
removing bias calculations, ws distribution calculation, and those outputs
</commit_message>
<xml_diff>
--- a/data-raw/data.default.xlsx
+++ b/data-raw/data.default.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Forrester\Models\3-PG\r3PG_mortality_management_defoliation\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A073BA2D-C924-40F2-8E67-416E65DDE160}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4794D4DA-529C-4ADA-815D-660F68455283}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{61EEFE5B-6AE1-A641-A9AB-273DC4213F59}"/>
+    <workbookView xWindow="4425" yWindow="1260" windowWidth="28800" windowHeight="15225" activeTab="2" xr2:uid="{61EEFE5B-6AE1-A641-A9AB-273DC4213F59}"/>
   </bookViews>
   <sheets>
     <sheet name="parameters" sheetId="8" r:id="rId1"/>
@@ -1752,99 +1752,66 @@
     <t>DWeibullLocation</t>
   </si>
   <si>
-    <t>wsweibullscale</t>
-  </si>
-  <si>
     <t>Weibull scale parameter of stem biomass distribution</t>
   </si>
   <si>
     <t>wsWeibullScale</t>
   </si>
   <si>
-    <t>wsweibullshape</t>
-  </si>
-  <si>
     <t>Weibull shape parameter of stem biomass distribution</t>
   </si>
   <si>
     <t>wsWeibullShape</t>
   </si>
   <si>
-    <t>wsweibulllocation</t>
-  </si>
-  <si>
     <t>Weibull location parameter of stem biomass distribution</t>
   </si>
   <si>
     <t>wsWeibullLocation</t>
   </si>
   <si>
-    <t>CVdbhDistribution</t>
-  </si>
-  <si>
     <t>Slope of CV of avDBH distribution vs age relationship</t>
   </si>
   <si>
     <t>CV of dbh Distribution</t>
   </si>
   <si>
-    <t>CVwsDistribution</t>
-  </si>
-  <si>
     <t>Coefficient of variation of stem biomass distribution</t>
   </si>
   <si>
     <t>CV of ws Distribution</t>
   </si>
   <si>
-    <t>wsrelBias</t>
-  </si>
-  <si>
     <t xml:space="preserve">Relative bias of calculating avDBH from mean stem biomass </t>
   </si>
   <si>
     <t>Relative bias in dbh from using mean ws</t>
   </si>
   <si>
-    <t>DrelBiaspFS</t>
-  </si>
-  <si>
     <t xml:space="preserve">Relative bias of calculating pFS from avDBH </t>
   </si>
   <si>
     <t>Relative bias in pFS from using mean dbh</t>
   </si>
   <si>
-    <t>DrelBiasheight</t>
-  </si>
-  <si>
     <t xml:space="preserve">Relative bias of calculating mean Height from avDBH </t>
   </si>
   <si>
     <t>Relative bias in height from using mean dbh</t>
   </si>
   <si>
-    <t>DrelBiasBasArea</t>
-  </si>
-  <si>
     <t xml:space="preserve">Relative bias of calculating mean tree basal area from avDBH </t>
   </si>
   <si>
     <t>Relative bias in basal area from using mean dbh</t>
   </si>
   <si>
-    <t>DrelBiasLCL</t>
-  </si>
-  <si>
     <t xml:space="preserve">Relative bias of calculating mean live-crown length from avDBH </t>
   </si>
   <si>
     <t>Relative bias in LCL from using mean dbh</t>
   </si>
   <si>
-    <t>DrelBiasCrowndiameter</t>
-  </si>
-  <si>
     <t xml:space="preserve">Relative bias of calculating mean crown diameter from avDBH </t>
   </si>
   <si>
@@ -2284,6 +2251,39 @@
   </si>
   <si>
     <t>Parameter of crown length equation</t>
+  </si>
+  <si>
+    <t>var_10_4</t>
+  </si>
+  <si>
+    <t>var_10_5</t>
+  </si>
+  <si>
+    <t>var_10_6</t>
+  </si>
+  <si>
+    <t>var_10_7</t>
+  </si>
+  <si>
+    <t>var_10_8</t>
+  </si>
+  <si>
+    <t>var_10_9</t>
+  </si>
+  <si>
+    <t>var_10_10</t>
+  </si>
+  <si>
+    <t>var_10_11</t>
+  </si>
+  <si>
+    <t>var_10_12</t>
+  </si>
+  <si>
+    <t>var_10_13</t>
+  </si>
+  <si>
+    <t>var_10_14</t>
   </si>
 </sst>
 </file>
@@ -2934,7 +2934,7 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>735</v>
+        <v>724</v>
       </c>
       <c r="C18" t="s">
         <v>118</v>
@@ -3155,10 +3155,10 @@
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="1" t="s">
-        <v>608</v>
+        <v>597</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>614</v>
+        <v>603</v>
       </c>
       <c r="C34" s="1"/>
       <c r="D34" s="1">
@@ -3167,10 +3167,10 @@
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="1" t="s">
-        <v>609</v>
+        <v>598</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>615</v>
+        <v>604</v>
       </c>
       <c r="C35" s="1"/>
       <c r="D35" s="1">
@@ -3179,10 +3179,10 @@
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="1" t="s">
-        <v>610</v>
+        <v>599</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>616</v>
+        <v>605</v>
       </c>
       <c r="C36" s="1"/>
       <c r="D36" s="1">
@@ -3191,10 +3191,10 @@
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="1" t="s">
-        <v>611</v>
+        <v>600</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>617</v>
+        <v>606</v>
       </c>
       <c r="C37" s="1"/>
       <c r="D37" s="1">
@@ -3203,10 +3203,10 @@
     </row>
     <row r="38" spans="1:4">
       <c r="A38" s="1" t="s">
-        <v>612</v>
+        <v>601</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>618</v>
+        <v>607</v>
       </c>
       <c r="C38" s="1"/>
       <c r="D38" s="1">
@@ -3215,10 +3215,10 @@
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="1" t="s">
-        <v>613</v>
+        <v>602</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>619</v>
+        <v>608</v>
       </c>
       <c r="C39" s="1"/>
       <c r="D39" s="1">
@@ -3325,10 +3325,10 @@
     </row>
     <row r="47" spans="1:4">
       <c r="A47" s="1" t="s">
-        <v>721</v>
+        <v>710</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>722</v>
+        <v>711</v>
       </c>
       <c r="C47" s="1"/>
       <c r="D47" s="1">
@@ -3645,10 +3645,10 @@
     </row>
     <row r="70" spans="1:4">
       <c r="A70" s="1" t="s">
-        <v>719</v>
+        <v>708</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>720</v>
+        <v>709</v>
       </c>
       <c r="C70" s="1" t="s">
         <v>296</v>
@@ -3662,7 +3662,7 @@
         <v>61</v>
       </c>
       <c r="B71" t="s">
-        <v>748</v>
+        <v>737</v>
       </c>
       <c r="C71" t="s">
         <v>118</v>
@@ -3673,10 +3673,10 @@
     </row>
     <row r="72" spans="1:4">
       <c r="A72" t="s">
-        <v>736</v>
+        <v>725</v>
       </c>
       <c r="B72" t="s">
-        <v>748</v>
+        <v>737</v>
       </c>
       <c r="C72" t="s">
         <v>118</v>
@@ -3687,10 +3687,10 @@
     </row>
     <row r="73" spans="1:4">
       <c r="A73" t="s">
+        <v>726</v>
+      </c>
+      <c r="B73" t="s">
         <v>737</v>
-      </c>
-      <c r="B73" t="s">
-        <v>748</v>
       </c>
       <c r="C73" t="s">
         <v>118</v>
@@ -3701,18 +3701,18 @@
     </row>
     <row r="74" spans="1:4">
       <c r="A74" t="s">
-        <v>746</v>
+        <v>735</v>
       </c>
       <c r="B74" t="s">
-        <v>748</v>
+        <v>737</v>
       </c>
     </row>
     <row r="75" spans="1:4">
       <c r="A75" t="s">
-        <v>747</v>
+        <v>736</v>
       </c>
       <c r="B75" t="s">
-        <v>748</v>
+        <v>737</v>
       </c>
     </row>
     <row r="76" spans="1:4">
@@ -3776,7 +3776,7 @@
         <v>67</v>
       </c>
       <c r="B80" t="s">
-        <v>749</v>
+        <v>738</v>
       </c>
       <c r="C80" t="s">
         <v>118</v>
@@ -3787,10 +3787,10 @@
     </row>
     <row r="81" spans="1:4">
       <c r="A81" t="s">
+        <v>727</v>
+      </c>
+      <c r="B81" t="s">
         <v>738</v>
-      </c>
-      <c r="B81" t="s">
-        <v>749</v>
       </c>
       <c r="C81" t="s">
         <v>118</v>
@@ -3801,10 +3801,10 @@
     </row>
     <row r="82" spans="1:4">
       <c r="A82" t="s">
-        <v>739</v>
+        <v>728</v>
       </c>
       <c r="B82" t="s">
-        <v>749</v>
+        <v>738</v>
       </c>
       <c r="C82" t="s">
         <v>118</v>
@@ -3815,10 +3815,10 @@
     </row>
     <row r="83" spans="1:4">
       <c r="A83" t="s">
-        <v>740</v>
+        <v>729</v>
       </c>
       <c r="B83" t="s">
-        <v>749</v>
+        <v>738</v>
       </c>
       <c r="C83" t="s">
         <v>118</v>
@@ -3829,10 +3829,10 @@
     </row>
     <row r="84" spans="1:4">
       <c r="A84" t="s">
-        <v>741</v>
+        <v>730</v>
       </c>
       <c r="B84" t="s">
-        <v>749</v>
+        <v>738</v>
       </c>
       <c r="C84" t="s">
         <v>118</v>
@@ -3846,7 +3846,7 @@
         <v>68</v>
       </c>
       <c r="B85" t="s">
-        <v>750</v>
+        <v>739</v>
       </c>
       <c r="C85" t="s">
         <v>118</v>
@@ -3857,10 +3857,10 @@
     </row>
     <row r="86" spans="1:4">
       <c r="A86" t="s">
-        <v>742</v>
+        <v>731</v>
       </c>
       <c r="B86" t="s">
-        <v>750</v>
+        <v>739</v>
       </c>
       <c r="C86" t="s">
         <v>118</v>
@@ -3871,10 +3871,10 @@
     </row>
     <row r="87" spans="1:4">
       <c r="A87" t="s">
-        <v>743</v>
+        <v>732</v>
       </c>
       <c r="B87" t="s">
-        <v>750</v>
+        <v>739</v>
       </c>
       <c r="C87" t="s">
         <v>118</v>
@@ -3885,10 +3885,10 @@
     </row>
     <row r="88" spans="1:4">
       <c r="A88" t="s">
-        <v>744</v>
+        <v>733</v>
       </c>
       <c r="B88" t="s">
-        <v>750</v>
+        <v>739</v>
       </c>
       <c r="C88" t="s">
         <v>118</v>
@@ -3899,10 +3899,10 @@
     </row>
     <row r="89" spans="1:4">
       <c r="A89" t="s">
-        <v>745</v>
+        <v>734</v>
       </c>
       <c r="B89" t="s">
-        <v>750</v>
+        <v>739</v>
       </c>
       <c r="C89" t="s">
         <v>118</v>
@@ -4772,7 +4772,7 @@
         <v>16</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>655</v>
+        <v>644</v>
       </c>
       <c r="D17" s="4" t="s">
         <v>237</v>
@@ -4786,7 +4786,7 @@
         <v>17</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>656</v>
+        <v>645</v>
       </c>
       <c r="D18" s="4" t="s">
         <v>237</v>
@@ -4800,7 +4800,7 @@
         <v>18</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>657</v>
+        <v>646</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>237</v>
@@ -4814,7 +4814,7 @@
         <v>19</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>658</v>
+        <v>647</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>237</v>
@@ -4828,7 +4828,7 @@
         <v>20</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>659</v>
+        <v>648</v>
       </c>
       <c r="D21" s="4" t="s">
         <v>237</v>
@@ -5169,7 +5169,7 @@
         <v>16</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>660</v>
+        <v>649</v>
       </c>
       <c r="D37" s="4" t="s">
         <v>276</v>
@@ -5183,7 +5183,7 @@
         <v>17</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>661</v>
+        <v>650</v>
       </c>
       <c r="D38" s="4" t="s">
         <v>276</v>
@@ -5197,7 +5197,7 @@
         <v>18</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>662</v>
+        <v>651</v>
       </c>
       <c r="D39" s="4" t="s">
         <v>276</v>
@@ -5211,7 +5211,7 @@
         <v>19</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>663</v>
+        <v>652</v>
       </c>
       <c r="D40" s="4" t="s">
         <v>276</v>
@@ -5225,7 +5225,7 @@
         <v>20</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>664</v>
+        <v>653</v>
       </c>
       <c r="D41" s="4" t="s">
         <v>276</v>
@@ -5489,13 +5489,13 @@
         <v>12</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>723</v>
+        <v>712</v>
       </c>
       <c r="D53" t="s">
         <v>324</v>
       </c>
       <c r="E53" t="s">
-        <v>724</v>
+        <v>713</v>
       </c>
     </row>
     <row r="54" spans="1:7">
@@ -5548,7 +5548,7 @@
         <v>16</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>665</v>
+        <v>654</v>
       </c>
       <c r="D57" s="4" t="s">
         <v>324</v>
@@ -5562,7 +5562,7 @@
         <v>17</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>666</v>
+        <v>655</v>
       </c>
       <c r="D58" s="4" t="s">
         <v>324</v>
@@ -5576,7 +5576,7 @@
         <v>18</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>667</v>
+        <v>656</v>
       </c>
       <c r="D59" s="4" t="s">
         <v>324</v>
@@ -5590,7 +5590,7 @@
         <v>19</v>
       </c>
       <c r="C60" s="4" t="s">
-        <v>668</v>
+        <v>657</v>
       </c>
       <c r="D60" s="4" t="s">
         <v>324</v>
@@ -5604,7 +5604,7 @@
         <v>20</v>
       </c>
       <c r="C61" s="4" t="s">
-        <v>669</v>
+        <v>658</v>
       </c>
       <c r="D61" s="4" t="s">
         <v>324</v>
@@ -5924,7 +5924,7 @@
         <v>16</v>
       </c>
       <c r="C77" s="4" t="s">
-        <v>670</v>
+        <v>659</v>
       </c>
       <c r="D77" s="4" t="s">
         <v>364</v>
@@ -5938,7 +5938,7 @@
         <v>17</v>
       </c>
       <c r="C78" s="4" t="s">
-        <v>671</v>
+        <v>660</v>
       </c>
       <c r="D78" s="4" t="s">
         <v>364</v>
@@ -5952,7 +5952,7 @@
         <v>18</v>
       </c>
       <c r="C79" s="4" t="s">
-        <v>672</v>
+        <v>661</v>
       </c>
       <c r="D79" s="4" t="s">
         <v>364</v>
@@ -5966,7 +5966,7 @@
         <v>19</v>
       </c>
       <c r="C80" s="4" t="s">
-        <v>673</v>
+        <v>662</v>
       </c>
       <c r="D80" s="4" t="s">
         <v>364</v>
@@ -5980,7 +5980,7 @@
         <v>20</v>
       </c>
       <c r="C81" s="4" t="s">
-        <v>674</v>
+        <v>663</v>
       </c>
       <c r="D81" s="4" t="s">
         <v>364</v>
@@ -6309,7 +6309,7 @@
         <v>16</v>
       </c>
       <c r="C97" s="4" t="s">
-        <v>675</v>
+        <v>664</v>
       </c>
       <c r="D97" s="4" t="s">
         <v>403</v>
@@ -6323,7 +6323,7 @@
         <v>17</v>
       </c>
       <c r="C98" s="4" t="s">
-        <v>676</v>
+        <v>665</v>
       </c>
       <c r="D98" s="4" t="s">
         <v>403</v>
@@ -6337,7 +6337,7 @@
         <v>18</v>
       </c>
       <c r="C99" s="4" t="s">
-        <v>677</v>
+        <v>666</v>
       </c>
       <c r="D99" s="4" t="s">
         <v>403</v>
@@ -6351,7 +6351,7 @@
         <v>19</v>
       </c>
       <c r="C100" s="4" t="s">
-        <v>678</v>
+        <v>667</v>
       </c>
       <c r="D100" s="4" t="s">
         <v>403</v>
@@ -6365,7 +6365,7 @@
         <v>20</v>
       </c>
       <c r="C101" s="4" t="s">
-        <v>679</v>
+        <v>668</v>
       </c>
       <c r="D101" s="4" t="s">
         <v>403</v>
@@ -6425,7 +6425,7 @@
         <v>3</v>
       </c>
       <c r="C104" t="s">
-        <v>607</v>
+        <v>596</v>
       </c>
       <c r="D104" t="s">
         <v>443</v>
@@ -6706,7 +6706,7 @@
         <v>16</v>
       </c>
       <c r="C117" s="4" t="s">
-        <v>680</v>
+        <v>669</v>
       </c>
       <c r="D117" s="4" t="s">
         <v>443</v>
@@ -6720,7 +6720,7 @@
         <v>17</v>
       </c>
       <c r="C118" s="4" t="s">
-        <v>681</v>
+        <v>670</v>
       </c>
       <c r="D118" s="4" t="s">
         <v>443</v>
@@ -6734,7 +6734,7 @@
         <v>18</v>
       </c>
       <c r="C119" s="4" t="s">
-        <v>682</v>
+        <v>671</v>
       </c>
       <c r="D119" s="4" t="s">
         <v>443</v>
@@ -6748,7 +6748,7 @@
         <v>19</v>
       </c>
       <c r="C120" s="4" t="s">
-        <v>683</v>
+        <v>672</v>
       </c>
       <c r="D120" s="4" t="s">
         <v>443</v>
@@ -6762,7 +6762,7 @@
         <v>20</v>
       </c>
       <c r="C121" s="4" t="s">
-        <v>684</v>
+        <v>673</v>
       </c>
       <c r="D121" s="4" t="s">
         <v>443</v>
@@ -7103,7 +7103,7 @@
         <v>16</v>
       </c>
       <c r="C137" s="4" t="s">
-        <v>685</v>
+        <v>674</v>
       </c>
       <c r="D137" s="4" t="s">
         <v>485</v>
@@ -7117,7 +7117,7 @@
         <v>17</v>
       </c>
       <c r="C138" s="4" t="s">
-        <v>686</v>
+        <v>675</v>
       </c>
       <c r="D138" s="4" t="s">
         <v>485</v>
@@ -7131,7 +7131,7 @@
         <v>18</v>
       </c>
       <c r="C139" s="4" t="s">
-        <v>687</v>
+        <v>676</v>
       </c>
       <c r="D139" s="4" t="s">
         <v>485</v>
@@ -7145,7 +7145,7 @@
         <v>19</v>
       </c>
       <c r="C140" s="4" t="s">
-        <v>688</v>
+        <v>677</v>
       </c>
       <c r="D140" s="4" t="s">
         <v>485</v>
@@ -7159,7 +7159,7 @@
         <v>20</v>
       </c>
       <c r="C141" s="4" t="s">
-        <v>689</v>
+        <v>678</v>
       </c>
       <c r="D141" s="4" t="s">
         <v>485</v>
@@ -7219,13 +7219,13 @@
         <v>3</v>
       </c>
       <c r="C144" s="1" t="s">
-        <v>620</v>
+        <v>609</v>
       </c>
       <c r="D144" t="s">
         <v>529</v>
       </c>
       <c r="E144" t="s">
-        <v>625</v>
+        <v>614</v>
       </c>
       <c r="F144" t="s">
         <v>281</v>
@@ -7242,7 +7242,7 @@
         <v>4</v>
       </c>
       <c r="C145" s="1" t="s">
-        <v>626</v>
+        <v>615</v>
       </c>
       <c r="D145" t="s">
         <v>529</v>
@@ -7256,7 +7256,7 @@
         <v>5</v>
       </c>
       <c r="C146" s="1" t="s">
-        <v>627</v>
+        <v>616</v>
       </c>
       <c r="D146" t="s">
         <v>529</v>
@@ -7270,7 +7270,7 @@
         <v>6</v>
       </c>
       <c r="C147" s="1" t="s">
-        <v>628</v>
+        <v>617</v>
       </c>
       <c r="D147" t="s">
         <v>529</v>
@@ -7284,13 +7284,13 @@
         <v>7</v>
       </c>
       <c r="C148" s="1" t="s">
-        <v>715</v>
+        <v>704</v>
       </c>
       <c r="D148" t="s">
         <v>529</v>
       </c>
       <c r="E148" t="s">
-        <v>717</v>
+        <v>706</v>
       </c>
     </row>
     <row r="149" spans="1:5">
@@ -7301,13 +7301,13 @@
         <v>8</v>
       </c>
       <c r="C149" s="1" t="s">
-        <v>716</v>
+        <v>705</v>
       </c>
       <c r="D149" t="s">
         <v>529</v>
       </c>
       <c r="E149" t="s">
-        <v>718</v>
+        <v>707</v>
       </c>
     </row>
     <row r="150" spans="1:5">
@@ -7318,7 +7318,7 @@
         <v>9</v>
       </c>
       <c r="C150" s="1" t="s">
-        <v>621</v>
+        <v>610</v>
       </c>
       <c r="D150" t="s">
         <v>529</v>
@@ -7335,13 +7335,13 @@
         <v>10</v>
       </c>
       <c r="C151" s="1" t="s">
-        <v>622</v>
+        <v>611</v>
       </c>
       <c r="D151" t="s">
         <v>529</v>
       </c>
       <c r="E151" t="s">
-        <v>629</v>
+        <v>618</v>
       </c>
     </row>
     <row r="152" spans="1:5">
@@ -7352,7 +7352,7 @@
         <v>11</v>
       </c>
       <c r="C152" s="1" t="s">
-        <v>733</v>
+        <v>722</v>
       </c>
       <c r="D152" t="s">
         <v>529</v>
@@ -7366,7 +7366,7 @@
         <v>12</v>
       </c>
       <c r="C153" s="1" t="s">
-        <v>734</v>
+        <v>723</v>
       </c>
       <c r="D153" t="s">
         <v>529</v>
@@ -7380,7 +7380,7 @@
         <v>13</v>
       </c>
       <c r="C154" s="1" t="s">
-        <v>623</v>
+        <v>612</v>
       </c>
       <c r="D154" t="s">
         <v>529</v>
@@ -7394,7 +7394,7 @@
         <v>14</v>
       </c>
       <c r="C155" s="1" t="s">
-        <v>624</v>
+        <v>613</v>
       </c>
       <c r="D155" t="s">
         <v>529</v>
@@ -7422,7 +7422,7 @@
         <v>16</v>
       </c>
       <c r="C157" s="4" t="s">
-        <v>690</v>
+        <v>679</v>
       </c>
       <c r="D157" s="4" t="s">
         <v>529</v>
@@ -7436,7 +7436,7 @@
         <v>17</v>
       </c>
       <c r="C158" s="4" t="s">
-        <v>691</v>
+        <v>680</v>
       </c>
       <c r="D158" s="4" t="s">
         <v>529</v>
@@ -7450,7 +7450,7 @@
         <v>18</v>
       </c>
       <c r="C159" s="4" t="s">
-        <v>692</v>
+        <v>681</v>
       </c>
       <c r="D159" s="4" t="s">
         <v>529</v>
@@ -7464,7 +7464,7 @@
         <v>19</v>
       </c>
       <c r="C160" s="4" t="s">
-        <v>693</v>
+        <v>682</v>
       </c>
       <c r="D160" s="4" t="s">
         <v>529</v>
@@ -7478,7 +7478,7 @@
         <v>20</v>
       </c>
       <c r="C161" s="4" t="s">
-        <v>694</v>
+        <v>683</v>
       </c>
       <c r="D161" s="4" t="s">
         <v>529</v>
@@ -7741,7 +7741,7 @@
         <v>16</v>
       </c>
       <c r="C177" s="4" t="s">
-        <v>695</v>
+        <v>684</v>
       </c>
       <c r="D177" s="4" t="s">
         <v>539</v>
@@ -7755,7 +7755,7 @@
         <v>17</v>
       </c>
       <c r="C178" s="4" t="s">
-        <v>696</v>
+        <v>685</v>
       </c>
       <c r="D178" s="4" t="s">
         <v>539</v>
@@ -7769,7 +7769,7 @@
         <v>18</v>
       </c>
       <c r="C179" s="4" t="s">
-        <v>697</v>
+        <v>686</v>
       </c>
       <c r="D179" s="4" t="s">
         <v>539</v>
@@ -7783,7 +7783,7 @@
         <v>19</v>
       </c>
       <c r="C180" s="4" t="s">
-        <v>698</v>
+        <v>687</v>
       </c>
       <c r="D180" s="4" t="s">
         <v>539</v>
@@ -7797,7 +7797,7 @@
         <v>20</v>
       </c>
       <c r="C181" s="4" t="s">
-        <v>699</v>
+        <v>688</v>
       </c>
       <c r="D181" s="4" t="s">
         <v>539</v>
@@ -7879,20 +7879,20 @@
       <c r="B185">
         <v>4</v>
       </c>
-      <c r="C185" t="s">
-        <v>573</v>
+      <c r="C185" s="1" t="s">
+        <v>740</v>
       </c>
       <c r="D185" t="s">
         <v>564</v>
       </c>
       <c r="E185" t="s">
+        <v>573</v>
+      </c>
+      <c r="F185" t="s">
+        <v>118</v>
+      </c>
+      <c r="G185" t="s">
         <v>574</v>
-      </c>
-      <c r="F185" t="s">
-        <v>118</v>
-      </c>
-      <c r="G185" t="s">
-        <v>575</v>
       </c>
     </row>
     <row r="186" spans="1:7">
@@ -7902,20 +7902,20 @@
       <c r="B186">
         <v>5</v>
       </c>
-      <c r="C186" t="s">
-        <v>576</v>
+      <c r="C186" s="1" t="s">
+        <v>741</v>
       </c>
       <c r="D186" t="s">
         <v>564</v>
       </c>
       <c r="E186" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="F186" t="s">
         <v>118</v>
       </c>
       <c r="G186" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
     </row>
     <row r="187" spans="1:7">
@@ -7925,20 +7925,20 @@
       <c r="B187">
         <v>6</v>
       </c>
-      <c r="C187" t="s">
-        <v>579</v>
+      <c r="C187" s="1" t="s">
+        <v>742</v>
       </c>
       <c r="D187" t="s">
         <v>564</v>
       </c>
       <c r="E187" t="s">
-        <v>580</v>
+        <v>577</v>
       </c>
       <c r="F187" t="s">
         <v>118</v>
       </c>
       <c r="G187" t="s">
-        <v>581</v>
+        <v>578</v>
       </c>
     </row>
     <row r="188" spans="1:7">
@@ -7948,20 +7948,20 @@
       <c r="B188">
         <v>7</v>
       </c>
-      <c r="C188" t="s">
-        <v>582</v>
+      <c r="C188" s="1" t="s">
+        <v>743</v>
       </c>
       <c r="D188" t="s">
         <v>564</v>
       </c>
       <c r="E188" t="s">
-        <v>583</v>
+        <v>579</v>
       </c>
       <c r="F188" t="s">
         <v>343</v>
       </c>
       <c r="G188" t="s">
-        <v>584</v>
+        <v>580</v>
       </c>
     </row>
     <row r="189" spans="1:7">
@@ -7971,20 +7971,20 @@
       <c r="B189">
         <v>8</v>
       </c>
-      <c r="C189" t="s">
-        <v>585</v>
+      <c r="C189" s="1" t="s">
+        <v>744</v>
       </c>
       <c r="D189" t="s">
         <v>564</v>
       </c>
       <c r="E189" t="s">
-        <v>586</v>
+        <v>581</v>
       </c>
       <c r="F189" t="s">
         <v>343</v>
       </c>
       <c r="G189" t="s">
-        <v>587</v>
+        <v>582</v>
       </c>
     </row>
     <row r="190" spans="1:7">
@@ -7994,20 +7994,20 @@
       <c r="B190">
         <v>9</v>
       </c>
-      <c r="C190" t="s">
-        <v>588</v>
+      <c r="C190" s="1" t="s">
+        <v>745</v>
       </c>
       <c r="D190" t="s">
         <v>564</v>
       </c>
       <c r="E190" t="s">
-        <v>589</v>
+        <v>583</v>
       </c>
       <c r="F190" t="s">
         <v>343</v>
       </c>
       <c r="G190" t="s">
-        <v>590</v>
+        <v>584</v>
       </c>
     </row>
     <row r="191" spans="1:7">
@@ -8017,20 +8017,20 @@
       <c r="B191">
         <v>10</v>
       </c>
-      <c r="C191" t="s">
-        <v>591</v>
+      <c r="C191" s="1" t="s">
+        <v>746</v>
       </c>
       <c r="D191" t="s">
         <v>564</v>
       </c>
       <c r="E191" t="s">
-        <v>592</v>
+        <v>585</v>
       </c>
       <c r="F191" t="s">
         <v>343</v>
       </c>
       <c r="G191" t="s">
-        <v>593</v>
+        <v>586</v>
       </c>
     </row>
     <row r="192" spans="1:7">
@@ -8040,20 +8040,20 @@
       <c r="B192">
         <v>11</v>
       </c>
-      <c r="C192" t="s">
-        <v>594</v>
+      <c r="C192" s="1" t="s">
+        <v>747</v>
       </c>
       <c r="D192" t="s">
         <v>564</v>
       </c>
       <c r="E192" t="s">
-        <v>595</v>
+        <v>587</v>
       </c>
       <c r="F192" t="s">
         <v>343</v>
       </c>
       <c r="G192" t="s">
-        <v>596</v>
+        <v>588</v>
       </c>
     </row>
     <row r="193" spans="1:7">
@@ -8063,20 +8063,20 @@
       <c r="B193">
         <v>12</v>
       </c>
-      <c r="C193" t="s">
-        <v>597</v>
+      <c r="C193" s="1" t="s">
+        <v>748</v>
       </c>
       <c r="D193" t="s">
         <v>564</v>
       </c>
       <c r="E193" t="s">
-        <v>598</v>
+        <v>589</v>
       </c>
       <c r="F193" t="s">
         <v>343</v>
       </c>
       <c r="G193" t="s">
-        <v>599</v>
+        <v>590</v>
       </c>
     </row>
     <row r="194" spans="1:7">
@@ -8086,20 +8086,20 @@
       <c r="B194">
         <v>13</v>
       </c>
-      <c r="C194" t="s">
-        <v>600</v>
+      <c r="C194" s="1" t="s">
+        <v>749</v>
       </c>
       <c r="D194" t="s">
         <v>564</v>
       </c>
       <c r="E194" t="s">
-        <v>601</v>
+        <v>591</v>
       </c>
       <c r="F194" t="s">
         <v>343</v>
       </c>
       <c r="G194" t="s">
-        <v>602</v>
+        <v>592</v>
       </c>
     </row>
     <row r="195" spans="1:7">
@@ -8109,20 +8109,20 @@
       <c r="B195">
         <v>14</v>
       </c>
-      <c r="C195" t="s">
-        <v>603</v>
+      <c r="C195" s="1" t="s">
+        <v>750</v>
       </c>
       <c r="D195" t="s">
         <v>564</v>
       </c>
       <c r="E195" t="s">
-        <v>604</v>
+        <v>593</v>
       </c>
       <c r="F195" t="s">
         <v>343</v>
       </c>
       <c r="G195" t="s">
-        <v>605</v>
+        <v>594</v>
       </c>
     </row>
     <row r="196" spans="1:7">
@@ -8132,8 +8132,8 @@
       <c r="B196">
         <v>15</v>
       </c>
-      <c r="C196" t="s">
-        <v>606</v>
+      <c r="C196" s="1" t="s">
+        <v>595</v>
       </c>
       <c r="D196" t="s">
         <v>564</v>
@@ -8147,7 +8147,7 @@
         <v>16</v>
       </c>
       <c r="C197" s="4" t="s">
-        <v>700</v>
+        <v>689</v>
       </c>
       <c r="D197" s="4" t="s">
         <v>564</v>
@@ -8161,7 +8161,7 @@
         <v>17</v>
       </c>
       <c r="C198" s="4" t="s">
-        <v>701</v>
+        <v>690</v>
       </c>
       <c r="D198" s="4" t="s">
         <v>564</v>
@@ -8175,7 +8175,7 @@
         <v>18</v>
       </c>
       <c r="C199" s="4" t="s">
-        <v>702</v>
+        <v>691</v>
       </c>
       <c r="D199" s="4" t="s">
         <v>564</v>
@@ -8189,7 +8189,7 @@
         <v>19</v>
       </c>
       <c r="C200" s="4" t="s">
-        <v>703</v>
+        <v>692</v>
       </c>
       <c r="D200" s="4" t="s">
         <v>564</v>
@@ -8203,7 +8203,7 @@
         <v>20</v>
       </c>
       <c r="C201" s="4" t="s">
-        <v>704</v>
+        <v>693</v>
       </c>
       <c r="D201" s="4" t="s">
         <v>564</v>
@@ -8217,13 +8217,13 @@
         <v>1</v>
       </c>
       <c r="C202" t="s">
-        <v>631</v>
+        <v>620</v>
       </c>
       <c r="D202" t="s">
-        <v>630</v>
+        <v>619</v>
       </c>
       <c r="E202" t="s">
-        <v>635</v>
+        <v>624</v>
       </c>
       <c r="F202" t="s">
         <v>281</v>
@@ -8237,13 +8237,13 @@
         <v>2</v>
       </c>
       <c r="C203" t="s">
-        <v>632</v>
+        <v>621</v>
       </c>
       <c r="D203" t="s">
-        <v>630</v>
+        <v>619</v>
       </c>
       <c r="E203" t="s">
-        <v>636</v>
+        <v>625</v>
       </c>
       <c r="F203" t="s">
         <v>366</v>
@@ -8257,13 +8257,13 @@
         <v>3</v>
       </c>
       <c r="C204" t="s">
-        <v>633</v>
+        <v>622</v>
       </c>
       <c r="D204" t="s">
-        <v>630</v>
+        <v>619</v>
       </c>
       <c r="E204" t="s">
-        <v>637</v>
+        <v>626</v>
       </c>
       <c r="F204" t="s">
         <v>366</v>
@@ -8277,13 +8277,13 @@
         <v>4</v>
       </c>
       <c r="C205" t="s">
-        <v>634</v>
+        <v>623</v>
       </c>
       <c r="D205" t="s">
-        <v>630</v>
+        <v>619</v>
       </c>
       <c r="E205" t="s">
-        <v>638</v>
+        <v>627</v>
       </c>
       <c r="F205" t="s">
         <v>366</v>
@@ -8297,13 +8297,13 @@
         <v>5</v>
       </c>
       <c r="C206" t="s">
-        <v>639</v>
+        <v>628</v>
       </c>
       <c r="D206" t="s">
-        <v>630</v>
+        <v>619</v>
       </c>
       <c r="E206" t="s">
-        <v>643</v>
+        <v>632</v>
       </c>
       <c r="F206" t="s">
         <v>281</v>
@@ -8317,13 +8317,13 @@
         <v>6</v>
       </c>
       <c r="C207" t="s">
-        <v>640</v>
+        <v>629</v>
       </c>
       <c r="D207" t="s">
-        <v>630</v>
+        <v>619</v>
       </c>
       <c r="E207" t="s">
-        <v>644</v>
+        <v>633</v>
       </c>
       <c r="F207" t="s">
         <v>366</v>
@@ -8337,13 +8337,13 @@
         <v>7</v>
       </c>
       <c r="C208" t="s">
-        <v>641</v>
+        <v>630</v>
       </c>
       <c r="D208" t="s">
-        <v>630</v>
+        <v>619</v>
       </c>
       <c r="E208" t="s">
-        <v>645</v>
+        <v>634</v>
       </c>
       <c r="F208" t="s">
         <v>366</v>
@@ -8357,13 +8357,13 @@
         <v>8</v>
       </c>
       <c r="C209" t="s">
-        <v>642</v>
+        <v>631</v>
       </c>
       <c r="D209" t="s">
-        <v>630</v>
+        <v>619</v>
       </c>
       <c r="E209" t="s">
-        <v>646</v>
+        <v>635</v>
       </c>
       <c r="F209" t="s">
         <v>366</v>
@@ -8377,13 +8377,13 @@
         <v>9</v>
       </c>
       <c r="C210" t="s">
-        <v>647</v>
+        <v>636</v>
       </c>
       <c r="D210" t="s">
-        <v>630</v>
+        <v>619</v>
       </c>
       <c r="E210" t="s">
-        <v>651</v>
+        <v>640</v>
       </c>
       <c r="F210" t="s">
         <v>281</v>
@@ -8397,13 +8397,13 @@
         <v>10</v>
       </c>
       <c r="C211" t="s">
-        <v>648</v>
+        <v>637</v>
       </c>
       <c r="D211" t="s">
-        <v>630</v>
+        <v>619</v>
       </c>
       <c r="E211" t="s">
-        <v>652</v>
+        <v>641</v>
       </c>
       <c r="F211" t="s">
         <v>366</v>
@@ -8417,13 +8417,13 @@
         <v>11</v>
       </c>
       <c r="C212" t="s">
-        <v>649</v>
+        <v>638</v>
       </c>
       <c r="D212" t="s">
-        <v>630</v>
+        <v>619</v>
       </c>
       <c r="E212" t="s">
-        <v>653</v>
+        <v>642</v>
       </c>
       <c r="F212" t="s">
         <v>366</v>
@@ -8437,13 +8437,13 @@
         <v>12</v>
       </c>
       <c r="C213" t="s">
-        <v>650</v>
+        <v>639</v>
       </c>
       <c r="D213" t="s">
-        <v>630</v>
+        <v>619</v>
       </c>
       <c r="E213" t="s">
-        <v>654</v>
+        <v>643</v>
       </c>
       <c r="F213" t="s">
         <v>366</v>
@@ -8457,13 +8457,13 @@
         <v>13</v>
       </c>
       <c r="C214" s="1" t="s">
-        <v>711</v>
+        <v>700</v>
       </c>
       <c r="D214" t="s">
-        <v>630</v>
+        <v>619</v>
       </c>
       <c r="E214" t="s">
-        <v>727</v>
+        <v>716</v>
       </c>
       <c r="F214" t="s">
         <v>281</v>
@@ -8477,13 +8477,13 @@
         <v>14</v>
       </c>
       <c r="C215" s="1" t="s">
-        <v>712</v>
+        <v>701</v>
       </c>
       <c r="D215" t="s">
-        <v>630</v>
+        <v>619</v>
       </c>
       <c r="E215" t="s">
-        <v>728</v>
+        <v>717</v>
       </c>
       <c r="F215" t="s">
         <v>366</v>
@@ -8497,13 +8497,13 @@
         <v>15</v>
       </c>
       <c r="C216" s="1" t="s">
-        <v>713</v>
+        <v>702</v>
       </c>
       <c r="D216" t="s">
-        <v>630</v>
+        <v>619</v>
       </c>
       <c r="E216" t="s">
-        <v>729</v>
+        <v>718</v>
       </c>
       <c r="F216" t="s">
         <v>366</v>
@@ -8517,13 +8517,13 @@
         <v>16</v>
       </c>
       <c r="C217" s="1" t="s">
-        <v>714</v>
+        <v>703</v>
       </c>
       <c r="D217" s="4" t="s">
-        <v>630</v>
+        <v>619</v>
       </c>
       <c r="E217" t="s">
-        <v>732</v>
+        <v>721</v>
       </c>
       <c r="F217" t="s">
         <v>366</v>
@@ -8537,13 +8537,13 @@
         <v>17</v>
       </c>
       <c r="C218" s="6" t="s">
-        <v>725</v>
+        <v>714</v>
       </c>
       <c r="D218" s="4" t="s">
-        <v>630</v>
+        <v>619</v>
       </c>
       <c r="E218" t="s">
-        <v>730</v>
+        <v>719</v>
       </c>
     </row>
     <row r="219" spans="1:6">
@@ -8554,13 +8554,13 @@
         <v>18</v>
       </c>
       <c r="C219" s="6" t="s">
-        <v>726</v>
+        <v>715</v>
       </c>
       <c r="D219" s="4" t="s">
-        <v>630</v>
+        <v>619</v>
       </c>
       <c r="E219" t="s">
-        <v>731</v>
+        <v>720</v>
       </c>
       <c r="F219" s="4" t="s">
         <v>128</v>
@@ -8574,10 +8574,10 @@
         <v>19</v>
       </c>
       <c r="C220" s="4" t="s">
-        <v>708</v>
+        <v>697</v>
       </c>
       <c r="D220" s="4" t="s">
-        <v>630</v>
+        <v>619</v>
       </c>
     </row>
     <row r="221" spans="1:6">
@@ -8588,10 +8588,10 @@
         <v>20</v>
       </c>
       <c r="C221" s="4" t="s">
-        <v>709</v>
+        <v>698</v>
       </c>
       <c r="D221" s="4" t="s">
-        <v>630</v>
+        <v>619</v>
       </c>
     </row>
   </sheetData>
@@ -8647,7 +8647,7 @@
         <v>16</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>655</v>
+        <v>644</v>
       </c>
       <c r="E3" s="4" t="s">
         <v>237</v>
@@ -8664,7 +8664,7 @@
         <v>17</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>656</v>
+        <v>645</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>237</v>
@@ -8681,7 +8681,7 @@
         <v>18</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>657</v>
+        <v>646</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>237</v>
@@ -8698,7 +8698,7 @@
         <v>19</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>658</v>
+        <v>647</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>237</v>
@@ -8715,7 +8715,7 @@
         <v>20</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>659</v>
+        <v>648</v>
       </c>
       <c r="E7" s="4" t="s">
         <v>237</v>
@@ -8732,7 +8732,7 @@
         <v>16</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>660</v>
+        <v>649</v>
       </c>
       <c r="E8" s="4" t="s">
         <v>276</v>
@@ -8749,7 +8749,7 @@
         <v>17</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>661</v>
+        <v>650</v>
       </c>
       <c r="E9" s="4" t="s">
         <v>276</v>
@@ -8766,7 +8766,7 @@
         <v>18</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>662</v>
+        <v>651</v>
       </c>
       <c r="E10" s="4" t="s">
         <v>276</v>
@@ -8783,7 +8783,7 @@
         <v>19</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>663</v>
+        <v>652</v>
       </c>
       <c r="E11" s="4" t="s">
         <v>276</v>
@@ -8800,7 +8800,7 @@
         <v>20</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>664</v>
+        <v>653</v>
       </c>
       <c r="E12" s="4" t="s">
         <v>276</v>
@@ -8817,7 +8817,7 @@
         <v>16</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>665</v>
+        <v>654</v>
       </c>
       <c r="E13" s="4" t="s">
         <v>324</v>
@@ -8834,7 +8834,7 @@
         <v>17</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>666</v>
+        <v>655</v>
       </c>
       <c r="E14" s="4" t="s">
         <v>324</v>
@@ -8851,7 +8851,7 @@
         <v>18</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>667</v>
+        <v>656</v>
       </c>
       <c r="E15" s="4" t="s">
         <v>324</v>
@@ -8868,7 +8868,7 @@
         <v>19</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>668</v>
+        <v>657</v>
       </c>
       <c r="E16" s="4" t="s">
         <v>324</v>
@@ -8885,7 +8885,7 @@
         <v>20</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>669</v>
+        <v>658</v>
       </c>
       <c r="E17" s="4" t="s">
         <v>324</v>
@@ -8902,7 +8902,7 @@
         <v>16</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>670</v>
+        <v>659</v>
       </c>
       <c r="E18" s="4" t="s">
         <v>364</v>
@@ -8919,7 +8919,7 @@
         <v>17</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>671</v>
+        <v>660</v>
       </c>
       <c r="E19" s="4" t="s">
         <v>364</v>
@@ -8936,7 +8936,7 @@
         <v>18</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>672</v>
+        <v>661</v>
       </c>
       <c r="E20" s="4" t="s">
         <v>364</v>
@@ -8953,7 +8953,7 @@
         <v>19</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>673</v>
+        <v>662</v>
       </c>
       <c r="E21" s="4" t="s">
         <v>364</v>
@@ -8970,7 +8970,7 @@
         <v>20</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>674</v>
+        <v>663</v>
       </c>
       <c r="E22" s="4" t="s">
         <v>364</v>
@@ -8987,7 +8987,7 @@
         <v>16</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>675</v>
+        <v>664</v>
       </c>
       <c r="E23" s="4" t="s">
         <v>403</v>
@@ -9004,7 +9004,7 @@
         <v>17</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>676</v>
+        <v>665</v>
       </c>
       <c r="E24" s="4" t="s">
         <v>403</v>
@@ -9021,7 +9021,7 @@
         <v>18</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>677</v>
+        <v>666</v>
       </c>
       <c r="E25" s="4" t="s">
         <v>403</v>
@@ -9038,7 +9038,7 @@
         <v>19</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>678</v>
+        <v>667</v>
       </c>
       <c r="E26" s="4" t="s">
         <v>403</v>
@@ -9055,7 +9055,7 @@
         <v>20</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>679</v>
+        <v>668</v>
       </c>
       <c r="E27" s="4" t="s">
         <v>403</v>
@@ -9072,7 +9072,7 @@
         <v>16</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>680</v>
+        <v>669</v>
       </c>
       <c r="E28" s="4" t="s">
         <v>443</v>
@@ -9089,7 +9089,7 @@
         <v>17</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>681</v>
+        <v>670</v>
       </c>
       <c r="E29" s="4" t="s">
         <v>443</v>
@@ -9106,7 +9106,7 @@
         <v>18</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>682</v>
+        <v>671</v>
       </c>
       <c r="E30" s="4" t="s">
         <v>443</v>
@@ -9123,7 +9123,7 @@
         <v>19</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>683</v>
+        <v>672</v>
       </c>
       <c r="E31" s="4" t="s">
         <v>443</v>
@@ -9140,7 +9140,7 @@
         <v>20</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>684</v>
+        <v>673</v>
       </c>
       <c r="E32" s="4" t="s">
         <v>443</v>
@@ -9157,7 +9157,7 @@
         <v>16</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>685</v>
+        <v>674</v>
       </c>
       <c r="E33" s="4" t="s">
         <v>485</v>
@@ -9174,7 +9174,7 @@
         <v>17</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>686</v>
+        <v>675</v>
       </c>
       <c r="E34" s="4" t="s">
         <v>485</v>
@@ -9191,7 +9191,7 @@
         <v>18</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>687</v>
+        <v>676</v>
       </c>
       <c r="E35" s="4" t="s">
         <v>485</v>
@@ -9208,7 +9208,7 @@
         <v>19</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>688</v>
+        <v>677</v>
       </c>
       <c r="E36" s="4" t="s">
         <v>485</v>
@@ -9225,7 +9225,7 @@
         <v>20</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>689</v>
+        <v>678</v>
       </c>
       <c r="E37" s="4" t="s">
         <v>485</v>
@@ -9242,7 +9242,7 @@
         <v>16</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>690</v>
+        <v>679</v>
       </c>
       <c r="E38" s="4" t="s">
         <v>529</v>
@@ -9259,7 +9259,7 @@
         <v>17</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>691</v>
+        <v>680</v>
       </c>
       <c r="E39" s="4" t="s">
         <v>529</v>
@@ -9276,7 +9276,7 @@
         <v>18</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>692</v>
+        <v>681</v>
       </c>
       <c r="E40" s="4" t="s">
         <v>529</v>
@@ -9293,7 +9293,7 @@
         <v>19</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>693</v>
+        <v>682</v>
       </c>
       <c r="E41" s="4" t="s">
         <v>529</v>
@@ -9310,7 +9310,7 @@
         <v>20</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>694</v>
+        <v>683</v>
       </c>
       <c r="E42" s="4" t="s">
         <v>529</v>
@@ -9327,7 +9327,7 @@
         <v>16</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>695</v>
+        <v>684</v>
       </c>
       <c r="E43" s="4" t="s">
         <v>539</v>
@@ -9344,7 +9344,7 @@
         <v>17</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>696</v>
+        <v>685</v>
       </c>
       <c r="E44" s="4" t="s">
         <v>539</v>
@@ -9361,7 +9361,7 @@
         <v>18</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>697</v>
+        <v>686</v>
       </c>
       <c r="E45" s="4" t="s">
         <v>539</v>
@@ -9378,7 +9378,7 @@
         <v>19</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>698</v>
+        <v>687</v>
       </c>
       <c r="E46" s="4" t="s">
         <v>539</v>
@@ -9395,7 +9395,7 @@
         <v>20</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>699</v>
+        <v>688</v>
       </c>
       <c r="E47" s="4" t="s">
         <v>539</v>
@@ -9412,7 +9412,7 @@
         <v>16</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>700</v>
+        <v>689</v>
       </c>
       <c r="E48" s="4" t="s">
         <v>564</v>
@@ -9429,7 +9429,7 @@
         <v>17</v>
       </c>
       <c r="D49" s="4" t="s">
-        <v>701</v>
+        <v>690</v>
       </c>
       <c r="E49" s="4" t="s">
         <v>564</v>
@@ -9446,7 +9446,7 @@
         <v>18</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>702</v>
+        <v>691</v>
       </c>
       <c r="E50" s="4" t="s">
         <v>564</v>
@@ -9463,7 +9463,7 @@
         <v>19</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>703</v>
+        <v>692</v>
       </c>
       <c r="E51" s="4" t="s">
         <v>564</v>
@@ -9480,7 +9480,7 @@
         <v>20</v>
       </c>
       <c r="D52" s="4" t="s">
-        <v>704</v>
+        <v>693</v>
       </c>
       <c r="E52" s="4" t="s">
         <v>564</v>
@@ -9497,10 +9497,10 @@
         <v>16</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>705</v>
+        <v>694</v>
       </c>
       <c r="E53" s="4" t="s">
-        <v>630</v>
+        <v>619</v>
       </c>
     </row>
     <row r="54" spans="1:5">
@@ -9514,10 +9514,10 @@
         <v>17</v>
       </c>
       <c r="D54" s="4" t="s">
-        <v>706</v>
+        <v>695</v>
       </c>
       <c r="E54" s="4" t="s">
-        <v>630</v>
+        <v>619</v>
       </c>
     </row>
     <row r="55" spans="1:5">
@@ -9531,10 +9531,10 @@
         <v>18</v>
       </c>
       <c r="D55" s="4" t="s">
-        <v>707</v>
+        <v>696</v>
       </c>
       <c r="E55" s="4" t="s">
-        <v>630</v>
+        <v>619</v>
       </c>
     </row>
     <row r="56" spans="1:5">
@@ -9548,10 +9548,10 @@
         <v>19</v>
       </c>
       <c r="D56" s="4" t="s">
-        <v>708</v>
+        <v>697</v>
       </c>
       <c r="E56" s="4" t="s">
-        <v>630</v>
+        <v>619</v>
       </c>
     </row>
     <row r="57" spans="1:5">
@@ -9565,15 +9565,15 @@
         <v>20</v>
       </c>
       <c r="D57" s="4" t="s">
-        <v>709</v>
+        <v>698</v>
       </c>
       <c r="E57" s="4" t="s">
-        <v>630</v>
+        <v>619</v>
       </c>
     </row>
     <row r="58" spans="1:5">
       <c r="A58" s="5" t="s">
-        <v>710</v>
+        <v>699</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
testing to fine NaN
</commit_message>
<xml_diff>
--- a/data-raw/data.default.xlsx
+++ b/data-raw/data.default.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Forrester\Models\3-PG\r3PG_mortality_management_defoliation - Copy before adding crown_width_option_baseline_to_start5\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96C9E117-6C3D-4F4D-8756-7E3AE82304A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B729FDBE-40D5-4AB8-BF7E-C7D5E73B80E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{61EEFE5B-6AE1-A641-A9AB-273DC4213F59}"/>
+    <workbookView xWindow="8730" yWindow="3435" windowWidth="19125" windowHeight="11235" activeTab="2" xr2:uid="{61EEFE5B-6AE1-A641-A9AB-273DC4213F59}"/>
   </bookViews>
   <sheets>
     <sheet name="parameters" sheetId="8" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1240" uniqueCount="722">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1240" uniqueCount="719">
   <si>
     <t>pFS2</t>
   </si>
@@ -2172,24 +2172,6 @@
     <t>var_10_8</t>
   </si>
   <si>
-    <t>var_10_9</t>
-  </si>
-  <si>
-    <t>var_10_10</t>
-  </si>
-  <si>
-    <t>var_10_11</t>
-  </si>
-  <si>
-    <t>var_10_12</t>
-  </si>
-  <si>
-    <t>var_10_13</t>
-  </si>
-  <si>
-    <t>var_10_14</t>
-  </si>
-  <si>
     <t>biom_incr_foliage_def</t>
   </si>
   <si>
@@ -2197,13 +2179,22 @@
   </si>
   <si>
     <t>Increment due to use of non-structural carbohydrates following defoliation</t>
+  </si>
+  <si>
+    <t>prop_carbs</t>
+  </si>
+  <si>
+    <t>biom_foliage_adj_pre_def</t>
+  </si>
+  <si>
+    <t>growing_season_length</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -2247,6 +2238,13 @@
       <name val="Lucida Grande"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -2275,7 +2273,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -2283,6 +2281,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5586,13 +5585,13 @@
         <v>12</v>
       </c>
       <c r="C73" t="s">
-        <v>719</v>
+        <v>713</v>
       </c>
       <c r="D73" t="s">
         <v>334</v>
       </c>
       <c r="E73" t="s">
-        <v>721</v>
+        <v>715</v>
       </c>
       <c r="F73" t="s">
         <v>336</v>
@@ -5606,13 +5605,13 @@
         <v>13</v>
       </c>
       <c r="C74" t="s">
-        <v>720</v>
+        <v>714</v>
       </c>
       <c r="D74" t="s">
         <v>334</v>
       </c>
       <c r="E74" t="s">
-        <v>721</v>
+        <v>715</v>
       </c>
       <c r="F74" t="s">
         <v>336</v>
@@ -7724,8 +7723,8 @@
       <c r="B190">
         <v>9</v>
       </c>
-      <c r="C190" s="1" t="s">
-        <v>713</v>
+      <c r="C190" s="7" t="s">
+        <v>716</v>
       </c>
       <c r="D190" t="s">
         <v>532</v>
@@ -7747,8 +7746,8 @@
       <c r="B191">
         <v>10</v>
       </c>
-      <c r="C191" s="1" t="s">
-        <v>714</v>
+      <c r="C191" s="7" t="s">
+        <v>717</v>
       </c>
       <c r="D191" t="s">
         <v>532</v>
@@ -7770,8 +7769,8 @@
       <c r="B192">
         <v>11</v>
       </c>
-      <c r="C192" s="1" t="s">
-        <v>715</v>
+      <c r="C192" s="7" t="s">
+        <v>683</v>
       </c>
       <c r="D192" t="s">
         <v>532</v>
@@ -7793,8 +7792,8 @@
       <c r="B193">
         <v>12</v>
       </c>
-      <c r="C193" s="1" t="s">
-        <v>716</v>
+      <c r="C193" s="7" t="s">
+        <v>718</v>
       </c>
       <c r="D193" t="s">
         <v>532</v>
@@ -7816,8 +7815,8 @@
       <c r="B194">
         <v>13</v>
       </c>
-      <c r="C194" s="1" t="s">
-        <v>717</v>
+      <c r="C194" s="7" t="s">
+        <v>436</v>
       </c>
       <c r="D194" t="s">
         <v>532</v>
@@ -7839,8 +7838,8 @@
       <c r="B195">
         <v>14</v>
       </c>
-      <c r="C195" s="1" t="s">
-        <v>718</v>
+      <c r="C195" s="7" t="s">
+        <v>445</v>
       </c>
       <c r="D195" t="s">
         <v>532</v>

</xml_diff>

<commit_message>
adding the third self-thinning option
</commit_message>
<xml_diff>
--- a/data-raw/data.default.xlsx
+++ b/data-raw/data.default.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Forrester\Models\3-PG\r3PG_mortality_management_defoliation - Copy before adding crown_width_option_baseline_to_start8\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0832C5C5-BCD6-4ED4-91FB-204AED1F0736}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A20CA1E-2584-452A-B5C8-D6DB4FE5F73B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{61EEFE5B-6AE1-A641-A9AB-273DC4213F59}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1236" uniqueCount="718">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1258" uniqueCount="728">
   <si>
     <t>pFS2</t>
   </si>
@@ -2185,6 +2185,36 @@
   </si>
   <si>
     <t>Intercept for self-thinning rule when mort_model = 2</t>
+  </si>
+  <si>
+    <t>ln(trees ha-1)</t>
+  </si>
+  <si>
+    <t>beta0</t>
+  </si>
+  <si>
+    <t>constant for self-thinning when mort_model = 2</t>
+  </si>
+  <si>
+    <t>betaB</t>
+  </si>
+  <si>
+    <t>Power for B when mort_model = 2</t>
+  </si>
+  <si>
+    <t>betaN</t>
+  </si>
+  <si>
+    <t>Power in tree density when mort_model = 2</t>
+  </si>
+  <si>
+    <t>betafN</t>
+  </si>
+  <si>
+    <t>betafT</t>
+  </si>
+  <si>
+    <t>betafPhys</t>
   </si>
 </sst>
 </file>
@@ -2586,7 +2616,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E287297-02C0-BF44-BF0C-8FADE2A87F8F}">
-  <dimension ref="A1:D91"/>
+  <dimension ref="A1:D97"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
   <cols>
     <col min="2" max="2" width="80" bestFit="1" customWidth="1"/>
@@ -3061,7 +3091,9 @@
       <c r="B34" s="1" t="s">
         <v>717</v>
       </c>
-      <c r="C34" s="1"/>
+      <c r="C34" s="1" t="s">
+        <v>718</v>
+      </c>
       <c r="D34" s="1">
         <v>12</v>
       </c>
@@ -3073,7 +3105,9 @@
       <c r="B35" s="1" t="s">
         <v>565</v>
       </c>
-      <c r="C35" s="1"/>
+      <c r="C35" s="1" t="s">
+        <v>103</v>
+      </c>
       <c r="D35" s="1">
         <v>0</v>
       </c>
@@ -3085,7 +3119,9 @@
       <c r="B36" s="1" t="s">
         <v>566</v>
       </c>
-      <c r="C36" s="1"/>
+      <c r="C36" s="1" t="s">
+        <v>103</v>
+      </c>
       <c r="D36" s="1">
         <v>0</v>
       </c>
@@ -3097,533 +3133,535 @@
       <c r="B37" s="1" t="s">
         <v>567</v>
       </c>
-      <c r="C37" s="1"/>
+      <c r="C37" s="1" t="s">
+        <v>103</v>
+      </c>
       <c r="D37" s="1">
         <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:4">
-      <c r="A38" t="s">
-        <v>33</v>
-      </c>
-      <c r="B38" t="s">
-        <v>141</v>
-      </c>
-      <c r="C38" t="s">
-        <v>103</v>
-      </c>
-      <c r="D38">
+      <c r="A38" s="1" t="s">
+        <v>719</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>720</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="D38" s="1">
+        <v>-20.399999999999999</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4">
+      <c r="A39" s="1" t="s">
+        <v>721</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>722</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="D39" s="1">
+        <v>1.86</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4">
+      <c r="A40" s="1" t="s">
+        <v>723</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>724</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="D40" s="1">
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4">
+      <c r="A41" s="1" t="s">
+        <v>725</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>565</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="D41" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:4">
-      <c r="A39" t="s">
-        <v>34</v>
-      </c>
-      <c r="B39" t="s">
-        <v>142</v>
-      </c>
-      <c r="C39" t="s">
-        <v>103</v>
-      </c>
-      <c r="D39">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4">
-      <c r="A40" t="s">
-        <v>35</v>
-      </c>
-      <c r="B40" t="s">
-        <v>143</v>
-      </c>
-      <c r="C40" t="s">
-        <v>103</v>
-      </c>
-      <c r="D40">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4">
-      <c r="A41" t="s">
-        <v>36</v>
-      </c>
-      <c r="B41" t="s">
-        <v>144</v>
-      </c>
-      <c r="C41" t="s">
-        <v>145</v>
-      </c>
-      <c r="D41">
-        <v>11</v>
-      </c>
-    </row>
     <row r="42" spans="1:4">
-      <c r="A42" t="s">
-        <v>37</v>
-      </c>
-      <c r="B42" t="s">
-        <v>146</v>
-      </c>
-      <c r="C42" t="s">
-        <v>145</v>
-      </c>
-      <c r="D42">
-        <v>4</v>
+      <c r="A42" s="1" t="s">
+        <v>726</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>566</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="D42" s="1">
+        <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:4">
-      <c r="A43" t="s">
-        <v>38</v>
-      </c>
-      <c r="B43" t="s">
-        <v>147</v>
-      </c>
-      <c r="C43" t="s">
-        <v>130</v>
-      </c>
-      <c r="D43">
-        <v>2.5</v>
+      <c r="A43" s="1" t="s">
+        <v>727</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="D43" s="1">
+        <v>0</v>
       </c>
     </row>
     <row r="44" spans="1:4">
       <c r="A44" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="B44" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="C44" t="s">
         <v>103</v>
       </c>
       <c r="D44">
-        <v>0.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45" spans="1:4">
-      <c r="A45" s="1" t="s">
-        <v>669</v>
-      </c>
-      <c r="B45" s="1" t="s">
-        <v>670</v>
-      </c>
-      <c r="C45" s="1"/>
-      <c r="D45" s="1">
-        <v>0</v>
+      <c r="A45" t="s">
+        <v>34</v>
+      </c>
+      <c r="B45" t="s">
+        <v>142</v>
+      </c>
+      <c r="C45" t="s">
+        <v>103</v>
+      </c>
+      <c r="D45">
+        <v>0.2</v>
       </c>
     </row>
     <row r="46" spans="1:4">
       <c r="A46" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="B46" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="C46" t="s">
-        <v>130</v>
+        <v>103</v>
       </c>
       <c r="D46">
-        <v>3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="47" spans="1:4">
       <c r="A47" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="B47" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="C47" t="s">
-        <v>103</v>
+        <v>145</v>
       </c>
       <c r="D47">
-        <v>0.15</v>
+        <v>11</v>
       </c>
     </row>
     <row r="48" spans="1:4">
       <c r="A48" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="B48" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="C48" t="s">
-        <v>103</v>
+        <v>145</v>
       </c>
       <c r="D48">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="49" spans="1:4">
       <c r="A49" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B49" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="C49" t="s">
-        <v>103</v>
+        <v>130</v>
       </c>
       <c r="D49">
-        <v>5</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="50" spans="1:4">
       <c r="A50" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="B50" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="C50" t="s">
-        <v>154</v>
+        <v>103</v>
       </c>
       <c r="D50">
-        <v>0.06</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="51" spans="1:4">
-      <c r="A51" t="s">
-        <v>45</v>
-      </c>
-      <c r="B51" t="s">
-        <v>155</v>
-      </c>
-      <c r="C51" t="s">
-        <v>103</v>
-      </c>
-      <c r="D51">
-        <v>0.47</v>
+      <c r="A51" s="1" t="s">
+        <v>669</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>670</v>
+      </c>
+      <c r="C51" s="1"/>
+      <c r="D51" s="1">
+        <v>0</v>
       </c>
     </row>
     <row r="52" spans="1:4">
       <c r="A52" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="B52" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="C52" t="s">
-        <v>157</v>
+        <v>130</v>
       </c>
       <c r="D52">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="53" spans="1:4">
       <c r="A53" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="B53" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="C53" t="s">
-        <v>157</v>
+        <v>103</v>
       </c>
       <c r="D53">
-        <v>0.02</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="54" spans="1:4">
       <c r="A54" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="B54" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="C54" t="s">
         <v>103</v>
       </c>
       <c r="D54">
-        <v>3.33</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55" spans="1:4">
       <c r="A55" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="B55" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="C55" t="s">
-        <v>161</v>
+        <v>103</v>
       </c>
       <c r="D55">
-        <v>0.05</v>
+        <v>5</v>
       </c>
     </row>
     <row r="56" spans="1:4">
       <c r="A56" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="B56" t="s">
-        <v>162</v>
+        <v>153</v>
       </c>
       <c r="C56" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="D56">
-        <v>0.2</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="57" spans="1:4">
       <c r="A57" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="B57" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="C57" t="s">
         <v>103</v>
       </c>
       <c r="D57">
-        <v>0.66</v>
+        <v>0.47</v>
       </c>
     </row>
     <row r="58" spans="1:4">
       <c r="A58" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="B58" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="C58" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="D58">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="59" spans="1:4">
       <c r="A59" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="B59" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="C59" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="D59">
-        <v>4.4000000000000004</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="60" spans="1:4">
       <c r="A60" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="B60" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="C60" t="s">
-        <v>165</v>
+        <v>103</v>
       </c>
       <c r="D60">
-        <v>27</v>
+        <v>3.33</v>
       </c>
     </row>
     <row r="61" spans="1:4">
       <c r="A61" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="B61" t="s">
-        <v>168</v>
+        <v>160</v>
       </c>
       <c r="C61" t="s">
-        <v>103</v>
+        <v>161</v>
       </c>
       <c r="D61">
-        <v>0.75</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="62" spans="1:4">
       <c r="A62" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="B62" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="C62" t="s">
-        <v>103</v>
+        <v>157</v>
       </c>
       <c r="D62">
-        <v>0.15</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="63" spans="1:4">
       <c r="A63" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="B63" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="C63" t="s">
-        <v>130</v>
+        <v>103</v>
       </c>
       <c r="D63">
-        <v>2</v>
+        <v>0.66</v>
       </c>
     </row>
     <row r="64" spans="1:4">
       <c r="A64" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="B64" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="C64" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="D64">
-        <v>0.45</v>
+        <v>2</v>
       </c>
     </row>
     <row r="65" spans="1:4">
       <c r="A65" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B65" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="C65" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="D65">
-        <v>0.45</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="66" spans="1:4">
       <c r="A66" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="B66" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="C66" t="s">
-        <v>130</v>
+        <v>165</v>
       </c>
       <c r="D66">
-        <v>4</v>
+        <v>27</v>
       </c>
     </row>
     <row r="67" spans="1:4">
       <c r="A67" t="s">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="B67" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="C67" t="s">
         <v>103</v>
       </c>
       <c r="D67">
-        <v>3</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="68" spans="1:4">
-      <c r="A68" s="1" t="s">
-        <v>667</v>
-      </c>
-      <c r="B68" s="1" t="s">
-        <v>668</v>
-      </c>
-      <c r="C68" s="1" t="s">
-        <v>266</v>
-      </c>
-      <c r="D68" s="1">
-        <v>1.3</v>
+      <c r="A68" t="s">
+        <v>56</v>
+      </c>
+      <c r="B68" t="s">
+        <v>169</v>
+      </c>
+      <c r="C68" t="s">
+        <v>103</v>
+      </c>
+      <c r="D68">
+        <v>0.15</v>
       </c>
     </row>
     <row r="69" spans="1:4">
       <c r="A69" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="B69" t="s">
-        <v>696</v>
+        <v>170</v>
       </c>
       <c r="C69" t="s">
-        <v>103</v>
+        <v>130</v>
       </c>
       <c r="D69">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="70" spans="1:4">
       <c r="A70" t="s">
-        <v>684</v>
+        <v>58</v>
       </c>
       <c r="B70" t="s">
-        <v>696</v>
+        <v>171</v>
       </c>
       <c r="C70" t="s">
-        <v>103</v>
+        <v>172</v>
       </c>
       <c r="D70">
-        <v>0</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="71" spans="1:4">
       <c r="A71" t="s">
-        <v>685</v>
+        <v>59</v>
       </c>
       <c r="B71" t="s">
-        <v>696</v>
+        <v>173</v>
       </c>
       <c r="C71" t="s">
-        <v>103</v>
+        <v>172</v>
       </c>
       <c r="D71">
-        <v>0</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="72" spans="1:4">
       <c r="A72" t="s">
-        <v>694</v>
+        <v>60</v>
       </c>
       <c r="B72" t="s">
-        <v>696</v>
+        <v>174</v>
       </c>
       <c r="C72" t="s">
-        <v>103</v>
+        <v>130</v>
       </c>
       <c r="D72">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="73" spans="1:4">
       <c r="A73" t="s">
-        <v>695</v>
+        <v>66</v>
       </c>
       <c r="B73" t="s">
-        <v>696</v>
+        <v>175</v>
       </c>
       <c r="C73" t="s">
         <v>103</v>
       </c>
       <c r="D73">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="74" spans="1:4">
-      <c r="A74" t="s">
-        <v>62</v>
-      </c>
-      <c r="B74" t="s">
-        <v>176</v>
-      </c>
-      <c r="C74" t="s">
-        <v>103</v>
-      </c>
-      <c r="D74">
-        <v>0</v>
+      <c r="A74" s="1" t="s">
+        <v>667</v>
+      </c>
+      <c r="B74" s="1" t="s">
+        <v>668</v>
+      </c>
+      <c r="C74" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="D74" s="1">
+        <v>1.3</v>
       </c>
     </row>
     <row r="75" spans="1:4">
       <c r="A75" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B75" t="s">
-        <v>177</v>
+        <v>696</v>
       </c>
       <c r="C75" t="s">
         <v>103</v>
@@ -3634,10 +3672,10 @@
     </row>
     <row r="76" spans="1:4">
       <c r="A76" t="s">
-        <v>64</v>
+        <v>684</v>
       </c>
       <c r="B76" t="s">
-        <v>178</v>
+        <v>696</v>
       </c>
       <c r="C76" t="s">
         <v>103</v>
@@ -3648,10 +3686,10 @@
     </row>
     <row r="77" spans="1:4">
       <c r="A77" t="s">
-        <v>65</v>
+        <v>685</v>
       </c>
       <c r="B77" t="s">
-        <v>179</v>
+        <v>696</v>
       </c>
       <c r="C77" t="s">
         <v>103</v>
@@ -3662,10 +3700,10 @@
     </row>
     <row r="78" spans="1:4">
       <c r="A78" t="s">
-        <v>67</v>
+        <v>694</v>
       </c>
       <c r="B78" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="C78" t="s">
         <v>103</v>
@@ -3676,10 +3714,10 @@
     </row>
     <row r="79" spans="1:4">
       <c r="A79" t="s">
-        <v>686</v>
+        <v>695</v>
       </c>
       <c r="B79" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="C79" t="s">
         <v>103</v>
@@ -3690,10 +3728,10 @@
     </row>
     <row r="80" spans="1:4">
       <c r="A80" t="s">
-        <v>687</v>
+        <v>62</v>
       </c>
       <c r="B80" t="s">
-        <v>697</v>
+        <v>176</v>
       </c>
       <c r="C80" t="s">
         <v>103</v>
@@ -3704,10 +3742,10 @@
     </row>
     <row r="81" spans="1:4">
       <c r="A81" t="s">
-        <v>688</v>
+        <v>63</v>
       </c>
       <c r="B81" t="s">
-        <v>697</v>
+        <v>177</v>
       </c>
       <c r="C81" t="s">
         <v>103</v>
@@ -3718,10 +3756,10 @@
     </row>
     <row r="82" spans="1:4">
       <c r="A82" t="s">
-        <v>689</v>
+        <v>64</v>
       </c>
       <c r="B82" t="s">
-        <v>697</v>
+        <v>178</v>
       </c>
       <c r="C82" t="s">
         <v>103</v>
@@ -3732,10 +3770,10 @@
     </row>
     <row r="83" spans="1:4">
       <c r="A83" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B83" t="s">
-        <v>698</v>
+        <v>179</v>
       </c>
       <c r="C83" t="s">
         <v>103</v>
@@ -3746,10 +3784,10 @@
     </row>
     <row r="84" spans="1:4">
       <c r="A84" t="s">
-        <v>690</v>
+        <v>67</v>
       </c>
       <c r="B84" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="C84" t="s">
         <v>103</v>
@@ -3760,10 +3798,10 @@
     </row>
     <row r="85" spans="1:4">
       <c r="A85" t="s">
-        <v>691</v>
+        <v>686</v>
       </c>
       <c r="B85" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="C85" t="s">
         <v>103</v>
@@ -3774,10 +3812,10 @@
     </row>
     <row r="86" spans="1:4">
       <c r="A86" t="s">
-        <v>692</v>
+        <v>687</v>
       </c>
       <c r="B86" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="C86" t="s">
         <v>103</v>
@@ -3788,10 +3826,10 @@
     </row>
     <row r="87" spans="1:4">
       <c r="A87" t="s">
-        <v>693</v>
+        <v>688</v>
       </c>
       <c r="B87" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="C87" t="s">
         <v>103</v>
@@ -3802,57 +3840,141 @@
     </row>
     <row r="88" spans="1:4">
       <c r="A88" t="s">
-        <v>84</v>
+        <v>689</v>
       </c>
       <c r="B88" t="s">
-        <v>180</v>
+        <v>697</v>
       </c>
       <c r="C88" t="s">
-        <v>181</v>
+        <v>103</v>
       </c>
       <c r="D88">
-        <v>-90</v>
+        <v>0</v>
       </c>
     </row>
     <row r="89" spans="1:4">
       <c r="A89" t="s">
-        <v>85</v>
+        <v>68</v>
       </c>
       <c r="B89" t="s">
-        <v>182</v>
+        <v>698</v>
       </c>
       <c r="C89" t="s">
         <v>103</v>
       </c>
       <c r="D89">
-        <v>0.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="90" spans="1:4">
       <c r="A90" t="s">
-        <v>86</v>
+        <v>690</v>
       </c>
       <c r="B90" t="s">
-        <v>183</v>
+        <v>698</v>
       </c>
       <c r="C90" t="s">
-        <v>184</v>
+        <v>103</v>
       </c>
       <c r="D90">
-        <v>24</v>
+        <v>0</v>
       </c>
     </row>
     <row r="91" spans="1:4">
       <c r="A91" t="s">
+        <v>691</v>
+      </c>
+      <c r="B91" t="s">
+        <v>698</v>
+      </c>
+      <c r="C91" t="s">
+        <v>103</v>
+      </c>
+      <c r="D91">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4">
+      <c r="A92" t="s">
+        <v>692</v>
+      </c>
+      <c r="B92" t="s">
+        <v>698</v>
+      </c>
+      <c r="C92" t="s">
+        <v>103</v>
+      </c>
+      <c r="D92">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4">
+      <c r="A93" t="s">
+        <v>693</v>
+      </c>
+      <c r="B93" t="s">
+        <v>698</v>
+      </c>
+      <c r="C93" t="s">
+        <v>103</v>
+      </c>
+      <c r="D93">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4">
+      <c r="A94" t="s">
+        <v>84</v>
+      </c>
+      <c r="B94" t="s">
+        <v>180</v>
+      </c>
+      <c r="C94" t="s">
+        <v>181</v>
+      </c>
+      <c r="D94">
+        <v>-90</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4">
+      <c r="A95" t="s">
+        <v>85</v>
+      </c>
+      <c r="B95" t="s">
+        <v>182</v>
+      </c>
+      <c r="C95" t="s">
+        <v>103</v>
+      </c>
+      <c r="D95">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4">
+      <c r="A96" t="s">
+        <v>86</v>
+      </c>
+      <c r="B96" t="s">
+        <v>183</v>
+      </c>
+      <c r="C96" t="s">
+        <v>184</v>
+      </c>
+      <c r="D96">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4">
+      <c r="A97" t="s">
         <v>87</v>
       </c>
-      <c r="B91" t="s">
+      <c r="B97" t="s">
         <v>185</v>
       </c>
-      <c r="C91" t="s">
+      <c r="C97" t="s">
         <v>186</v>
       </c>
-      <c r="D91">
+      <c r="D97">
         <v>2.2999999999999998</v>
       </c>
     </row>

</xml_diff>

<commit_message>
removed n_sp dimensions from self-thinning options 2 and 3
</commit_message>
<xml_diff>
--- a/data-raw/data.default.xlsx
+++ b/data-raw/data.default.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Forrester\Models\3-PG\r3PG_mortality_management_defoliation - Copy before adding crown_width_option_baseline_to_start8\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EE52741-CD98-414D-93C6-C8D1C4FB94AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB8E2B3C-CCD8-482F-99F8-2F8352F296FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{61EEFE5B-6AE1-A641-A9AB-273DC4213F59}"/>
   </bookViews>
@@ -21,17 +21,28 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">output!$A$1:$G$221</definedName>
   </definedNames>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1258" uniqueCount="731">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1228" uniqueCount="710">
   <si>
     <t>pFS2</t>
   </si>
@@ -2154,73 +2165,10 @@
     <t>var_10_14</t>
   </si>
   <si>
-    <t>thinIntercept</t>
-  </si>
-  <si>
-    <t>thinfN</t>
-  </si>
-  <si>
-    <t>thinfT</t>
-  </si>
-  <si>
-    <t>thinfPhys</t>
-  </si>
-  <si>
-    <t>ln(trees ha-1)</t>
-  </si>
-  <si>
-    <t>beta0</t>
-  </si>
-  <si>
-    <t>betaB</t>
-  </si>
-  <si>
-    <t>betaN</t>
-  </si>
-  <si>
-    <t>betafN</t>
-  </si>
-  <si>
-    <t>betafT</t>
-  </si>
-  <si>
-    <t>betafPhys</t>
-  </si>
-  <si>
     <t>Maximum stem mass per tree @ N = 1000 trees/hectare (mort_model = 1)</t>
   </si>
   <si>
     <t>Power in self-thinning rule (mort_model = 1 or 2)</t>
-  </si>
-  <si>
-    <t>Intercept for self-thinning rule (mort_model = 2)</t>
-  </si>
-  <si>
-    <t>Power in fertility modifier (mort_model = 2)</t>
-  </si>
-  <si>
-    <t>Power in temperature modifier (mort_model = 2)</t>
-  </si>
-  <si>
-    <t>Power in physmod modifier (mort_model = 2)</t>
-  </si>
-  <si>
-    <t>constant for self-thinning (mort_model = 3)</t>
-  </si>
-  <si>
-    <t>Power for B (mort_model = 3)</t>
-  </si>
-  <si>
-    <t>Power in tree density (mort_model = 3)</t>
-  </si>
-  <si>
-    <t>Power in nutrition modifier (mort_model = 3)</t>
-  </si>
-  <si>
-    <t>Power in temperature modifier (mort_model = 3)</t>
-  </si>
-  <si>
-    <t>Power in physmod modifier (mort_model = 3)</t>
   </si>
   <si>
     <t>Parameter of crown ratio equation</t>
@@ -2625,7 +2573,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E287297-02C0-BF44-BF0C-8FADE2A87F8F}">
-  <dimension ref="A1:D97"/>
+  <dimension ref="A1:D87"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
   <cols>
     <col min="2" max="2" width="80" bestFit="1" customWidth="1"/>
@@ -3070,7 +3018,7 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>718</v>
+        <v>707</v>
       </c>
       <c r="C32" t="s">
         <v>138</v>
@@ -3084,7 +3032,7 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>719</v>
+        <v>708</v>
       </c>
       <c r="C33" t="s">
         <v>103</v>
@@ -3094,151 +3042,149 @@
       </c>
     </row>
     <row r="34" spans="1:4">
-      <c r="A34" s="1" t="s">
-        <v>707</v>
+      <c r="A34" t="s">
+        <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>720</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>711</v>
-      </c>
-      <c r="D34" s="1">
-        <v>12</v>
+        <v>139</v>
+      </c>
+      <c r="C34" t="s">
+        <v>103</v>
+      </c>
+      <c r="D34">
+        <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:4">
-      <c r="A35" s="1" t="s">
-        <v>708</v>
+      <c r="A35" t="s">
+        <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>721</v>
-      </c>
-      <c r="C35" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="C35" t="s">
         <v>103</v>
       </c>
-      <c r="D35" s="1">
-        <v>0</v>
+      <c r="D35">
+        <v>0.2</v>
       </c>
     </row>
     <row r="36" spans="1:4">
-      <c r="A36" s="1" t="s">
-        <v>709</v>
+      <c r="A36" t="s">
+        <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>722</v>
-      </c>
-      <c r="C36" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="C36" t="s">
         <v>103</v>
       </c>
-      <c r="D36" s="1">
-        <v>0</v>
+      <c r="D36">
+        <v>0.2</v>
       </c>
     </row>
     <row r="37" spans="1:4">
-      <c r="A37" s="1" t="s">
-        <v>710</v>
+      <c r="A37" t="s">
+        <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>723</v>
-      </c>
-      <c r="C37" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="C37" t="s">
+        <v>143</v>
+      </c>
+      <c r="D37">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4">
+      <c r="A38" t="s">
+        <v>37</v>
+      </c>
+      <c r="B38" t="s">
+        <v>144</v>
+      </c>
+      <c r="C38" t="s">
+        <v>143</v>
+      </c>
+      <c r="D38">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4">
+      <c r="A39" t="s">
+        <v>38</v>
+      </c>
+      <c r="B39" t="s">
+        <v>145</v>
+      </c>
+      <c r="C39" t="s">
+        <v>130</v>
+      </c>
+      <c r="D39">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4">
+      <c r="A40" t="s">
+        <v>39</v>
+      </c>
+      <c r="B40" t="s">
+        <v>146</v>
+      </c>
+      <c r="C40" t="s">
         <v>103</v>
       </c>
-      <c r="D37" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4">
-      <c r="A38" s="1" t="s">
-        <v>712</v>
-      </c>
-      <c r="B38" t="s">
-        <v>724</v>
-      </c>
-      <c r="C38" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="D38" s="1">
-        <v>-20.399999999999999</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4">
-      <c r="A39" s="1" t="s">
-        <v>713</v>
-      </c>
-      <c r="B39" t="s">
-        <v>725</v>
-      </c>
-      <c r="C39" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="D39" s="1">
-        <v>1.86</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4">
-      <c r="A40" s="1" t="s">
-        <v>714</v>
-      </c>
-      <c r="B40" t="s">
-        <v>726</v>
-      </c>
-      <c r="C40" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="D40" s="1">
-        <v>2.6</v>
+      <c r="D40">
+        <v>0.5</v>
       </c>
     </row>
     <row r="41" spans="1:4">
       <c r="A41" s="1" t="s">
-        <v>715</v>
-      </c>
-      <c r="B41" t="s">
-        <v>727</v>
-      </c>
-      <c r="C41" s="1" t="s">
-        <v>103</v>
-      </c>
+        <v>664</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>665</v>
+      </c>
+      <c r="C41" s="1"/>
       <c r="D41" s="1">
         <v>0</v>
       </c>
     </row>
     <row r="42" spans="1:4">
-      <c r="A42" s="1" t="s">
-        <v>716</v>
+      <c r="A42" t="s">
+        <v>40</v>
       </c>
       <c r="B42" t="s">
-        <v>728</v>
-      </c>
-      <c r="C42" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="C42" t="s">
+        <v>130</v>
+      </c>
+      <c r="D42">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4">
+      <c r="A43" t="s">
+        <v>41</v>
+      </c>
+      <c r="B43" t="s">
+        <v>148</v>
+      </c>
+      <c r="C43" t="s">
         <v>103</v>
       </c>
-      <c r="D42" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4">
-      <c r="A43" s="1" t="s">
-        <v>717</v>
-      </c>
-      <c r="B43" t="s">
-        <v>729</v>
-      </c>
-      <c r="C43" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="D43" s="1">
-        <v>0</v>
+      <c r="D43">
+        <v>0.15</v>
       </c>
     </row>
     <row r="44" spans="1:4">
       <c r="A44" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="B44" t="s">
-        <v>139</v>
+        <v>149</v>
       </c>
       <c r="C44" t="s">
         <v>103</v>
@@ -3249,428 +3195,430 @@
     </row>
     <row r="45" spans="1:4">
       <c r="A45" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="B45" t="s">
-        <v>140</v>
+        <v>150</v>
       </c>
       <c r="C45" t="s">
         <v>103</v>
       </c>
       <c r="D45">
-        <v>0.2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="46" spans="1:4">
       <c r="A46" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="B46" t="s">
-        <v>141</v>
+        <v>151</v>
       </c>
       <c r="C46" t="s">
-        <v>103</v>
+        <v>152</v>
       </c>
       <c r="D46">
-        <v>0.2</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="47" spans="1:4">
       <c r="A47" t="s">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="B47" t="s">
-        <v>142</v>
+        <v>153</v>
       </c>
       <c r="C47" t="s">
-        <v>143</v>
+        <v>103</v>
       </c>
       <c r="D47">
-        <v>11</v>
+        <v>0.47</v>
       </c>
     </row>
     <row r="48" spans="1:4">
       <c r="A48" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="B48" t="s">
-        <v>144</v>
+        <v>154</v>
       </c>
       <c r="C48" t="s">
-        <v>143</v>
+        <v>155</v>
       </c>
       <c r="D48">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49" spans="1:4">
       <c r="A49" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="B49" t="s">
-        <v>145</v>
+        <v>156</v>
       </c>
       <c r="C49" t="s">
-        <v>130</v>
+        <v>155</v>
       </c>
       <c r="D49">
-        <v>2.5</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="50" spans="1:4">
       <c r="A50" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="B50" t="s">
-        <v>146</v>
+        <v>157</v>
       </c>
       <c r="C50" t="s">
         <v>103</v>
       </c>
       <c r="D50">
-        <v>0.5</v>
+        <v>3.33</v>
       </c>
     </row>
     <row r="51" spans="1:4">
-      <c r="A51" s="1" t="s">
-        <v>664</v>
-      </c>
-      <c r="B51" s="1" t="s">
-        <v>665</v>
-      </c>
-      <c r="C51" s="1"/>
-      <c r="D51" s="1">
-        <v>0</v>
+      <c r="A51" t="s">
+        <v>49</v>
+      </c>
+      <c r="B51" t="s">
+        <v>158</v>
+      </c>
+      <c r="C51" t="s">
+        <v>159</v>
+      </c>
+      <c r="D51">
+        <v>0.05</v>
       </c>
     </row>
     <row r="52" spans="1:4">
       <c r="A52" t="s">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="B52" t="s">
-        <v>147</v>
+        <v>160</v>
       </c>
       <c r="C52" t="s">
-        <v>130</v>
+        <v>155</v>
       </c>
       <c r="D52">
-        <v>3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="53" spans="1:4">
       <c r="A53" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="B53" t="s">
-        <v>148</v>
+        <v>161</v>
       </c>
       <c r="C53" t="s">
         <v>103</v>
       </c>
       <c r="D53">
-        <v>0.15</v>
+        <v>0.66</v>
       </c>
     </row>
     <row r="54" spans="1:4">
       <c r="A54" t="s">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="B54" t="s">
-        <v>149</v>
+        <v>162</v>
       </c>
       <c r="C54" t="s">
-        <v>103</v>
+        <v>163</v>
       </c>
       <c r="D54">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="55" spans="1:4">
       <c r="A55" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="B55" t="s">
-        <v>150</v>
+        <v>164</v>
       </c>
       <c r="C55" t="s">
-        <v>103</v>
+        <v>163</v>
       </c>
       <c r="D55">
-        <v>5</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="56" spans="1:4">
       <c r="A56" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="B56" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="C56" t="s">
-        <v>152</v>
+        <v>163</v>
       </c>
       <c r="D56">
-        <v>0.06</v>
+        <v>27</v>
       </c>
     </row>
     <row r="57" spans="1:4">
       <c r="A57" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="B57" t="s">
-        <v>153</v>
+        <v>166</v>
       </c>
       <c r="C57" t="s">
         <v>103</v>
       </c>
       <c r="D57">
-        <v>0.47</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="58" spans="1:4">
       <c r="A58" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="B58" t="s">
-        <v>154</v>
+        <v>167</v>
       </c>
       <c r="C58" t="s">
-        <v>155</v>
+        <v>103</v>
       </c>
       <c r="D58">
-        <v>0</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="59" spans="1:4">
       <c r="A59" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="B59" t="s">
-        <v>156</v>
+        <v>168</v>
       </c>
       <c r="C59" t="s">
-        <v>155</v>
+        <v>130</v>
       </c>
       <c r="D59">
-        <v>0.02</v>
+        <v>2</v>
       </c>
     </row>
     <row r="60" spans="1:4">
       <c r="A60" t="s">
-        <v>48</v>
+        <v>58</v>
       </c>
       <c r="B60" t="s">
-        <v>157</v>
+        <v>169</v>
       </c>
       <c r="C60" t="s">
-        <v>103</v>
+        <v>170</v>
       </c>
       <c r="D60">
-        <v>3.33</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="61" spans="1:4">
       <c r="A61" t="s">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="B61" t="s">
-        <v>158</v>
+        <v>171</v>
       </c>
       <c r="C61" t="s">
-        <v>159</v>
+        <v>170</v>
       </c>
       <c r="D61">
-        <v>0.05</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="62" spans="1:4">
       <c r="A62" t="s">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="B62" t="s">
-        <v>160</v>
+        <v>172</v>
       </c>
       <c r="C62" t="s">
-        <v>155</v>
+        <v>130</v>
       </c>
       <c r="D62">
-        <v>0.2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="63" spans="1:4">
       <c r="A63" t="s">
-        <v>51</v>
+        <v>66</v>
       </c>
       <c r="B63" t="s">
-        <v>161</v>
+        <v>173</v>
       </c>
       <c r="C63" t="s">
         <v>103</v>
       </c>
       <c r="D63">
-        <v>0.66</v>
+        <v>3</v>
       </c>
     </row>
     <row r="64" spans="1:4">
-      <c r="A64" t="s">
-        <v>52</v>
-      </c>
-      <c r="B64" t="s">
-        <v>162</v>
-      </c>
-      <c r="C64" t="s">
-        <v>163</v>
-      </c>
-      <c r="D64">
-        <v>2</v>
+      <c r="A64" s="1" t="s">
+        <v>662</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>663</v>
+      </c>
+      <c r="C64" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="D64" s="1">
+        <v>1.3</v>
       </c>
     </row>
     <row r="65" spans="1:4">
       <c r="A65" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="B65" t="s">
-        <v>164</v>
+        <v>691</v>
       </c>
       <c r="C65" t="s">
-        <v>163</v>
+        <v>103</v>
       </c>
       <c r="D65">
-        <v>4.4000000000000004</v>
+        <v>0</v>
       </c>
     </row>
     <row r="66" spans="1:4">
       <c r="A66" t="s">
-        <v>54</v>
+        <v>679</v>
       </c>
       <c r="B66" t="s">
-        <v>165</v>
+        <v>691</v>
       </c>
       <c r="C66" t="s">
-        <v>163</v>
+        <v>103</v>
       </c>
       <c r="D66">
-        <v>27</v>
+        <v>0</v>
       </c>
     </row>
     <row r="67" spans="1:4">
       <c r="A67" t="s">
-        <v>55</v>
+        <v>680</v>
       </c>
       <c r="B67" t="s">
-        <v>166</v>
+        <v>691</v>
       </c>
       <c r="C67" t="s">
         <v>103</v>
       </c>
       <c r="D67">
-        <v>0.75</v>
+        <v>0</v>
       </c>
     </row>
     <row r="68" spans="1:4">
       <c r="A68" t="s">
-        <v>56</v>
+        <v>689</v>
       </c>
       <c r="B68" t="s">
-        <v>167</v>
+        <v>691</v>
       </c>
       <c r="C68" t="s">
         <v>103</v>
       </c>
       <c r="D68">
-        <v>0.15</v>
+        <v>0</v>
       </c>
     </row>
     <row r="69" spans="1:4">
       <c r="A69" t="s">
-        <v>57</v>
+        <v>690</v>
       </c>
       <c r="B69" t="s">
-        <v>168</v>
+        <v>691</v>
       </c>
       <c r="C69" t="s">
-        <v>130</v>
+        <v>103</v>
       </c>
       <c r="D69">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="70" spans="1:4">
       <c r="A70" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B70" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="C70" t="s">
-        <v>170</v>
+        <v>103</v>
       </c>
       <c r="D70">
-        <v>0.45</v>
+        <v>0</v>
       </c>
     </row>
     <row r="71" spans="1:4">
       <c r="A71" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B71" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="C71" t="s">
-        <v>170</v>
+        <v>103</v>
       </c>
       <c r="D71">
-        <v>0.45</v>
+        <v>0</v>
       </c>
     </row>
     <row r="72" spans="1:4">
       <c r="A72" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="B72" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="C72" t="s">
-        <v>130</v>
+        <v>103</v>
       </c>
       <c r="D72">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="73" spans="1:4">
       <c r="A73" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B73" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="C73" t="s">
         <v>103</v>
       </c>
       <c r="D73">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="74" spans="1:4">
-      <c r="A74" s="1" t="s">
-        <v>662</v>
-      </c>
-      <c r="B74" s="1" t="s">
-        <v>663</v>
-      </c>
-      <c r="C74" s="1" t="s">
-        <v>264</v>
-      </c>
-      <c r="D74" s="1">
-        <v>1.3</v>
+      <c r="A74" t="s">
+        <v>67</v>
+      </c>
+      <c r="B74" t="s">
+        <v>692</v>
+      </c>
+      <c r="C74" t="s">
+        <v>103</v>
+      </c>
+      <c r="D74">
+        <v>0</v>
       </c>
     </row>
     <row r="75" spans="1:4">
       <c r="A75" t="s">
-        <v>61</v>
+        <v>681</v>
       </c>
       <c r="B75" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="C75" t="s">
         <v>103</v>
@@ -3681,10 +3629,10 @@
     </row>
     <row r="76" spans="1:4">
       <c r="A76" t="s">
-        <v>679</v>
+        <v>682</v>
       </c>
       <c r="B76" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="C76" t="s">
         <v>103</v>
@@ -3695,10 +3643,10 @@
     </row>
     <row r="77" spans="1:4">
       <c r="A77" t="s">
-        <v>680</v>
+        <v>683</v>
       </c>
       <c r="B77" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="C77" t="s">
         <v>103</v>
@@ -3709,10 +3657,10 @@
     </row>
     <row r="78" spans="1:4">
       <c r="A78" t="s">
-        <v>689</v>
+        <v>684</v>
       </c>
       <c r="B78" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="C78" t="s">
         <v>103</v>
@@ -3723,10 +3671,10 @@
     </row>
     <row r="79" spans="1:4">
       <c r="A79" t="s">
-        <v>690</v>
+        <v>68</v>
       </c>
       <c r="B79" t="s">
-        <v>691</v>
+        <v>709</v>
       </c>
       <c r="C79" t="s">
         <v>103</v>
@@ -3737,10 +3685,10 @@
     </row>
     <row r="80" spans="1:4">
       <c r="A80" t="s">
-        <v>62</v>
+        <v>685</v>
       </c>
       <c r="B80" t="s">
-        <v>174</v>
+        <v>709</v>
       </c>
       <c r="C80" t="s">
         <v>103</v>
@@ -3751,10 +3699,10 @@
     </row>
     <row r="81" spans="1:4">
       <c r="A81" t="s">
-        <v>63</v>
+        <v>686</v>
       </c>
       <c r="B81" t="s">
-        <v>175</v>
+        <v>709</v>
       </c>
       <c r="C81" t="s">
         <v>103</v>
@@ -3765,10 +3713,10 @@
     </row>
     <row r="82" spans="1:4">
       <c r="A82" t="s">
-        <v>64</v>
+        <v>687</v>
       </c>
       <c r="B82" t="s">
-        <v>176</v>
+        <v>709</v>
       </c>
       <c r="C82" t="s">
         <v>103</v>
@@ -3779,10 +3727,10 @@
     </row>
     <row r="83" spans="1:4">
       <c r="A83" t="s">
-        <v>65</v>
+        <v>688</v>
       </c>
       <c r="B83" t="s">
-        <v>177</v>
+        <v>709</v>
       </c>
       <c r="C83" t="s">
         <v>103</v>
@@ -3793,197 +3741,57 @@
     </row>
     <row r="84" spans="1:4">
       <c r="A84" t="s">
-        <v>67</v>
+        <v>84</v>
       </c>
       <c r="B84" t="s">
-        <v>692</v>
+        <v>178</v>
       </c>
       <c r="C84" t="s">
-        <v>103</v>
+        <v>179</v>
       </c>
       <c r="D84">
-        <v>0</v>
+        <v>-90</v>
       </c>
     </row>
     <row r="85" spans="1:4">
       <c r="A85" t="s">
-        <v>681</v>
+        <v>85</v>
       </c>
       <c r="B85" t="s">
-        <v>692</v>
+        <v>180</v>
       </c>
       <c r="C85" t="s">
         <v>103</v>
       </c>
       <c r="D85">
-        <v>0</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="86" spans="1:4">
       <c r="A86" t="s">
-        <v>682</v>
+        <v>86</v>
       </c>
       <c r="B86" t="s">
-        <v>692</v>
+        <v>181</v>
       </c>
       <c r="C86" t="s">
-        <v>103</v>
+        <v>182</v>
       </c>
       <c r="D86">
-        <v>0</v>
+        <v>24</v>
       </c>
     </row>
     <row r="87" spans="1:4">
       <c r="A87" t="s">
-        <v>683</v>
+        <v>87</v>
       </c>
       <c r="B87" t="s">
-        <v>692</v>
+        <v>183</v>
       </c>
       <c r="C87" t="s">
-        <v>103</v>
+        <v>184</v>
       </c>
       <c r="D87">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="88" spans="1:4">
-      <c r="A88" t="s">
-        <v>684</v>
-      </c>
-      <c r="B88" t="s">
-        <v>692</v>
-      </c>
-      <c r="C88" t="s">
-        <v>103</v>
-      </c>
-      <c r="D88">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="89" spans="1:4">
-      <c r="A89" t="s">
-        <v>68</v>
-      </c>
-      <c r="B89" t="s">
-        <v>730</v>
-      </c>
-      <c r="C89" t="s">
-        <v>103</v>
-      </c>
-      <c r="D89">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="90" spans="1:4">
-      <c r="A90" t="s">
-        <v>685</v>
-      </c>
-      <c r="B90" t="s">
-        <v>730</v>
-      </c>
-      <c r="C90" t="s">
-        <v>103</v>
-      </c>
-      <c r="D90">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="91" spans="1:4">
-      <c r="A91" t="s">
-        <v>686</v>
-      </c>
-      <c r="B91" t="s">
-        <v>730</v>
-      </c>
-      <c r="C91" t="s">
-        <v>103</v>
-      </c>
-      <c r="D91">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="92" spans="1:4">
-      <c r="A92" t="s">
-        <v>687</v>
-      </c>
-      <c r="B92" t="s">
-        <v>730</v>
-      </c>
-      <c r="C92" t="s">
-        <v>103</v>
-      </c>
-      <c r="D92">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="93" spans="1:4">
-      <c r="A93" t="s">
-        <v>688</v>
-      </c>
-      <c r="B93" t="s">
-        <v>730</v>
-      </c>
-      <c r="C93" t="s">
-        <v>103</v>
-      </c>
-      <c r="D93">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="94" spans="1:4">
-      <c r="A94" t="s">
-        <v>84</v>
-      </c>
-      <c r="B94" t="s">
-        <v>178</v>
-      </c>
-      <c r="C94" t="s">
-        <v>179</v>
-      </c>
-      <c r="D94">
-        <v>-90</v>
-      </c>
-    </row>
-    <row r="95" spans="1:4">
-      <c r="A95" t="s">
-        <v>85</v>
-      </c>
-      <c r="B95" t="s">
-        <v>180</v>
-      </c>
-      <c r="C95" t="s">
-        <v>103</v>
-      </c>
-      <c r="D95">
-        <v>0.8</v>
-      </c>
-    </row>
-    <row r="96" spans="1:4">
-      <c r="A96" t="s">
-        <v>86</v>
-      </c>
-      <c r="B96" t="s">
-        <v>181</v>
-      </c>
-      <c r="C96" t="s">
-        <v>182</v>
-      </c>
-      <c r="D96">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="97" spans="1:4">
-      <c r="A97" t="s">
-        <v>87</v>
-      </c>
-      <c r="B97" t="s">
-        <v>183</v>
-      </c>
-      <c r="C97" t="s">
-        <v>184</v>
-      </c>
-      <c r="D97">
         <v>2.2999999999999998</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add height_rel_wt to outputs for testing
</commit_message>
<xml_diff>
--- a/data-raw/data.default.xlsx
+++ b/data-raw/data.default.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Forrester\Models\3-PG\r3PG_mortality_management_defoliation2\data-raw\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Forrester\Models\3-PG\r3PG_mortality_management_defoliation\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{442BC11E-450B-47D6-AEDC-2C8AF52FE263}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{361E04DA-59D5-426C-994C-093B10A6608E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{61EEFE5B-6AE1-A641-A9AB-273DC4213F59}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1224" uniqueCount="709">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1222" uniqueCount="708">
   <si>
     <t>pFS2</t>
   </si>
@@ -2051,9 +2051,6 @@
     <t>def_type</t>
   </si>
   <si>
-    <t>def_recover_t</t>
-  </si>
-  <si>
     <t>Number of trees removed due to defoliation</t>
   </si>
   <si>
@@ -2066,9 +2063,6 @@
     <t>Defoliation type (1 = Pruning; 2 = Epicormic; 3 = Coppice; 4 = Stand-replacing)</t>
   </si>
   <si>
-    <t>Maximum number of months required to recover the pre-defoliation foliage biomass (pruning or epicormic responses) or foliage + stem mass (coppice responses) of the trees that survived the defoliation event.</t>
-  </si>
-  <si>
     <t>Foliage biomass removed due to defoliation</t>
   </si>
   <si>
@@ -2169,6 +2163,9 @@
   </si>
   <si>
     <t>var_4_13</t>
+  </si>
+  <si>
+    <t>height_rel_wt</t>
   </si>
 </sst>
 </file>
@@ -2220,7 +2217,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2230,6 +2227,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2247,7 +2250,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -2255,6 +2258,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2819,7 +2823,7 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>678</v>
+        <v>676</v>
       </c>
       <c r="C18" t="s">
         <v>103</v>
@@ -3015,7 +3019,7 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>704</v>
+        <v>702</v>
       </c>
       <c r="C32" t="s">
         <v>138</v>
@@ -3029,7 +3033,7 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>705</v>
+        <v>703</v>
       </c>
       <c r="C33" t="s">
         <v>103</v>
@@ -3475,7 +3479,7 @@
         <v>61</v>
       </c>
       <c r="B65" t="s">
-        <v>691</v>
+        <v>689</v>
       </c>
       <c r="C65" t="s">
         <v>103</v>
@@ -3486,10 +3490,10 @@
     </row>
     <row r="66" spans="1:4">
       <c r="A66" t="s">
-        <v>679</v>
+        <v>677</v>
       </c>
       <c r="B66" t="s">
-        <v>691</v>
+        <v>689</v>
       </c>
       <c r="C66" t="s">
         <v>103</v>
@@ -3500,10 +3504,10 @@
     </row>
     <row r="67" spans="1:4">
       <c r="A67" t="s">
-        <v>680</v>
+        <v>678</v>
       </c>
       <c r="B67" t="s">
-        <v>691</v>
+        <v>689</v>
       </c>
       <c r="C67" t="s">
         <v>103</v>
@@ -3514,10 +3518,10 @@
     </row>
     <row r="68" spans="1:4">
       <c r="A68" t="s">
+        <v>687</v>
+      </c>
+      <c r="B68" t="s">
         <v>689</v>
-      </c>
-      <c r="B68" t="s">
-        <v>691</v>
       </c>
       <c r="C68" t="s">
         <v>103</v>
@@ -3528,10 +3532,10 @@
     </row>
     <row r="69" spans="1:4">
       <c r="A69" t="s">
-        <v>690</v>
+        <v>688</v>
       </c>
       <c r="B69" t="s">
-        <v>691</v>
+        <v>689</v>
       </c>
       <c r="C69" t="s">
         <v>103</v>
@@ -3601,7 +3605,7 @@
         <v>67</v>
       </c>
       <c r="B74" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="C74" t="s">
         <v>103</v>
@@ -3612,10 +3616,10 @@
     </row>
     <row r="75" spans="1:4">
       <c r="A75" t="s">
-        <v>681</v>
+        <v>679</v>
       </c>
       <c r="B75" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="C75" t="s">
         <v>103</v>
@@ -3626,10 +3630,10 @@
     </row>
     <row r="76" spans="1:4">
       <c r="A76" t="s">
-        <v>682</v>
+        <v>680</v>
       </c>
       <c r="B76" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="C76" t="s">
         <v>103</v>
@@ -3640,10 +3644,10 @@
     </row>
     <row r="77" spans="1:4">
       <c r="A77" t="s">
-        <v>683</v>
+        <v>681</v>
       </c>
       <c r="B77" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="C77" t="s">
         <v>103</v>
@@ -3654,10 +3658,10 @@
     </row>
     <row r="78" spans="1:4">
       <c r="A78" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="B78" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="C78" t="s">
         <v>103</v>
@@ -3671,7 +3675,7 @@
         <v>68</v>
       </c>
       <c r="B79" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="C79" t="s">
         <v>103</v>
@@ -3682,10 +3686,10 @@
     </row>
     <row r="80" spans="1:4">
       <c r="A80" t="s">
-        <v>685</v>
+        <v>683</v>
       </c>
       <c r="B80" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="C80" t="s">
         <v>103</v>
@@ -3696,10 +3700,10 @@
     </row>
     <row r="81" spans="1:4">
       <c r="A81" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
       <c r="B81" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="C81" t="s">
         <v>103</v>
@@ -3710,10 +3714,10 @@
     </row>
     <row r="82" spans="1:4">
       <c r="A82" t="s">
-        <v>687</v>
+        <v>685</v>
       </c>
       <c r="B82" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="C82" t="s">
         <v>103</v>
@@ -3724,10 +3728,10 @@
     </row>
     <row r="83" spans="1:4">
       <c r="A83" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
       <c r="B83" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="C83" t="s">
         <v>103</v>
@@ -5486,7 +5490,7 @@
         <v>12</v>
       </c>
       <c r="C73" t="s">
-        <v>707</v>
+        <v>705</v>
       </c>
       <c r="D73" t="s">
         <v>332</v>
@@ -5500,7 +5504,7 @@
         <v>13</v>
       </c>
       <c r="C74" t="s">
-        <v>708</v>
+        <v>706</v>
       </c>
       <c r="D74" t="s">
         <v>332</v>
@@ -6970,7 +6974,7 @@
         <v>11</v>
       </c>
       <c r="C152" s="1" t="s">
-        <v>676</v>
+        <v>674</v>
       </c>
       <c r="D152" t="s">
         <v>495</v>
@@ -6984,7 +6988,7 @@
         <v>12</v>
       </c>
       <c r="C153" s="1" t="s">
-        <v>677</v>
+        <v>675</v>
       </c>
       <c r="D153" t="s">
         <v>495</v>
@@ -7498,7 +7502,7 @@
         <v>4</v>
       </c>
       <c r="C185" s="1" t="s">
-        <v>693</v>
+        <v>691</v>
       </c>
       <c r="D185" t="s">
         <v>530</v>
@@ -7521,7 +7525,7 @@
         <v>5</v>
       </c>
       <c r="C186" s="1" t="s">
-        <v>694</v>
+        <v>692</v>
       </c>
       <c r="D186" t="s">
         <v>530</v>
@@ -7544,7 +7548,7 @@
         <v>6</v>
       </c>
       <c r="C187" s="1" t="s">
-        <v>695</v>
+        <v>693</v>
       </c>
       <c r="D187" t="s">
         <v>530</v>
@@ -7567,7 +7571,7 @@
         <v>7</v>
       </c>
       <c r="C188" s="1" t="s">
-        <v>696</v>
+        <v>694</v>
       </c>
       <c r="D188" t="s">
         <v>530</v>
@@ -7590,7 +7594,7 @@
         <v>8</v>
       </c>
       <c r="C189" s="1" t="s">
-        <v>697</v>
+        <v>695</v>
       </c>
       <c r="D189" t="s">
         <v>530</v>
@@ -7613,7 +7617,7 @@
         <v>9</v>
       </c>
       <c r="C190" s="1" t="s">
-        <v>698</v>
+        <v>696</v>
       </c>
       <c r="D190" t="s">
         <v>530</v>
@@ -7636,7 +7640,7 @@
         <v>10</v>
       </c>
       <c r="C191" s="1" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="D191" t="s">
         <v>530</v>
@@ -7659,7 +7663,7 @@
         <v>11</v>
       </c>
       <c r="C192" s="1" t="s">
-        <v>700</v>
+        <v>698</v>
       </c>
       <c r="D192" t="s">
         <v>530</v>
@@ -7682,7 +7686,7 @@
         <v>12</v>
       </c>
       <c r="C193" s="1" t="s">
-        <v>701</v>
+        <v>699</v>
       </c>
       <c r="D193" t="s">
         <v>530</v>
@@ -7705,7 +7709,7 @@
         <v>13</v>
       </c>
       <c r="C194" s="1" t="s">
-        <v>702</v>
+        <v>700</v>
       </c>
       <c r="D194" t="s">
         <v>530</v>
@@ -7728,7 +7732,7 @@
         <v>14</v>
       </c>
       <c r="C195" s="1" t="s">
-        <v>703</v>
+        <v>701</v>
       </c>
       <c r="D195" t="s">
         <v>530</v>
@@ -8081,7 +8085,7 @@
         <v>573</v>
       </c>
       <c r="E214" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="F214" t="s">
         <v>249</v>
@@ -8101,7 +8105,7 @@
         <v>573</v>
       </c>
       <c r="E215" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="F215" t="s">
         <v>334</v>
@@ -8121,7 +8125,7 @@
         <v>573</v>
       </c>
       <c r="E216" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="F216" t="s">
         <v>334</v>
@@ -8141,7 +8145,7 @@
         <v>573</v>
       </c>
       <c r="E217" t="s">
-        <v>675</v>
+        <v>673</v>
       </c>
       <c r="F217" t="s">
         <v>334</v>
@@ -8161,7 +8165,7 @@
         <v>573</v>
       </c>
       <c r="E218" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
     </row>
     <row r="219" spans="1:6">
@@ -8171,18 +8175,13 @@
       <c r="B219" s="4">
         <v>18</v>
       </c>
-      <c r="C219" s="6" t="s">
-        <v>669</v>
+      <c r="C219" s="7" t="s">
+        <v>707</v>
       </c>
       <c r="D219" s="4" t="s">
         <v>573</v>
       </c>
-      <c r="E219" t="s">
-        <v>674</v>
-      </c>
-      <c r="F219" s="4" t="s">
-        <v>113</v>
-      </c>
+      <c r="F219" s="4"/>
     </row>
     <row r="220" spans="1:6">
       <c r="A220" s="4">

</xml_diff>